<commit_message>
project 관련 파일 업로드_20260820_2
</commit_message>
<xml_diff>
--- a/Project_1/Project Status.xlsx
+++ b/Project_1/Project Status.xlsx
@@ -5,41 +5,35 @@
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\pyostry\Desktop\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\pyostry\workspace\aiffel\ai-data-bootcamp\Project_1\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5E4B0169-8DDB-49ED-84C5-E0A6A8DC3783}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1C4A70F7-0946-42CC-9AAA-0C772D520FE5}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-90" yWindow="-90" windowWidth="25780" windowHeight="15460" activeTab="2" xr2:uid="{6B636699-A6E6-472F-A92F-8A8168DF527A}"/>
+    <workbookView xWindow="30612" yWindow="-108" windowWidth="30936" windowHeight="16776" activeTab="3" xr2:uid="{6B636699-A6E6-472F-A92F-8A8168DF527A}"/>
   </bookViews>
   <sheets>
     <sheet name="0. Status" sheetId="3" r:id="rId1"/>
     <sheet name="1. Dataset type" sheetId="2" r:id="rId2"/>
     <sheet name="2. 문제 정의와 분석 설계" sheetId="5" r:id="rId3"/>
-    <sheet name="발표자료 목차" sheetId="1" r:id="rId4"/>
-    <sheet name="평가 사항" sheetId="4" r:id="rId5"/>
+    <sheet name="3. 분석 계획서" sheetId="7" r:id="rId4"/>
+    <sheet name="발표자료 목차" sheetId="1" r:id="rId5"/>
+    <sheet name="평가 사항" sheetId="4" r:id="rId6"/>
   </sheets>
+  <definedNames>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'2. 문제 정의와 분석 설계'!$A$1:$C$1</definedName>
+  </definedNames>
   <calcPr calcId="191029"/>
   <extLst>
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
       <x15:workbookPr chartTrackingRefBase="1"/>
-    </ext>
-    <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
-      <xcalcf:calcFeatures>
-        <xcalcf:feature name="microsoft.com:RD"/>
-        <xcalcf:feature name="microsoft.com:Single"/>
-        <xcalcf:feature name="microsoft.com:FV"/>
-        <xcalcf:feature name="microsoft.com:CNMTM"/>
-        <xcalcf:feature name="microsoft.com:LET_WF"/>
-        <xcalcf:feature name="microsoft.com:ARRAYTEXT_WF"/>
-      </xcalcf:calcFeatures>
     </ext>
   </extLst>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="114" uniqueCount="82">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="137" uniqueCount="102">
   <si>
     <t>Dataset</t>
     <phoneticPr fontId="1" type="noConversion"/>
@@ -853,7 +847,7 @@
       </rPr>
       <t xml:space="preserve">1. 업종별 (추정매출÷점포수), 즉 '점포 1곳당 평균 매출'이 높은데도 점포 수 자체는 적은 업종일수록, 신규 진입 시 성공 가능성이 높을 것이다.
 2. 지하철역·버스정류소 밀도(유동인구 대체지표)는 높지만, 특정 업종의 추정매출은 서울시 평균보다 낮은 행정동이 존재하며, 이런 곳은 '아직 개발 안 된 틈새 상권'일 것이다.
-3. 1인가구·젊은 연령대 밀집 지역엔 배달형이 유리하다
+3. 10~30대 밀집 지역엔 배달형이 유리하다
 </t>
     </r>
     <r>
@@ -868,6 +862,319 @@
       </rPr>
       <t>데이터셋과 분석 방법의 선택 근거</t>
     </r>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>2026-08-20~21</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>팀명</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>서현 없는 서현팀</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>너무 무난한 주제</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>https://docs.google.com/document/d/1OyaboMkOYqWNSGp_u1YU_gjkvz1d8PbxVPWkj3sAovo/edit?usp=sharing
+키워드 위주로 주제 정해졌으며 세부 내용은 추가 논의 필요</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>https://docs.google.com/document/d/1Hr7D1ghJJJS2J0RdheFv9XuYWkOJ3qB2UXs0U-28q6g/edit?usp=sharing
+시계열 분석으로 한계점 있음.</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>의사결정자와 비즈니스 상황</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>각 질문에 대한 가설</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>데이터셋과 분석 방법의 선택 근거를 정리</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>항목</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>분석 계획서</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>ERD</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>https://claude.ai/code/artifact/c5fa9def-8885-4da1-8dce-49f5c6ec8ea8</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>핵심 질문 1개</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>보조 질문 2개</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="맑은 고딕"/>
+        <family val="3"/>
+        <charset val="129"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>데이터 출처</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="맑은 고딕"/>
+        <family val="2"/>
+        <charset val="129"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">: 서울 열린데이터광장(https://data.seoul.go.kr)
+서울시 상권분석서비스(https://golmok.seoul.go.kr/main.do)
+공공데이터포털(https://www.data.go.kr)
+서울시 상권분석서비스(추정매출-자치구)
+</t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="맑은 고딕"/>
+        <family val="3"/>
+        <charset val="129"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>분석 방법:
+분석 대상:</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="맑은 고딕"/>
+        <family val="2"/>
+        <charset val="129"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> 서울시 25개 자치구 × 서비스업종 × 분기 패널 데이터
+</t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="맑은 고딕"/>
+        <family val="3"/>
+        <charset val="129"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>주 평가변수(핵심질문):</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="맑은 고딕"/>
+        <family val="2"/>
+        <charset val="129"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> 다음 분기 순감소 전환 여부(이진변수) — 패널 로지스틱 회귀(분기 고정효과 포함)로 분석
+</t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="맑은 고딕"/>
+        <family val="3"/>
+        <charset val="129"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">주 평가변수(핵심질문): </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="맑은 고딕"/>
+        <family val="2"/>
+        <charset val="129"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>카이제곱·Kruskal-Wallis 검정 - 상권 유형·업종별 폐업위험 차이가 실제로 존재하는지 확인하고 Cramér’s V·</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <charset val="161"/>
+      </rPr>
+      <t>ε</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="맑은 고딕"/>
+        <family val="2"/>
+        <charset val="129"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">²로 효과크기를 측정.
+</t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="맑은 고딕"/>
+        <family val="3"/>
+        <charset val="129"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>PSM(성향점수매칭):</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="맑은 고딕"/>
+        <family val="2"/>
+        <charset val="129"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> 매출·유동인구·규모 등이 비슷한 상권끼리 매칭해 특정 조건에 따른 폐업위험 차이를 비교.
+</t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="맑은 고딕"/>
+        <family val="3"/>
+        <charset val="129"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>로지스틱 회귀·랜덤포레스트·XGBoost</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="맑은 고딕"/>
+        <family val="2"/>
+        <charset val="129"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> -  현재 상권 정보로 다음 분기 폐업위험을 예측하고 모델 성능을 비교.
+</t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="맑은 고딕"/>
+        <family val="3"/>
+        <charset val="129"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>SHAP</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="맑은 고딕"/>
+        <family val="2"/>
+        <charset val="129"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> - 최종 예측모델에서 매출·임대료·유동인구 등 어떤 변수가 폐업위험 판단에 크게 기여했는지 확인.
+</t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="맑은 고딕"/>
+        <family val="3"/>
+        <charset val="129"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">선택 근거:
+</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="맑은 고딕"/>
+        <family val="3"/>
+        <charset val="129"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>23년 코로나 이후 상권 활성화 상태의 자료</t>
+    </r>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <r>
+      <t xml:space="preserve">1. 동일 업종이라도 자치구별 상권 유형에 따라 폐업위험이 다르다.
+</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FFFF0000"/>
+        <rFont val="맑은 고딕"/>
+        <family val="3"/>
+        <charset val="129"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>2. 신생 점포(개업 초기)는 기존 점포 대비 폐업위험이 높다.</t>
+    </r>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>서울시 상권 공공 데이터 기반 요식업 점포 폐업 위험 예측 조기 경보</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>자치구별 다음 분기 점포 순감소로 전환될 요식업 업종은 무엇일까?</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>1. 점포 순감소 전환 가능성은 자치구와 업종에 따라 어떻게 다른가?
+2. 매출, 유동인구, 점포 밀도 등 어떤 특성이 다음 분기 순감소 전환과 관련되는가?</t>
     <phoneticPr fontId="1" type="noConversion"/>
   </si>
 </sst>
@@ -875,7 +1182,7 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="9" x14ac:knownFonts="1">
+  <fonts count="12" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -949,6 +1256,29 @@
       <charset val="129"/>
       <scheme val="minor"/>
     </font>
+    <font>
+      <sz val="11"/>
+      <color rgb="FFFF0000"/>
+      <name val="맑은 고딕"/>
+      <family val="3"/>
+      <charset val="129"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="맑은 고딕"/>
+      <family val="3"/>
+      <charset val="129"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <charset val="161"/>
+    </font>
   </fonts>
   <fills count="5">
     <fill>
@@ -976,7 +1306,7 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="2">
+  <borders count="4">
     <border>
       <left/>
       <right/>
@@ -999,6 +1329,32 @@
       </bottom>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin">
+        <color indexed="64"/>
+      </left>
+      <right/>
+      <top style="thin">
+        <color indexed="64"/>
+      </top>
+      <bottom style="thin">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="thin">
+        <color indexed="64"/>
+      </right>
+      <top style="thin">
+        <color indexed="64"/>
+      </top>
+      <bottom style="thin">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0">
@@ -1008,7 +1364,7 @@
       <alignment vertical="center"/>
     </xf>
   </cellStyleXfs>
-  <cellXfs count="35">
+  <cellXfs count="40">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0">
       <alignment vertical="center"/>
     </xf>
@@ -1027,7 +1383,7 @@
     <xf numFmtId="22" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
@@ -1048,9 +1404,6 @@
     <xf numFmtId="0" fontId="3" fillId="0" borderId="1" xfId="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1" readingOrder="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="2" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1" readingOrder="1"/>
     </xf>
@@ -1090,28 +1443,46 @@
     <xf numFmtId="0" fontId="7" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
     <xf numFmtId="22" fontId="7" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="8" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="1" xfId="1" quotePrefix="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="7" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="14" fontId="6" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="22" fontId="6" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="1" xfId="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
@@ -1429,7 +1800,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{2E6BAA0C-FF2D-4443-80AC-2A45A5480151}">
-  <dimension ref="A1:D10"/>
+  <dimension ref="A1:D11"/>
   <sheetFormatPr defaultRowHeight="17" x14ac:dyDescent="0.45"/>
   <cols>
     <col min="1" max="1" width="25.9140625" customWidth="1"/>
@@ -1453,102 +1824,128 @@
       </c>
     </row>
     <row r="2" spans="1:4" x14ac:dyDescent="0.45">
-      <c r="A2" s="22" t="s">
+      <c r="A2" s="21" t="s">
         <v>0</v>
       </c>
-      <c r="B2" s="33" t="s">
+      <c r="B2" s="28" t="s">
         <v>77</v>
       </c>
-      <c r="C2" s="25">
+      <c r="C2" s="24">
         <v>46254</v>
       </c>
-      <c r="D2" s="24" t="s">
+      <c r="D2" s="23" t="s">
         <v>15</v>
       </c>
     </row>
-    <row r="3" spans="1:4" ht="64" x14ac:dyDescent="0.45">
-      <c r="A3" s="22" t="s">
+    <row r="3" spans="1:4" x14ac:dyDescent="0.45">
+      <c r="A3" s="21" t="s">
+        <v>83</v>
+      </c>
+      <c r="B3" s="28"/>
+      <c r="C3" s="24">
+        <v>46254</v>
+      </c>
+      <c r="D3" s="23" t="s">
+        <v>84</v>
+      </c>
+    </row>
+    <row r="4" spans="1:4" ht="64" x14ac:dyDescent="0.45">
+      <c r="A4" s="21" t="s">
         <v>49</v>
       </c>
-      <c r="B3" s="20" t="s">
+      <c r="B4" s="19" t="s">
         <v>54</v>
       </c>
-      <c r="C3" s="25">
+      <c r="C4" s="24">
         <v>46254</v>
       </c>
-      <c r="D3" s="24"/>
-    </row>
-    <row r="4" spans="1:4" ht="112" x14ac:dyDescent="0.45">
-      <c r="A4" s="23" t="s">
+      <c r="D4" s="23"/>
+    </row>
+    <row r="5" spans="1:4" ht="112" x14ac:dyDescent="0.45">
+      <c r="A5" s="22" t="s">
         <v>50</v>
       </c>
-      <c r="B4" s="21" t="s">
+      <c r="B5" s="20" t="s">
         <v>60</v>
       </c>
-      <c r="C4" s="27"/>
-      <c r="D4" s="24"/>
-    </row>
-    <row r="5" spans="1:4" ht="48" x14ac:dyDescent="0.45">
-      <c r="A5" s="23" t="s">
+      <c r="C5" s="24" t="s">
+        <v>82</v>
+      </c>
+      <c r="D5" s="23"/>
+    </row>
+    <row r="6" spans="1:4" ht="48" x14ac:dyDescent="0.45">
+      <c r="A6" s="22" t="s">
         <v>51</v>
       </c>
-      <c r="B5" s="21" t="s">
+      <c r="B6" s="20" t="s">
         <v>55</v>
       </c>
-      <c r="C5" s="27"/>
-      <c r="D5" s="24"/>
-    </row>
-    <row r="6" spans="1:4" ht="64" x14ac:dyDescent="0.45">
-      <c r="A6" s="23" t="s">
+      <c r="C6" s="30">
+        <v>46255</v>
+      </c>
+      <c r="D6" s="23"/>
+    </row>
+    <row r="7" spans="1:4" ht="64" x14ac:dyDescent="0.45">
+      <c r="A7" s="22" t="s">
         <v>52</v>
       </c>
-      <c r="B6" s="21" t="s">
+      <c r="B7" s="20" t="s">
         <v>56</v>
       </c>
-      <c r="C6" s="27"/>
-      <c r="D6" s="24"/>
-    </row>
-    <row r="7" spans="1:4" ht="80" x14ac:dyDescent="0.45">
-      <c r="A7" s="23" t="s">
+      <c r="C7" s="30">
+        <v>46258</v>
+      </c>
+      <c r="D7" s="23"/>
+    </row>
+    <row r="8" spans="1:4" ht="80" x14ac:dyDescent="0.45">
+      <c r="A8" s="22" t="s">
         <v>53</v>
       </c>
-      <c r="B7" s="21" t="s">
+      <c r="B8" s="20" t="s">
         <v>57</v>
       </c>
-      <c r="C7" s="27"/>
-      <c r="D7" s="24"/>
-    </row>
-    <row r="8" spans="1:4" ht="80" x14ac:dyDescent="0.45">
-      <c r="A8" s="23" t="s">
+      <c r="C8" s="30">
+        <v>46258</v>
+      </c>
+      <c r="D8" s="23"/>
+    </row>
+    <row r="9" spans="1:4" ht="80" x14ac:dyDescent="0.45">
+      <c r="A9" s="22" t="s">
         <v>59</v>
       </c>
-      <c r="B8" s="21" t="s">
+      <c r="B9" s="20" t="s">
         <v>58</v>
       </c>
-      <c r="C8" s="27"/>
-      <c r="D8" s="24"/>
-    </row>
-    <row r="9" spans="1:4" x14ac:dyDescent="0.45">
-      <c r="A9" s="28" t="s">
+      <c r="C9" s="30">
+        <v>46259</v>
+      </c>
+      <c r="D9" s="23"/>
+    </row>
+    <row r="10" spans="1:4" x14ac:dyDescent="0.45">
+      <c r="A10" s="33" t="s">
         <v>8</v>
       </c>
-      <c r="B9" s="28"/>
-      <c r="C9" s="29">
+      <c r="B10" s="34"/>
+      <c r="C10" s="31">
+        <v>46259.5</v>
+      </c>
+      <c r="D10" s="26"/>
+    </row>
+    <row r="11" spans="1:4" x14ac:dyDescent="0.45">
+      <c r="A11" s="33" t="s">
+        <v>9</v>
+      </c>
+      <c r="B11" s="34"/>
+      <c r="C11" s="31">
         <v>46259.645833333336</v>
       </c>
-      <c r="D9" s="29"/>
-    </row>
-    <row r="10" spans="1:4" x14ac:dyDescent="0.45">
-      <c r="A10" s="28" t="s">
-        <v>9</v>
-      </c>
-      <c r="B10" s="28"/>
-      <c r="C10" s="29">
-        <v>46259.5</v>
-      </c>
-      <c r="D10" s="29"/>
+      <c r="D11" s="26"/>
     </row>
   </sheetData>
+  <mergeCells count="2">
+    <mergeCell ref="A10:B10"/>
+    <mergeCell ref="A11:B11"/>
+  </mergeCells>
   <phoneticPr fontId="1" type="noConversion"/>
   <hyperlinks>
     <hyperlink ref="B2" location="'1. Dataset type'!A1" display="'1. Dataset type'!A1" xr:uid="{E265BD97-7DB2-4CB1-967B-BCF2D8B10C8D}"/>
@@ -1570,31 +1967,31 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:9" x14ac:dyDescent="0.45">
-      <c r="A1" s="14" t="s">
+      <c r="A1" s="13" t="s">
         <v>19</v>
       </c>
-      <c r="B1" s="14" t="s">
+      <c r="B1" s="13" t="s">
         <v>20</v>
       </c>
-      <c r="C1" s="14" t="s">
+      <c r="C1" s="13" t="s">
         <v>21</v>
       </c>
-      <c r="D1" s="14" t="s">
+      <c r="D1" s="13" t="s">
         <v>12</v>
       </c>
-      <c r="E1" s="15" t="s">
+      <c r="E1" s="14" t="s">
         <v>18</v>
       </c>
-      <c r="F1" s="15" t="s">
+      <c r="F1" s="14" t="s">
         <v>44</v>
       </c>
-      <c r="G1" s="15" t="s">
+      <c r="G1" s="14" t="s">
         <v>45</v>
       </c>
-      <c r="H1" s="15" t="s">
+      <c r="H1" s="14" t="s">
         <v>46</v>
       </c>
-      <c r="I1" s="15" t="s">
+      <c r="I1" s="14" t="s">
         <v>47</v>
       </c>
     </row>
@@ -1613,8 +2010,8 @@
       </c>
       <c r="E2" s="4"/>
       <c r="F2" s="4"/>
-      <c r="G2" s="16"/>
-      <c r="H2" s="16" t="s">
+      <c r="G2" s="15"/>
+      <c r="H2" s="15" t="s">
         <v>43</v>
       </c>
       <c r="I2" s="4"/>
@@ -1634,8 +2031,8 @@
       </c>
       <c r="E3" s="4"/>
       <c r="F3" s="4"/>
-      <c r="G3" s="16"/>
-      <c r="H3" s="16" t="s">
+      <c r="G3" s="15"/>
+      <c r="H3" s="15" t="s">
         <v>43</v>
       </c>
       <c r="I3" s="4"/>
@@ -1655,7 +2052,7 @@
       </c>
       <c r="E4" s="4"/>
       <c r="F4" s="4"/>
-      <c r="G4" s="16" t="s">
+      <c r="G4" s="15" t="s">
         <v>43</v>
       </c>
       <c r="H4" s="4"/>
@@ -1694,7 +2091,7 @@
         <v>39</v>
       </c>
       <c r="E6" s="4"/>
-      <c r="F6" s="16" t="s">
+      <c r="F6" s="15" t="s">
         <v>43</v>
       </c>
       <c r="G6" s="4"/>
@@ -1733,39 +2130,39 @@
       <c r="D8" s="10" t="s">
         <v>41</v>
       </c>
-      <c r="E8" s="16" t="s">
+      <c r="E8" s="15" t="s">
         <v>43</v>
       </c>
       <c r="F8" s="4"/>
-      <c r="G8" s="16" t="s">
+      <c r="G8" s="15" t="s">
         <v>43</v>
       </c>
       <c r="H8" s="4"/>
       <c r="I8" s="4"/>
     </row>
     <row r="9" spans="1:9" ht="51" x14ac:dyDescent="0.45">
-      <c r="A9" s="17">
+      <c r="A9" s="16">
         <v>8</v>
       </c>
-      <c r="B9" s="18" t="s">
+      <c r="B9" s="17" t="s">
         <v>15</v>
       </c>
-      <c r="C9" s="19" t="s">
+      <c r="C9" s="18" t="s">
         <v>28</v>
       </c>
-      <c r="D9" s="19" t="s">
+      <c r="D9" s="18" t="s">
         <v>42</v>
       </c>
-      <c r="E9" s="16" t="s">
+      <c r="E9" s="15" t="s">
         <v>43</v>
       </c>
-      <c r="F9" s="16" t="s">
+      <c r="F9" s="15" t="s">
         <v>43</v>
       </c>
-      <c r="G9" s="16" t="s">
+      <c r="G9" s="15" t="s">
         <v>43</v>
       </c>
-      <c r="H9" s="16" t="s">
+      <c r="H9" s="15" t="s">
         <v>43</v>
       </c>
       <c r="I9" s="4"/>
@@ -1783,7 +2180,7 @@
       <c r="D10" s="10" t="s">
         <v>32</v>
       </c>
-      <c r="E10" s="16"/>
+      <c r="E10" s="15"/>
       <c r="F10" s="4"/>
       <c r="G10" s="4"/>
       <c r="H10" s="4"/>
@@ -1802,10 +2199,10 @@
       <c r="D11" s="10" t="s">
         <v>34</v>
       </c>
-      <c r="E11" s="16" t="s">
+      <c r="E11" s="15" t="s">
         <v>43</v>
       </c>
-      <c r="F11" s="16" t="s">
+      <c r="F11" s="15" t="s">
         <v>43</v>
       </c>
       <c r="G11" s="4"/>
@@ -1832,75 +2229,188 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{9E9C4A99-AAB3-49B2-8D3F-2CED6FB92258}">
-  <dimension ref="A1:B8"/>
+  <dimension ref="A1:C7"/>
   <sheetFormatPr defaultRowHeight="17" x14ac:dyDescent="0.45"/>
   <cols>
-    <col min="1" max="1" width="25.9140625" customWidth="1"/>
-    <col min="2" max="2" width="124.33203125" customWidth="1"/>
+    <col min="1" max="1" width="39.83203125" customWidth="1"/>
+    <col min="2" max="2" width="140.75" customWidth="1"/>
+    <col min="3" max="3" width="33.83203125" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:2" x14ac:dyDescent="0.45">
+    <row r="1" spans="1:3" x14ac:dyDescent="0.45">
       <c r="A1" s="8" t="s">
         <v>11</v>
       </c>
       <c r="B1" s="9" t="s">
         <v>76</v>
       </c>
-    </row>
-    <row r="2" spans="1:2" ht="64" x14ac:dyDescent="0.45">
-      <c r="A2" s="22" t="s">
+      <c r="C1" s="9" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="2" spans="1:3" ht="64" x14ac:dyDescent="0.45">
+      <c r="A2" s="32" t="s">
         <v>49</v>
       </c>
-      <c r="B2" s="20" t="s">
+      <c r="B2" s="19" t="s">
         <v>54</v>
       </c>
-    </row>
-    <row r="3" spans="1:2" ht="12" customHeight="1" x14ac:dyDescent="0.45"/>
-    <row r="4" spans="1:2" ht="101.5" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="A4" s="15" t="s">
+      <c r="C2" s="2"/>
+    </row>
+    <row r="3" spans="1:3" ht="101.5" customHeight="1" x14ac:dyDescent="0.45">
+      <c r="A3" s="14" t="s">
         <v>18</v>
       </c>
-      <c r="B4" s="26" t="s">
+      <c r="B3" s="25" t="s">
         <v>80</v>
       </c>
-    </row>
-    <row r="5" spans="1:2" ht="299.5" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="A5" s="15" t="s">
+      <c r="C3" s="35" t="s">
+        <v>94</v>
+      </c>
+    </row>
+    <row r="4" spans="1:3" ht="299.5" customHeight="1" x14ac:dyDescent="0.45">
+      <c r="A4" s="14" t="s">
         <v>44</v>
       </c>
-      <c r="B5" s="34" t="s">
+      <c r="B4" s="29" t="s">
         <v>78</v>
       </c>
-    </row>
-    <row r="6" spans="1:2" ht="409.6" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="A6" s="15" t="s">
+      <c r="C4" s="35" t="s">
+        <v>87</v>
+      </c>
+    </row>
+    <row r="5" spans="1:3" ht="409.6" customHeight="1" x14ac:dyDescent="0.45">
+      <c r="A5" s="14" t="s">
         <v>45</v>
       </c>
-      <c r="B6" s="34" t="s">
+      <c r="B5" s="29" t="s">
         <v>79</v>
       </c>
-    </row>
-    <row r="7" spans="1:2" ht="325.5" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="A7" s="15" t="s">
+      <c r="C5" s="35" t="s">
+        <v>86</v>
+      </c>
+    </row>
+    <row r="6" spans="1:3" ht="287.5" customHeight="1" x14ac:dyDescent="0.45">
+      <c r="A6" s="14" t="s">
         <v>46</v>
       </c>
-      <c r="B7" s="20" t="s">
+      <c r="B6" s="19" t="s">
         <v>81</v>
       </c>
-    </row>
-    <row r="8" spans="1:2" ht="101.5" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="A8" s="15" t="s">
+      <c r="C6" s="25" t="s">
+        <v>85</v>
+      </c>
+    </row>
+    <row r="7" spans="1:3" ht="101.5" customHeight="1" x14ac:dyDescent="0.45">
+      <c r="A7" s="14" t="s">
         <v>47</v>
       </c>
-      <c r="B8" s="20"/>
+      <c r="B7" s="19"/>
+      <c r="C7" s="2"/>
     </row>
   </sheetData>
+  <autoFilter ref="A1:C1" xr:uid="{9E9C4A99-AAB3-49B2-8D3F-2CED6FB92258}"/>
+  <phoneticPr fontId="1" type="noConversion"/>
+  <hyperlinks>
+    <hyperlink ref="C5" r:id="rId1" xr:uid="{E52E8DF3-B84E-42C5-9FFC-A4EBE3401B54}"/>
+    <hyperlink ref="C4" r:id="rId2" xr:uid="{7A2380C7-7E5C-4F7B-B405-1B457C17A70A}"/>
+    <hyperlink ref="C3" r:id="rId3" xr:uid="{3E0E18F4-DA1C-46B3-8C0E-EBB325BE9E25}"/>
+  </hyperlinks>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{41889BD0-A4A8-4188-AE8A-C708D84C89CC}">
+  <dimension ref="A1:C10"/>
+  <sheetFormatPr defaultRowHeight="17" x14ac:dyDescent="0.45"/>
+  <cols>
+    <col min="1" max="1" width="37.08203125" customWidth="1"/>
+    <col min="2" max="2" width="96.9140625" customWidth="1"/>
+    <col min="3" max="3" width="23.33203125" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:3" x14ac:dyDescent="0.45">
+      <c r="A1" s="36" t="s">
+        <v>92</v>
+      </c>
+      <c r="B1" s="36"/>
+      <c r="C1" s="36"/>
+    </row>
+    <row r="2" spans="1:3" ht="16.5" customHeight="1" x14ac:dyDescent="0.45">
+      <c r="A2" s="8" t="s">
+        <v>91</v>
+      </c>
+      <c r="B2" s="8" t="s">
+        <v>76</v>
+      </c>
+      <c r="C2" s="8" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="3" spans="1:3" x14ac:dyDescent="0.45">
+      <c r="A3" s="3" t="s">
+        <v>88</v>
+      </c>
+      <c r="B3" s="2" t="s">
+        <v>99</v>
+      </c>
+      <c r="C3" s="2"/>
+    </row>
+    <row r="4" spans="1:3" x14ac:dyDescent="0.45">
+      <c r="A4" s="3" t="s">
+        <v>95</v>
+      </c>
+      <c r="B4" s="38" t="s">
+        <v>100</v>
+      </c>
+      <c r="C4" s="2"/>
+    </row>
+    <row r="5" spans="1:3" ht="34" x14ac:dyDescent="0.45">
+      <c r="A5" s="3" t="s">
+        <v>96</v>
+      </c>
+      <c r="B5" s="38" t="s">
+        <v>101</v>
+      </c>
+      <c r="C5" s="2"/>
+    </row>
+    <row r="6" spans="1:3" ht="34" x14ac:dyDescent="0.45">
+      <c r="A6" s="3" t="s">
+        <v>89</v>
+      </c>
+      <c r="B6" s="38" t="s">
+        <v>98</v>
+      </c>
+      <c r="C6" s="2"/>
+    </row>
+    <row r="7" spans="1:3" ht="382.5" customHeight="1" x14ac:dyDescent="0.45">
+      <c r="A7" s="3" t="s">
+        <v>90</v>
+      </c>
+      <c r="B7" s="39" t="s">
+        <v>97</v>
+      </c>
+      <c r="C7" s="2"/>
+    </row>
+    <row r="10" spans="1:3" x14ac:dyDescent="0.45">
+      <c r="A10" s="37" t="s">
+        <v>93</v>
+      </c>
+      <c r="B10" s="37"/>
+      <c r="C10" s="37"/>
+    </row>
+  </sheetData>
+  <mergeCells count="2">
+    <mergeCell ref="A1:C1"/>
+    <mergeCell ref="A10:C10"/>
+  </mergeCells>
   <phoneticPr fontId="1" type="noConversion"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{69BE8514-AB01-4835-A33F-71EE9B36E5CF}">
   <dimension ref="A1:B14"/>
   <sheetFormatPr defaultRowHeight="17" x14ac:dyDescent="0.45"/>
@@ -1930,7 +2440,7 @@
       <c r="A3" s="2"/>
       <c r="B3" s="4"/>
     </row>
-    <row r="4" spans="1:2" ht="34" x14ac:dyDescent="0.45">
+    <row r="4" spans="1:2" x14ac:dyDescent="0.45">
       <c r="A4" s="7" t="s">
         <v>10</v>
       </c>
@@ -1942,7 +2452,7 @@
       </c>
       <c r="B5" s="4"/>
     </row>
-    <row r="6" spans="1:2" ht="51" x14ac:dyDescent="0.45">
+    <row r="6" spans="1:2" ht="34" x14ac:dyDescent="0.45">
       <c r="A6" s="7" t="s">
         <v>2</v>
       </c>
@@ -1966,13 +2476,13 @@
       </c>
       <c r="B9" s="4"/>
     </row>
-    <row r="10" spans="1:2" ht="34" x14ac:dyDescent="0.45">
+    <row r="10" spans="1:2" x14ac:dyDescent="0.45">
       <c r="A10" s="7" t="s">
         <v>6</v>
       </c>
       <c r="B10" s="4"/>
     </row>
-    <row r="11" spans="1:2" ht="34" x14ac:dyDescent="0.45">
+    <row r="11" spans="1:2" x14ac:dyDescent="0.45">
       <c r="A11" s="7" t="s">
         <v>7</v>
       </c>
@@ -2004,7 +2514,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{9F800CC1-8910-4E3F-9798-E9CC7FD99364}">
   <dimension ref="A1:A17"/>
   <sheetFormatPr defaultRowHeight="17" x14ac:dyDescent="0.45"/>
@@ -2013,83 +2523,77 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:1" ht="21" x14ac:dyDescent="0.45">
-      <c r="A1" s="32" t="s">
+      <c r="A1" s="27" t="s">
         <v>61</v>
       </c>
     </row>
     <row r="2" spans="1:1" x14ac:dyDescent="0.45">
-      <c r="A2" s="13" t="s">
+      <c r="A2" s="2" t="s">
         <v>62</v>
       </c>
     </row>
     <row r="3" spans="1:1" x14ac:dyDescent="0.45">
-      <c r="A3" s="31" t="s">
+      <c r="A3" s="3" t="s">
         <v>63</v>
       </c>
     </row>
     <row r="4" spans="1:1" x14ac:dyDescent="0.45">
-      <c r="A4" s="31" t="s">
+      <c r="A4" s="3" t="s">
         <v>64</v>
       </c>
     </row>
     <row r="5" spans="1:1" x14ac:dyDescent="0.45">
-      <c r="A5" s="31" t="s">
+      <c r="A5" s="3" t="s">
         <v>65</v>
       </c>
     </row>
     <row r="6" spans="1:1" x14ac:dyDescent="0.45">
-      <c r="A6" s="31" t="s">
+      <c r="A6" s="3" t="s">
         <v>66</v>
       </c>
     </row>
-    <row r="7" spans="1:1" x14ac:dyDescent="0.45">
-      <c r="A7" s="30"/>
-    </row>
     <row r="8" spans="1:1" ht="21" x14ac:dyDescent="0.45">
-      <c r="A8" s="32" t="s">
+      <c r="A8" s="27" t="s">
         <v>67</v>
       </c>
     </row>
     <row r="9" spans="1:1" x14ac:dyDescent="0.45">
-      <c r="A9" s="31" t="s">
+      <c r="A9" s="3" t="s">
         <v>68</v>
       </c>
     </row>
     <row r="10" spans="1:1" x14ac:dyDescent="0.45">
-      <c r="A10" s="31" t="s">
+      <c r="A10" s="3" t="s">
         <v>69</v>
       </c>
     </row>
     <row r="11" spans="1:1" x14ac:dyDescent="0.45">
-      <c r="A11" s="31" t="s">
+      <c r="A11" s="3" t="s">
         <v>70</v>
       </c>
     </row>
     <row r="12" spans="1:1" x14ac:dyDescent="0.45">
-      <c r="A12" s="31" t="s">
+      <c r="A12" s="3" t="s">
         <v>71</v>
       </c>
     </row>
-    <row r="13" spans="1:1" x14ac:dyDescent="0.45">
-      <c r="A13" s="30"/>
-    </row>
     <row r="14" spans="1:1" ht="21" x14ac:dyDescent="0.45">
-      <c r="A14" s="32" t="s">
+      <c r="A14" s="27" t="s">
         <v>72</v>
       </c>
     </row>
     <row r="15" spans="1:1" x14ac:dyDescent="0.45">
-      <c r="A15" s="13" t="s">
+      <c r="A15" s="2" t="s">
         <v>75</v>
       </c>
     </row>
     <row r="16" spans="1:1" x14ac:dyDescent="0.45">
-      <c r="A16" s="13" t="s">
+      <c r="A16" s="2" t="s">
         <v>73</v>
       </c>
     </row>
     <row r="17" spans="1:1" x14ac:dyDescent="0.45">
-      <c r="A17" s="13" t="s">
+      <c r="A17" s="2" t="s">
         <v>74</v>
       </c>
     </row>

</xml_diff>

<commit_message>
project 관련 파일 업로드_20260821
</commit_message>
<xml_diff>
--- a/Project_1/Project Status.xlsx
+++ b/Project_1/Project Status.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\pyostry\workspace\aiffel\ai-data-bootcamp\Project_1\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1C4A70F7-0946-42CC-9AAA-0C772D520FE5}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{960BF829-2DEC-47D0-BCD4-55A668DA426F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="30612" yWindow="-108" windowWidth="30936" windowHeight="16776" activeTab="3" xr2:uid="{6B636699-A6E6-472F-A92F-8A8168DF527A}"/>
   </bookViews>
@@ -33,7 +33,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="137" uniqueCount="102">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="139" uniqueCount="104">
   <si>
     <t>Dataset</t>
     <phoneticPr fontId="1" type="noConversion"/>
@@ -899,10 +899,6 @@
     <phoneticPr fontId="1" type="noConversion"/>
   </si>
   <si>
-    <t>데이터셋과 분석 방법의 선택 근거를 정리</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
     <t>항목</t>
     <phoneticPr fontId="1" type="noConversion"/>
   </si>
@@ -924,6 +920,41 @@
   </si>
   <si>
     <t>보조 질문 2개</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>자치구별 다음 분기 점포 순감소로 전환될 요식업 업종은 무엇일까?</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>1. 점포 순감소 전환 가능성은 자치구와 업종에 따라 어떻게 다른가?
+2. 매출, 유동인구, 점포 밀도 등 어떤 특성이 다음 분기 순감소 전환과 관련되는가?</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <r>
+      <t xml:space="preserve">1. 동일 업종이라도 자치구별 상권 유형에 따라 폐업위험이 다르다.
+</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FFFF0000"/>
+        <rFont val="맑은 고딕"/>
+        <family val="3"/>
+        <charset val="129"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>2. 발달상권 및 관광특구가 전통시장, 골목상권에 비해 폐업률이 낮을 것이다.</t>
+    </r>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t xml:space="preserve"> 분석 방법의 선택 근거를 정리</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>Dataset 정보</t>
     <phoneticPr fontId="1" type="noConversion"/>
   </si>
   <si>
@@ -937,7 +968,8 @@
         <charset val="129"/>
         <scheme val="minor"/>
       </rPr>
-      <t>데이터 출처</t>
+      <t xml:space="preserve">데이터 출처
+</t>
     </r>
     <r>
       <rPr>
@@ -948,10 +980,9 @@
         <charset val="129"/>
         <scheme val="minor"/>
       </rPr>
-      <t xml:space="preserve">: 서울 열린데이터광장(https://data.seoul.go.kr)
+      <t xml:space="preserve">서울 열린데이터광장(https://data.seoul.go.kr)
 서울시 상권분석서비스(https://golmok.seoul.go.kr/main.do)
 공공데이터포털(https://www.data.go.kr)
-서울시 상권분석서비스(추정매출-자치구)
 </t>
     </r>
     <r>
@@ -964,8 +995,7 @@
         <charset val="129"/>
         <scheme val="minor"/>
       </rPr>
-      <t>분석 방법:
-분석 대상:</t>
+      <t>Dataset</t>
     </r>
     <r>
       <rPr>
@@ -976,55 +1006,23 @@
         <charset val="129"/>
         <scheme val="minor"/>
       </rPr>
-      <t xml:space="preserve"> 서울시 25개 자치구 × 서비스업종 × 분기 패널 데이터
+      <t xml:space="preserve">
+서울시 상권분석서비스(점포-자치구)
+서울시 상권분석서비스(추정매출-자치구)
+서울시 상권분석서비스(점포-상권)
+서울시 상권분석서비스(점포-상권)_2024년
+서울시_상권분석서비스(점포-상권)_2023년
 </t>
     </r>
-    <r>
-      <rPr>
-        <b/>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="맑은 고딕"/>
-        <family val="3"/>
-        <charset val="129"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t>주 평가변수(핵심질문):</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="맑은 고딕"/>
-        <family val="2"/>
-        <charset val="129"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t xml:space="preserve"> 다음 분기 순감소 전환 여부(이진변수) — 패널 로지스틱 회귀(분기 고정효과 포함)로 분석
-</t>
-    </r>
-    <r>
-      <rPr>
-        <b/>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="맑은 고딕"/>
-        <family val="3"/>
-        <charset val="129"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t xml:space="preserve">주 평가변수(핵심질문): </t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="맑은 고딕"/>
-        <family val="2"/>
-        <charset val="129"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t>카이제곱·Kruskal-Wallis 검정 - 상권 유형·업종별 폐업위험 차이가 실제로 존재하는지 확인하고 Cramér’s V·</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <r>
+      <t xml:space="preserve">
+분석 방법:
+분석 대상: 서울시 25개 자치구 × 요식업 업종 × 분기 패널 데이터
+주 평가변수(핵심질문): 다음 분기 순감소 전환 여부(이진변수) — 패널 로지스틱 회귀(분기 고정효과 포함)로 분석
+주 평가변수(핵심질문): 카이제곱·Kruskal-Wallis 검정 - 상권 유형·업종별 폐업위험 차이가 실제로 존재하는지 확인하고 Cramér’s V·</t>
     </r>
     <r>
       <rPr>
@@ -1046,135 +1044,18 @@
         <scheme val="minor"/>
       </rPr>
       <t xml:space="preserve">²로 효과크기를 측정.
+PSM(성향점수매칭): 매출·유동인구·규모 등이 비슷한 상권끼리 매칭해 특정 조건에 따른 폐업위험 차이를 비교.
+로지스틱 회귀·랜덤포레스트·XGBoost -  현재 상권 정보로 다음 분기 폐업위험을 예측하고 모델 성능을 비교.
+SHAP - 최종 예측모델에서 매출·임대료·유동인구 등 어떤 변수가 폐업위험 판단에 크게 기여했는지 확인.
 </t>
     </r>
-    <r>
-      <rPr>
-        <b/>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="맑은 고딕"/>
-        <family val="3"/>
-        <charset val="129"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t>PSM(성향점수매칭):</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="맑은 고딕"/>
-        <family val="2"/>
-        <charset val="129"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t xml:space="preserve"> 매출·유동인구·규모 등이 비슷한 상권끼리 매칭해 특정 조건에 따른 폐업위험 차이를 비교.
-</t>
-    </r>
-    <r>
-      <rPr>
-        <b/>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="맑은 고딕"/>
-        <family val="3"/>
-        <charset val="129"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t>로지스틱 회귀·랜덤포레스트·XGBoost</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="맑은 고딕"/>
-        <family val="2"/>
-        <charset val="129"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t xml:space="preserve"> -  현재 상권 정보로 다음 분기 폐업위험을 예측하고 모델 성능을 비교.
-</t>
-    </r>
-    <r>
-      <rPr>
-        <b/>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="맑은 고딕"/>
-        <family val="3"/>
-        <charset val="129"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t>SHAP</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="맑은 고딕"/>
-        <family val="2"/>
-        <charset val="129"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t xml:space="preserve"> - 최종 예측모델에서 매출·임대료·유동인구 등 어떤 변수가 폐업위험 판단에 크게 기여했는지 확인.
-</t>
-    </r>
-    <r>
-      <rPr>
-        <b/>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="맑은 고딕"/>
-        <family val="3"/>
-        <charset val="129"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t xml:space="preserve">선택 근거:
-</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="맑은 고딕"/>
-        <family val="3"/>
-        <charset val="129"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t>23년 코로나 이후 상권 활성화 상태의 자료</t>
-    </r>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <r>
-      <t xml:space="preserve">1. 동일 업종이라도 자치구별 상권 유형에 따라 폐업위험이 다르다.
-</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color rgb="FFFF0000"/>
-        <rFont val="맑은 고딕"/>
-        <family val="3"/>
-        <charset val="129"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t>2. 신생 점포(개업 초기)는 기존 점포 대비 폐업위험이 높다.</t>
-    </r>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <t>서울시 상권 공공 데이터 기반 요식업 점포 폐업 위험 예측 조기 경보</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <t>자치구별 다음 분기 점포 순감소로 전환될 요식업 업종은 무엇일까?</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <t>1. 점포 순감소 전환 가능성은 자치구와 업종에 따라 어떻게 다른가?
-2. 매출, 유동인구, 점포 밀도 등 어떤 특성이 다음 분기 순감소 전환과 관련되는가?</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>소상공인시장진흥공단은 전국 소상공인의 경영안정과 폐업 예방을 지원하는 중소벤처기업부 산하 공공기관입니다.
+상권정보시스템을 통해 매출·유동인구·점포현황 데이터를 구축하여 경영컨설팅과 정책자금(저리융자, 임대료 지원 등) 배정에 활용하고 있으나현재는 이미 폐업이 발생한 이후 통계를 집계하는 사후적 방식에 머물러 있어, 한정된 예산을 어느 자치구·업종에 우선 배정할지 판단할 사전적 근거가 부족합니다.
+특히 요식업은 서울시 전체 폐업 건수 중 비중이 높다고 알려져 있고 자영업자 부채 문제와 직결되는 업종인 만큼, 다음 분기에 점포 수가 순감소로 전환될 가능성이 높은 자치구·업종을 조기에 식별해 컨설팅·자금 지원을 선제적으로 배정하기를 원합니다.
+소상공인시장진흥공단 정책기획팀에서 다음 분기 요식업 정책자금·컨설팅 예산 배정안을 수립해야 하는 입장입니다. 서울시 상권 공공 데이터를 기반으로하되 코로나 종식 이후인 2023년도 이후 데이터를 기준으로 다음 분기 요식업 점포 폐업 정보를 요청하였습니다.</t>
     <phoneticPr fontId="1" type="noConversion"/>
   </si>
 </sst>
@@ -1364,7 +1245,7 @@
       <alignment vertical="center"/>
     </xf>
   </cellStyleXfs>
-  <cellXfs count="40">
+  <cellXfs count="41">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0">
       <alignment vertical="center"/>
     </xf>
@@ -1464,26 +1345,29 @@
     <xf numFmtId="0" fontId="6" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="1" xfId="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="6" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="6" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="1" xfId="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
-    </xf>
     <xf numFmtId="0" fontId="2" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1">
+      <alignment vertical="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="2">
@@ -1922,20 +1806,20 @@
       <c r="D9" s="23"/>
     </row>
     <row r="10" spans="1:4" x14ac:dyDescent="0.45">
-      <c r="A10" s="33" t="s">
+      <c r="A10" s="36" t="s">
         <v>8</v>
       </c>
-      <c r="B10" s="34"/>
+      <c r="B10" s="37"/>
       <c r="C10" s="31">
         <v>46259.5</v>
       </c>
       <c r="D10" s="26"/>
     </row>
     <row r="11" spans="1:4" x14ac:dyDescent="0.45">
-      <c r="A11" s="33" t="s">
+      <c r="A11" s="36" t="s">
         <v>9</v>
       </c>
-      <c r="B11" s="34"/>
+      <c r="B11" s="37"/>
       <c r="C11" s="31">
         <v>46259.645833333336</v>
       </c>
@@ -2264,8 +2148,8 @@
       <c r="B3" s="25" t="s">
         <v>80</v>
       </c>
-      <c r="C3" s="35" t="s">
-        <v>94</v>
+      <c r="C3" s="33" t="s">
+        <v>93</v>
       </c>
     </row>
     <row r="4" spans="1:3" ht="299.5" customHeight="1" x14ac:dyDescent="0.45">
@@ -2275,7 +2159,7 @@
       <c r="B4" s="29" t="s">
         <v>78</v>
       </c>
-      <c r="C4" s="35" t="s">
+      <c r="C4" s="33" t="s">
         <v>87</v>
       </c>
     </row>
@@ -2286,7 +2170,7 @@
       <c r="B5" s="29" t="s">
         <v>79</v>
       </c>
-      <c r="C5" s="35" t="s">
+      <c r="C5" s="33" t="s">
         <v>86</v>
       </c>
     </row>
@@ -2325,53 +2209,53 @@
   <dimension ref="A1:C10"/>
   <sheetFormatPr defaultRowHeight="17" x14ac:dyDescent="0.45"/>
   <cols>
-    <col min="1" max="1" width="37.08203125" customWidth="1"/>
-    <col min="2" max="2" width="96.9140625" customWidth="1"/>
-    <col min="3" max="3" width="23.33203125" customWidth="1"/>
+    <col min="1" max="1" width="29.58203125" customWidth="1"/>
+    <col min="2" max="2" width="98" customWidth="1"/>
+    <col min="3" max="3" width="41.9140625" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:3" x14ac:dyDescent="0.45">
-      <c r="A1" s="36" t="s">
-        <v>92</v>
-      </c>
-      <c r="B1" s="36"/>
-      <c r="C1" s="36"/>
+      <c r="A1" s="38" t="s">
+        <v>91</v>
+      </c>
+      <c r="B1" s="38"/>
+      <c r="C1" s="38"/>
     </row>
     <row r="2" spans="1:3" ht="16.5" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="A2" s="8" t="s">
-        <v>91</v>
-      </c>
-      <c r="B2" s="8" t="s">
+      <c r="A2" s="9" t="s">
+        <v>90</v>
+      </c>
+      <c r="B2" s="9" t="s">
         <v>76</v>
       </c>
-      <c r="C2" s="8" t="s">
+      <c r="C2" s="9" t="s">
         <v>13</v>
       </c>
     </row>
-    <row r="3" spans="1:3" x14ac:dyDescent="0.45">
+    <row r="3" spans="1:3" ht="207.5" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A3" s="3" t="s">
         <v>88</v>
       </c>
-      <c r="B3" s="2" t="s">
-        <v>99</v>
+      <c r="B3" s="34" t="s">
+        <v>103</v>
       </c>
       <c r="C3" s="2"/>
     </row>
-    <row r="4" spans="1:3" x14ac:dyDescent="0.45">
+    <row r="4" spans="1:3" ht="25" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A4" s="3" t="s">
-        <v>95</v>
-      </c>
-      <c r="B4" s="38" t="s">
-        <v>100</v>
+        <v>94</v>
+      </c>
+      <c r="B4" s="34" t="s">
+        <v>96</v>
       </c>
       <c r="C4" s="2"/>
     </row>
     <row r="5" spans="1:3" ht="34" x14ac:dyDescent="0.45">
       <c r="A5" s="3" t="s">
-        <v>96</v>
-      </c>
-      <c r="B5" s="38" t="s">
-        <v>101</v>
+        <v>95</v>
+      </c>
+      <c r="B5" s="34" t="s">
+        <v>97</v>
       </c>
       <c r="C5" s="2"/>
     </row>
@@ -2379,26 +2263,35 @@
       <c r="A6" s="3" t="s">
         <v>89</v>
       </c>
-      <c r="B6" s="38" t="s">
+      <c r="B6" s="34" t="s">
         <v>98</v>
       </c>
       <c r="C6" s="2"/>
     </row>
-    <row r="7" spans="1:3" ht="382.5" customHeight="1" x14ac:dyDescent="0.45">
+    <row r="7" spans="1:3" ht="204" x14ac:dyDescent="0.45">
       <c r="A7" s="3" t="s">
-        <v>90</v>
-      </c>
-      <c r="B7" s="39" t="s">
-        <v>97</v>
-      </c>
-      <c r="C7" s="2"/>
+        <v>100</v>
+      </c>
+      <c r="B7" s="35" t="s">
+        <v>101</v>
+      </c>
+      <c r="C7" s="34"/>
+    </row>
+    <row r="8" spans="1:3" ht="221" x14ac:dyDescent="0.45">
+      <c r="A8" s="40" t="s">
+        <v>99</v>
+      </c>
+      <c r="B8" s="34" t="s">
+        <v>102</v>
+      </c>
+      <c r="C8" s="2"/>
     </row>
     <row r="10" spans="1:3" x14ac:dyDescent="0.45">
-      <c r="A10" s="37" t="s">
-        <v>93</v>
-      </c>
-      <c r="B10" s="37"/>
-      <c r="C10" s="37"/>
+      <c r="A10" s="39" t="s">
+        <v>92</v>
+      </c>
+      <c r="B10" s="39"/>
+      <c r="C10" s="39"/>
     </row>
   </sheetData>
   <mergeCells count="2">

</xml_diff>

<commit_message>
project 관련 파일 업로드_20260821_2
</commit_message>
<xml_diff>
--- a/Project_1/Project Status.xlsx
+++ b/Project_1/Project Status.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\pyostry\workspace\aiffel\ai-data-bootcamp\Project_1\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{960BF829-2DEC-47D0-BCD4-55A668DA426F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9A8C8186-2CDB-4A8C-B7E7-83F0CD17E58B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="30612" yWindow="-108" windowWidth="30936" windowHeight="16776" activeTab="3" xr2:uid="{6B636699-A6E6-472F-A92F-8A8168DF527A}"/>
   </bookViews>
@@ -33,7 +33,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="139" uniqueCount="104">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="141" uniqueCount="106">
   <si>
     <t>Dataset</t>
     <phoneticPr fontId="1" type="noConversion"/>
@@ -927,93 +927,11 @@
     <phoneticPr fontId="1" type="noConversion"/>
   </si>
   <si>
-    <t>1. 점포 순감소 전환 가능성은 자치구와 업종에 따라 어떻게 다른가?
-2. 매출, 유동인구, 점포 밀도 등 어떤 특성이 다음 분기 순감소 전환과 관련되는가?</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <r>
-      <t xml:space="preserve">1. 동일 업종이라도 자치구별 상권 유형에 따라 폐업위험이 다르다.
-</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color rgb="FFFF0000"/>
-        <rFont val="맑은 고딕"/>
-        <family val="3"/>
-        <charset val="129"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t>2. 발달상권 및 관광특구가 전통시장, 골목상권에 비해 폐업률이 낮을 것이다.</t>
-    </r>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
     <t xml:space="preserve"> 분석 방법의 선택 근거를 정리</t>
     <phoneticPr fontId="1" type="noConversion"/>
   </si>
   <si>
     <t>Dataset 정보</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <r>
-      <rPr>
-        <b/>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="맑은 고딕"/>
-        <family val="3"/>
-        <charset val="129"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t xml:space="preserve">데이터 출처
-</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="맑은 고딕"/>
-        <family val="2"/>
-        <charset val="129"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t xml:space="preserve">서울 열린데이터광장(https://data.seoul.go.kr)
-서울시 상권분석서비스(https://golmok.seoul.go.kr/main.do)
-공공데이터포털(https://www.data.go.kr)
-</t>
-    </r>
-    <r>
-      <rPr>
-        <b/>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="맑은 고딕"/>
-        <family val="3"/>
-        <charset val="129"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t>Dataset</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="맑은 고딕"/>
-        <family val="2"/>
-        <charset val="129"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t xml:space="preserve">
-서울시 상권분석서비스(점포-자치구)
-서울시 상권분석서비스(추정매출-자치구)
-서울시 상권분석서비스(점포-상권)
-서울시 상권분석서비스(점포-상권)_2024년
-서울시_상권분석서비스(점포-상권)_2023년
-</t>
-    </r>
     <phoneticPr fontId="1" type="noConversion"/>
   </si>
   <si>
@@ -1056,6 +974,99 @@
 상권정보시스템을 통해 매출·유동인구·점포현황 데이터를 구축하여 경영컨설팅과 정책자금(저리융자, 임대료 지원 등) 배정에 활용하고 있으나현재는 이미 폐업이 발생한 이후 통계를 집계하는 사후적 방식에 머물러 있어, 한정된 예산을 어느 자치구·업종에 우선 배정할지 판단할 사전적 근거가 부족합니다.
 특히 요식업은 서울시 전체 폐업 건수 중 비중이 높다고 알려져 있고 자영업자 부채 문제와 직결되는 업종인 만큼, 다음 분기에 점포 수가 순감소로 전환될 가능성이 높은 자치구·업종을 조기에 식별해 컨설팅·자금 지원을 선제적으로 배정하기를 원합니다.
 소상공인시장진흥공단 정책기획팀에서 다음 분기 요식업 정책자금·컨설팅 예산 배정안을 수립해야 하는 입장입니다. 서울시 상권 공공 데이터를 기반으로하되 코로나 종식 이후인 2023년도 이후 데이터를 기준으로 다음 분기 요식업 점포 폐업 정보를 요청하였습니다.</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>1. 동일 업종이라도 자치구별 상권 유형에 따라 폐업위험이 다르다.
+2. 골목상권의 순감소 위험이 높은 업종의 경우, 점포 규모와 유동인구를 맞추면 타 업종과 순감소 격차가 줄어들 것이다.</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>1. 동일 업종이라도 자치구별 상권 유형에 따라 폐업 위험에 차이가 있는가?
+2. 매출, 유동인구, 점포 밀도 등 어떤 특성이 다음 분기 순감소 전환과 관련되는가?</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="맑은 고딕"/>
+        <family val="3"/>
+        <charset val="129"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">데이터 출처
+</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="맑은 고딕"/>
+        <family val="2"/>
+        <charset val="129"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">서울 열린데이터광장(https://data.seoul.go.kr)
+서울시 상권분석서비스(https://golmok.seoul.go.kr/main.do)
+공공데이터포털(https://www.data.go.kr)
+</t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="맑은 고딕"/>
+        <family val="3"/>
+        <charset val="129"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>Dataset</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="맑은 고딕"/>
+        <family val="2"/>
+        <charset val="129"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">
+1. 서울시 상권분석서비스(점포-자치구)
+2. 서울시 상권분석서비스(추정매출-자치구)
+</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="맑은 고딕"/>
+        <family val="3"/>
+        <charset val="129"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>3. 서울시 상권분석서비스(소비-상권)
+4. 서울시 상권분석서비스(길단위인구-자치구)
+5. 서울시 상권분석서비스(점포-상권)
+6. 서울시 상권분석서비스(점포-상권)_2024년
+7. 서울시_상권분석서비스(점포-상권)_2023년
+8. 서울시 상권분석서비스(상권변화지표-자치구)
+9. 서울시 상권분석서비스(영역-상권)
+10. 서울시 상권분석서비스(집객시설-상권)</t>
+    </r>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>서울시 상권분석서비스(추정매출-자치구) 데이터의 당월_매출_금액은 해당 분기(3개월) 합산 금액</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>가설 1: 표시철, 유서영
+가설 2: 지선호, 오지운</t>
     <phoneticPr fontId="1" type="noConversion"/>
   </si>
 </sst>
@@ -1139,14 +1150,6 @@
     </font>
     <font>
       <sz val="11"/>
-      <color rgb="FFFF0000"/>
-      <name val="맑은 고딕"/>
-      <family val="3"/>
-      <charset val="129"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <sz val="11"/>
       <color theme="1"/>
       <name val="맑은 고딕"/>
       <family val="3"/>
@@ -1160,8 +1163,15 @@
       <family val="2"/>
       <charset val="161"/>
     </font>
+    <font>
+      <sz val="11"/>
+      <name val="맑은 고딕"/>
+      <family val="3"/>
+      <charset val="129"/>
+      <scheme val="minor"/>
+    </font>
   </fonts>
-  <fills count="5">
+  <fills count="6">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -1183,6 +1193,12 @@
     <fill>
       <patternFill patternType="solid">
         <fgColor theme="7" tint="0.79998168889431442"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFFFF00"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
@@ -1245,7 +1261,7 @@
       <alignment vertical="center"/>
     </xf>
   </cellStyleXfs>
-  <cellXfs count="41">
+  <cellXfs count="42">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0">
       <alignment vertical="center"/>
     </xf>
@@ -1351,7 +1367,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="10" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="6" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
@@ -1366,8 +1382,11 @@
     <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1">
-      <alignment vertical="center"/>
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="5" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="2">
@@ -2209,8 +2228,8 @@
   <dimension ref="A1:C10"/>
   <sheetFormatPr defaultRowHeight="17" x14ac:dyDescent="0.45"/>
   <cols>
-    <col min="1" max="1" width="29.58203125" customWidth="1"/>
-    <col min="2" max="2" width="98" customWidth="1"/>
+    <col min="1" max="1" width="28.25" customWidth="1"/>
+    <col min="2" max="2" width="100.4140625" customWidth="1"/>
     <col min="3" max="3" width="41.9140625" customWidth="1"/>
   </cols>
   <sheetData>
@@ -2237,7 +2256,7 @@
         <v>88</v>
       </c>
       <c r="B3" s="34" t="s">
-        <v>103</v>
+        <v>100</v>
       </c>
       <c r="C3" s="2"/>
     </row>
@@ -2255,34 +2274,38 @@
         <v>95</v>
       </c>
       <c r="B5" s="34" t="s">
-        <v>97</v>
+        <v>102</v>
       </c>
       <c r="C5" s="2"/>
     </row>
-    <row r="6" spans="1:3" ht="34" x14ac:dyDescent="0.45">
+    <row r="6" spans="1:3" ht="43.5" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A6" s="3" t="s">
         <v>89</v>
       </c>
-      <c r="B6" s="34" t="s">
+      <c r="B6" s="40" t="s">
+        <v>101</v>
+      </c>
+      <c r="C6" s="34" t="s">
+        <v>105</v>
+      </c>
+    </row>
+    <row r="7" spans="1:3" ht="272" x14ac:dyDescent="0.45">
+      <c r="A7" s="3" t="s">
         <v>98</v>
       </c>
-      <c r="C6" s="2"/>
-    </row>
-    <row r="7" spans="1:3" ht="204" x14ac:dyDescent="0.45">
-      <c r="A7" s="3" t="s">
-        <v>100</v>
-      </c>
       <c r="B7" s="35" t="s">
-        <v>101</v>
-      </c>
-      <c r="C7" s="34"/>
+        <v>103</v>
+      </c>
+      <c r="C7" s="29" t="s">
+        <v>104</v>
+      </c>
     </row>
     <row r="8" spans="1:3" ht="221" x14ac:dyDescent="0.45">
-      <c r="A8" s="40" t="s">
+      <c r="A8" s="3" t="s">
+        <v>97</v>
+      </c>
+      <c r="B8" s="41" t="s">
         <v>99</v>
-      </c>
-      <c r="B8" s="34" t="s">
-        <v>102</v>
       </c>
       <c r="C8" s="2"/>
     </row>

</xml_diff>

<commit_message>
project 관련 파일 업로드_20260821_3
</commit_message>
<xml_diff>
--- a/Project_1/Project Status.xlsx
+++ b/Project_1/Project Status.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\pyostry\workspace\aiffel\ai-data-bootcamp\Project_1\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9A8C8186-2CDB-4A8C-B7E7-83F0CD17E58B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{CB5C415B-0EE9-4C57-A864-DD17D04C780A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="30612" yWindow="-108" windowWidth="30936" windowHeight="16776" activeTab="3" xr2:uid="{6B636699-A6E6-472F-A92F-8A8168DF527A}"/>
   </bookViews>
@@ -17,8 +17,9 @@
     <sheet name="1. Dataset type" sheetId="2" r:id="rId2"/>
     <sheet name="2. 문제 정의와 분석 설계" sheetId="5" r:id="rId3"/>
     <sheet name="3. 분석 계획서" sheetId="7" r:id="rId4"/>
-    <sheet name="발표자료 목차" sheetId="1" r:id="rId5"/>
-    <sheet name="평가 사항" sheetId="4" r:id="rId6"/>
+    <sheet name="4. 데이터 이해와 전처리" sheetId="8" r:id="rId5"/>
+    <sheet name="발표자료 목차" sheetId="1" r:id="rId6"/>
+    <sheet name="평가 사항" sheetId="4" r:id="rId7"/>
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'2. 문제 정의와 분석 설계'!$A$1:$C$1</definedName>
@@ -33,7 +34,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="141" uniqueCount="106">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="146" uniqueCount="107">
   <si>
     <t>Dataset</t>
     <phoneticPr fontId="1" type="noConversion"/>
@@ -928,10 +929,6 @@
   </si>
   <si>
     <t xml:space="preserve"> 분석 방법의 선택 근거를 정리</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <t>Dataset 정보</t>
     <phoneticPr fontId="1" type="noConversion"/>
   </si>
   <si>
@@ -1067,6 +1064,15 @@
   <si>
     <t>가설 1: 표시철, 유서영
 가설 2: 지선호, 오지운</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>Dataset 상세 정보</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t xml:space="preserve">1. 각 Data의 [기준_년분기_코드]는 2023년 1분기 ~ 2025년 4분기까지 사용할 예정.
+</t>
     <phoneticPr fontId="1" type="noConversion"/>
   </si>
 </sst>
@@ -1261,7 +1267,7 @@
       <alignment vertical="center"/>
     </xf>
   </cellStyleXfs>
-  <cellXfs count="42">
+  <cellXfs count="45">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0">
       <alignment vertical="center"/>
     </xf>
@@ -1387,6 +1393,15 @@
     </xf>
     <xf numFmtId="0" fontId="0" fillId="5" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyBorder="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="2">
@@ -1404,6 +1419,61 @@
     </ext>
   </extLst>
 </styleSheet>
+</file>
+
+<file path=xl/drawings/drawing1.xml><?xml version="1.0" encoding="utf-8"?>
+<xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+  <xdr:twoCellAnchor editAs="oneCell">
+    <xdr:from>
+      <xdr:col>0</xdr:col>
+      <xdr:colOff>943831</xdr:colOff>
+      <xdr:row>11</xdr:row>
+      <xdr:rowOff>174213</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>2</xdr:col>
+      <xdr:colOff>915669</xdr:colOff>
+      <xdr:row>13</xdr:row>
+      <xdr:rowOff>1911887</xdr:rowOff>
+    </xdr:to>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="5" name="그림 4">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{F6B8DBC1-F950-3C57-0EA8-A911A664EECF}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvPicPr>
+          <a:picLocks noChangeAspect="1"/>
+        </xdr:cNvPicPr>
+      </xdr:nvPicPr>
+      <xdr:blipFill>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId1" cstate="print">
+          <a:extLst>
+            <a:ext uri="{28A0092B-C50C-407E-A947-70E740481C1C}">
+              <a14:useLocalDpi xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main" val="0"/>
+            </a:ext>
+          </a:extLst>
+        </a:blip>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </xdr:blipFill>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="943831" y="12536542"/>
+          <a:ext cx="10272285" cy="5861439"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+</xdr:wsDr>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -2225,12 +2295,13 @@
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{41889BD0-A4A8-4188-AE8A-C708D84C89CC}">
-  <dimension ref="A1:C10"/>
+  <dimension ref="A1:C14"/>
   <sheetFormatPr defaultRowHeight="17" x14ac:dyDescent="0.45"/>
   <cols>
     <col min="1" max="1" width="28.25" customWidth="1"/>
-    <col min="2" max="2" width="100.4140625" customWidth="1"/>
+    <col min="2" max="2" width="106.75" customWidth="1"/>
     <col min="3" max="3" width="41.9140625" customWidth="1"/>
+    <col min="4" max="16384" width="8.6640625" style="43"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:3" x14ac:dyDescent="0.45">
@@ -2256,7 +2327,7 @@
         <v>88</v>
       </c>
       <c r="B3" s="34" t="s">
-        <v>100</v>
+        <v>99</v>
       </c>
       <c r="C3" s="2"/>
     </row>
@@ -2274,59 +2345,112 @@
         <v>95</v>
       </c>
       <c r="B5" s="34" t="s">
-        <v>102</v>
+        <v>101</v>
       </c>
       <c r="C5" s="2"/>
     </row>
-    <row r="6" spans="1:3" ht="43.5" customHeight="1" x14ac:dyDescent="0.45">
+    <row r="6" spans="1:3" ht="34" x14ac:dyDescent="0.45">
       <c r="A6" s="3" t="s">
         <v>89</v>
       </c>
       <c r="B6" s="40" t="s">
-        <v>101</v>
+        <v>100</v>
       </c>
       <c r="C6" s="34" t="s">
+        <v>104</v>
+      </c>
+    </row>
+    <row r="7" spans="1:3" ht="282.5" customHeight="1" x14ac:dyDescent="0.45">
+      <c r="A7" s="3" t="s">
+        <v>0</v>
+      </c>
+      <c r="B7" s="35" t="s">
+        <v>102</v>
+      </c>
+      <c r="C7" s="29" t="s">
+        <v>103</v>
+      </c>
+    </row>
+    <row r="8" spans="1:3" ht="101.5" customHeight="1" x14ac:dyDescent="0.45">
+      <c r="A8" s="3" t="s">
         <v>105</v>
       </c>
-    </row>
-    <row r="7" spans="1:3" ht="272" x14ac:dyDescent="0.45">
-      <c r="A7" s="3" t="s">
+      <c r="B8" s="35" t="s">
+        <v>106</v>
+      </c>
+      <c r="C8" s="29"/>
+    </row>
+    <row r="9" spans="1:3" ht="221" x14ac:dyDescent="0.45">
+      <c r="A9" s="3" t="s">
+        <v>97</v>
+      </c>
+      <c r="B9" s="41" t="s">
         <v>98</v>
       </c>
-      <c r="B7" s="35" t="s">
-        <v>103</v>
-      </c>
-      <c r="C7" s="29" t="s">
-        <v>104</v>
-      </c>
-    </row>
-    <row r="8" spans="1:3" ht="221" x14ac:dyDescent="0.45">
-      <c r="A8" s="3" t="s">
-        <v>97</v>
-      </c>
-      <c r="B8" s="41" t="s">
-        <v>99</v>
-      </c>
-      <c r="C8" s="2"/>
-    </row>
-    <row r="10" spans="1:3" x14ac:dyDescent="0.45">
-      <c r="A10" s="39" t="s">
+      <c r="C9" s="2"/>
+    </row>
+    <row r="11" spans="1:3" x14ac:dyDescent="0.45">
+      <c r="A11" s="39" t="s">
         <v>92</v>
       </c>
-      <c r="B10" s="39"/>
-      <c r="C10" s="39"/>
+      <c r="B11" s="39"/>
+      <c r="C11" s="39"/>
+    </row>
+    <row r="12" spans="1:3" s="44" customFormat="1" ht="162" customHeight="1" x14ac:dyDescent="0.45">
+      <c r="A12" s="42"/>
+      <c r="B12" s="42"/>
+      <c r="C12" s="42"/>
+    </row>
+    <row r="13" spans="1:3" s="44" customFormat="1" ht="162" customHeight="1" x14ac:dyDescent="0.45">
+      <c r="A13" s="42"/>
+      <c r="B13" s="42"/>
+      <c r="C13" s="42"/>
+    </row>
+    <row r="14" spans="1:3" s="44" customFormat="1" ht="162" customHeight="1" x14ac:dyDescent="0.45">
+      <c r="A14" s="42"/>
+      <c r="B14" s="42"/>
+      <c r="C14" s="42"/>
     </row>
   </sheetData>
-  <mergeCells count="2">
+  <mergeCells count="3">
     <mergeCell ref="A1:C1"/>
-    <mergeCell ref="A10:C10"/>
+    <mergeCell ref="A11:C11"/>
+    <mergeCell ref="A12:C14"/>
   </mergeCells>
+  <phoneticPr fontId="1" type="noConversion"/>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <drawing r:id="rId1"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{1402F3D2-E44E-49CC-8D75-9BA854A3E719}">
+  <dimension ref="A1:C1"/>
+  <sheetFormatPr defaultRowHeight="17" x14ac:dyDescent="0.45"/>
+  <cols>
+    <col min="1" max="1" width="25.9140625" customWidth="1"/>
+    <col min="2" max="2" width="63.83203125" customWidth="1"/>
+    <col min="3" max="3" width="16.25" bestFit="1" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:3" x14ac:dyDescent="0.45">
+      <c r="A1" s="8" t="s">
+        <v>11</v>
+      </c>
+      <c r="B1" s="9" t="s">
+        <v>76</v>
+      </c>
+      <c r="C1" s="9" t="s">
+        <v>48</v>
+      </c>
+    </row>
+  </sheetData>
   <phoneticPr fontId="1" type="noConversion"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{69BE8514-AB01-4835-A33F-71EE9B36E5CF}">
   <dimension ref="A1:B14"/>
   <sheetFormatPr defaultRowHeight="17" x14ac:dyDescent="0.45"/>
@@ -2430,7 +2554,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{9F800CC1-8910-4E3F-9798-E9CC7FD99364}">
   <dimension ref="A1:A17"/>
   <sheetFormatPr defaultRowHeight="17" x14ac:dyDescent="0.45"/>

</xml_diff>

<commit_message>
project 관련 파일 업로드_20260821_4
</commit_message>
<xml_diff>
--- a/Project_1/Project Status.xlsx
+++ b/Project_1/Project Status.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\pyostry\workspace\aiffel\ai-data-bootcamp\Project_1\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{CB5C415B-0EE9-4C57-A864-DD17D04C780A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1A4AF439-D055-4D61-8723-26FBFACF8B71}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="30612" yWindow="-108" windowWidth="30936" windowHeight="16776" activeTab="3" xr2:uid="{6B636699-A6E6-472F-A92F-8A8168DF527A}"/>
+    <workbookView xWindow="30612" yWindow="-108" windowWidth="30936" windowHeight="16776" activeTab="4" xr2:uid="{6B636699-A6E6-472F-A92F-8A8168DF527A}"/>
   </bookViews>
   <sheets>
     <sheet name="0. Status" sheetId="3" r:id="rId1"/>
@@ -21,8 +21,12 @@
     <sheet name="발표자료 목차" sheetId="1" r:id="rId6"/>
     <sheet name="평가 사항" sheetId="4" r:id="rId7"/>
   </sheets>
+  <externalReferences>
+    <externalReference r:id="rId8"/>
+  </externalReferences>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'2. 문제 정의와 분석 설계'!$A$1:$C$1</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">'4. 데이터 이해와 전처리'!$B$2:$G$2</definedName>
   </definedNames>
   <calcPr calcId="191029"/>
   <extLst>
@@ -34,7 +38,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="146" uniqueCount="107">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="505" uniqueCount="268">
   <si>
     <t>Dataset</t>
     <phoneticPr fontId="1" type="noConversion"/>
@@ -932,41 +936,6 @@
     <phoneticPr fontId="1" type="noConversion"/>
   </si>
   <si>
-    <r>
-      <t xml:space="preserve">
-분석 방법:
-분석 대상: 서울시 25개 자치구 × 요식업 업종 × 분기 패널 데이터
-주 평가변수(핵심질문): 다음 분기 순감소 전환 여부(이진변수) — 패널 로지스틱 회귀(분기 고정효과 포함)로 분석
-주 평가변수(핵심질문): 카이제곱·Kruskal-Wallis 검정 - 상권 유형·업종별 폐업위험 차이가 실제로 존재하는지 확인하고 Cramér’s V·</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <charset val="161"/>
-      </rPr>
-      <t>ε</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="맑은 고딕"/>
-        <family val="2"/>
-        <charset val="129"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t xml:space="preserve">²로 효과크기를 측정.
-PSM(성향점수매칭): 매출·유동인구·규모 등이 비슷한 상권끼리 매칭해 특정 조건에 따른 폐업위험 차이를 비교.
-로지스틱 회귀·랜덤포레스트·XGBoost -  현재 상권 정보로 다음 분기 폐업위험을 예측하고 모델 성능을 비교.
-SHAP - 최종 예측모델에서 매출·임대료·유동인구 등 어떤 변수가 폐업위험 판단에 크게 기여했는지 확인.
-</t>
-    </r>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
     <t>소상공인시장진흥공단은 전국 소상공인의 경영안정과 폐업 예방을 지원하는 중소벤처기업부 산하 공공기관입니다.
 상권정보시스템을 통해 매출·유동인구·점포현황 데이터를 구축하여 경영컨설팅과 정책자금(저리융자, 임대료 지원 등) 배정에 활용하고 있으나현재는 이미 폐업이 발생한 이후 통계를 집계하는 사후적 방식에 머물러 있어, 한정된 예산을 어느 자치구·업종에 우선 배정할지 판단할 사전적 근거가 부족합니다.
 특히 요식업은 서울시 전체 폐업 건수 중 비중이 높다고 알려져 있고 자영업자 부채 문제와 직결되는 업종인 만큼, 다음 분기에 점포 수가 순감소로 전환될 가능성이 높은 자치구·업종을 조기에 식별해 컨설팅·자금 지원을 선제적으로 배정하기를 원합니다.
@@ -1058,21 +1027,542 @@
     <phoneticPr fontId="1" type="noConversion"/>
   </si>
   <si>
-    <t>서울시 상권분석서비스(추정매출-자치구) 데이터의 당월_매출_금액은 해당 분기(3개월) 합산 금액</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
     <t>가설 1: 표시철, 유서영
 가설 2: 지선호, 오지운</t>
     <phoneticPr fontId="1" type="noConversion"/>
   </si>
   <si>
-    <t>Dataset 상세 정보</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <t xml:space="preserve">1. 각 Data의 [기준_년분기_코드]는 2023년 1분기 ~ 2025년 4분기까지 사용할 예정.
-</t>
+    <t>서울시 상권분석서비스(추정매출-자치구) 데이터의 당월_매출_금액은 해당 분기(3개월) 합산 금액
+1. 각 Data의 [기준_년분기_코드]는 2023년 1분기 ~ 2025년 4분기까지 사용할 예정.</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>데이터셋 정보</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>점포-자치구</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>기준_년분기_코드</t>
+  </si>
+  <si>
+    <t>int64</t>
+  </si>
+  <si>
+    <t>자치구_코드</t>
+  </si>
+  <si>
+    <t>자치구_코드_명</t>
+  </si>
+  <si>
+    <t>str</t>
+  </si>
+  <si>
+    <t>서비스_업종_코드</t>
+  </si>
+  <si>
+    <t>서비스_업종_코드_명</t>
+  </si>
+  <si>
+    <t>전체_점포_수</t>
+  </si>
+  <si>
+    <t>일반_점포_수</t>
+  </si>
+  <si>
+    <t>프랜차이즈_점포_수</t>
+  </si>
+  <si>
+    <t>개업_율</t>
+  </si>
+  <si>
+    <t>float64</t>
+  </si>
+  <si>
+    <t>개업_점포_수</t>
+  </si>
+  <si>
+    <t>폐업_률</t>
+  </si>
+  <si>
+    <t>Name</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>Non-Null Count</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>#</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>Column</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>폐업_점포_수</t>
+  </si>
+  <si>
+    <t>폐업_점포_수</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>Dtype</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>Comment</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>분기 =  [20231, 20232, 20233, 20234, 20241, 20242, 20243, 20244, 20251, 20252, 20253, 20254] 기준으로 필터링</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>업종 = {"CS100001": "한식음식점", "CS100002": "중식음식점", "CS100003": "일식음식점", "CS100004": "양식음식점", "CS100005": "제과점", "CS100006": "패스트푸드점", "CS100007": "치킨전문점", "CS100008": "분식전문점", "CS100009": "호프-간이주점", "CS100010": "커피-음료",} 기준으로 필터링</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>프랜차이즈_점포_수</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>[일반_점포_수] + [프랜차이즈_점포_수]의 합</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>당월_매출_금액</t>
+  </si>
+  <si>
+    <t>당월_매출_건수</t>
+  </si>
+  <si>
+    <t>주중_매출_금액</t>
+  </si>
+  <si>
+    <t>주말_매출_금액</t>
+  </si>
+  <si>
+    <t>월요일_매출_금액</t>
+  </si>
+  <si>
+    <t>화요일_매출_금액</t>
+  </si>
+  <si>
+    <t>수요일_매출_금액</t>
+  </si>
+  <si>
+    <t>목요일_매출_금액</t>
+  </si>
+  <si>
+    <t>금요일_매출_금액</t>
+  </si>
+  <si>
+    <t>토요일_매출_금액</t>
+  </si>
+  <si>
+    <t>일요일_매출_금액</t>
+  </si>
+  <si>
+    <t>시간대_00~06_매출_금액</t>
+  </si>
+  <si>
+    <t>시간대_06~11_매출_금액</t>
+  </si>
+  <si>
+    <t>시간대_11~14_매출_금액</t>
+  </si>
+  <si>
+    <t>시간대_14~17_매출_금액</t>
+  </si>
+  <si>
+    <t>시간대_17~21_매출_금액</t>
+  </si>
+  <si>
+    <t>시간대_21~24_매출_금액</t>
+  </si>
+  <si>
+    <t>남성_매출_금액</t>
+  </si>
+  <si>
+    <t>여성_매출_금액</t>
+  </si>
+  <si>
+    <t>연령대_10_매출_금액</t>
+  </si>
+  <si>
+    <t>연령대_20_매출_금액</t>
+  </si>
+  <si>
+    <t>연령대_30_매출_금액</t>
+  </si>
+  <si>
+    <t>연령대_40_매출_금액</t>
+  </si>
+  <si>
+    <t>연령대_50_매출_금액</t>
+  </si>
+  <si>
+    <t>연령대_60_이상_매출_금액</t>
+  </si>
+  <si>
+    <t>주중_매출_건수</t>
+  </si>
+  <si>
+    <t>주말_매출_건수</t>
+  </si>
+  <si>
+    <t>월요일_매출_건수</t>
+  </si>
+  <si>
+    <t>화요일_매출_건수</t>
+  </si>
+  <si>
+    <t>수요일_매출_건수</t>
+  </si>
+  <si>
+    <t>목요일_매출_건수</t>
+  </si>
+  <si>
+    <t>금요일_매출_건수</t>
+  </si>
+  <si>
+    <t>토요일_매출_건수</t>
+  </si>
+  <si>
+    <t>일요일_매출_건수</t>
+  </si>
+  <si>
+    <t>시간대_건수~06_매출_건수</t>
+  </si>
+  <si>
+    <t>시간대_건수~11_매출_건수</t>
+  </si>
+  <si>
+    <t>시간대_건수~14_매출_건수</t>
+  </si>
+  <si>
+    <t>시간대_건수~17_매출_건수</t>
+  </si>
+  <si>
+    <t>시간대_건수~21_매출_건수</t>
+  </si>
+  <si>
+    <t>시간대_건수~24_매출_건수</t>
+  </si>
+  <si>
+    <t>남성_매출_건수</t>
+  </si>
+  <si>
+    <t>여성_매출_건수</t>
+  </si>
+  <si>
+    <t>연령대_10_매출_건수</t>
+  </si>
+  <si>
+    <t>연령대_20_매출_건수</t>
+  </si>
+  <si>
+    <t>연령대_30_매출_건수</t>
+  </si>
+  <si>
+    <t>연령대_40_매출_건수</t>
+  </si>
+  <si>
+    <t>연령대_50_매출_건수</t>
+  </si>
+  <si>
+    <t>연령대_60_이상_매출_건수</t>
+  </si>
+  <si>
+    <t>추정매출_자치구</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>해당 분기(3개월) 총 매출 금액</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>상권_구분_코드</t>
+  </si>
+  <si>
+    <t>상권_구분_코드_명</t>
+  </si>
+  <si>
+    <t>상권_코드</t>
+  </si>
+  <si>
+    <t>상권_코드_명</t>
+  </si>
+  <si>
+    <t>집객시설_수</t>
+  </si>
+  <si>
+    <t>관공서_수</t>
+  </si>
+  <si>
+    <t>은행_수</t>
+  </si>
+  <si>
+    <t>종합병원_수</t>
+  </si>
+  <si>
+    <t>일반_병원_수</t>
+  </si>
+  <si>
+    <t>약국_수</t>
+  </si>
+  <si>
+    <t>유치원_수</t>
+  </si>
+  <si>
+    <t>초등학교_수</t>
+  </si>
+  <si>
+    <t>중학교_수</t>
+  </si>
+  <si>
+    <t>고등학교_수</t>
+  </si>
+  <si>
+    <t>대학교_수</t>
+  </si>
+  <si>
+    <t>백화점_수</t>
+  </si>
+  <si>
+    <t>슈퍼마켓_수</t>
+  </si>
+  <si>
+    <t>극장_수</t>
+  </si>
+  <si>
+    <t>숙박_시설_수</t>
+  </si>
+  <si>
+    <t>공항_수</t>
+  </si>
+  <si>
+    <t>철도_역_수</t>
+  </si>
+  <si>
+    <t>버스_터미널_수</t>
+  </si>
+  <si>
+    <t>지하철_역_수</t>
+  </si>
+  <si>
+    <t>버스_정거장_수</t>
+  </si>
+  <si>
+    <t>집객시설_상권</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t xml:space="preserve"> </t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>분석 방법</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>No</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>점포-상권</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>2023, 2024년 점포-상권 Dataset의 경우 [점포_수]로 확인되어 2026년 Data 기준 [일반_점포_수]로 컬럼명 통일 후 병합하였습니다.</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>[일반_점포_수] + [프랜차이즈_점포_수]의 합
+2023, 2024년 점포-상권 Dataset의 경우 [유사_점포_수]로 확인되어 2026년 Data 기준 [전체_점포_수]로 컬럼명 통일 후 병합하였습니다.</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>행정동_코드</t>
+  </si>
+  <si>
+    <t>행정동_코드_명</t>
+  </si>
+  <si>
+    <t>지출_총금액</t>
+  </si>
+  <si>
+    <t>식료품_지출_총금액</t>
+  </si>
+  <si>
+    <t>의류_신발_지출_총금액</t>
+  </si>
+  <si>
+    <t>생활용품_지출_총금액</t>
+  </si>
+  <si>
+    <t>의료비_지출_총금액</t>
+  </si>
+  <si>
+    <t>교통_지출_총금액</t>
+  </si>
+  <si>
+    <t>교육_지출_총금액</t>
+  </si>
+  <si>
+    <t>유흥_지출_총금액</t>
+  </si>
+  <si>
+    <t>여가_문화_지출_총금액</t>
+  </si>
+  <si>
+    <t>기타_지출_총금액</t>
+  </si>
+  <si>
+    <t>음식_지출_총금액</t>
+  </si>
+  <si>
+    <t>소비_자치구</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>분기 =  [20231, 20232, 20233, 20234, 20241, 20242, 20243, 20244, 20251, 20252, 20253, 20254, 20261] 기준으로 필터링</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>길단위인구-자치구</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>영역-상권</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>엑스좌표_값</t>
+  </si>
+  <si>
+    <t>와이좌표_값</t>
+  </si>
+  <si>
+    <t>영역_면적</t>
+  </si>
+  <si>
+    <t>상권변화지표-자치구</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>상권_변화_지표</t>
+  </si>
+  <si>
+    <t>상권_변화_지표_명</t>
+  </si>
+  <si>
+    <t>운영_영업_개월_평균</t>
+  </si>
+  <si>
+    <t>폐업_영업_개월_평균</t>
+  </si>
+  <si>
+    <t>서울_운영_영업_개월_평균</t>
+  </si>
+  <si>
+    <t>서울_폐업_영업_개월_평균</t>
+  </si>
+  <si>
+    <t>총_유동인구_수</t>
+  </si>
+  <si>
+    <t>남성_유동인구_수</t>
+  </si>
+  <si>
+    <t>여성_유동인구_수</t>
+  </si>
+  <si>
+    <t>연령대_10_유동인구_수</t>
+  </si>
+  <si>
+    <t>연령대_20_유동인구_수</t>
+  </si>
+  <si>
+    <t>연령대_30_유동인구_수</t>
+  </si>
+  <si>
+    <t>연령대_40_유동인구_수</t>
+  </si>
+  <si>
+    <t>연령대_50_유동인구_수</t>
+  </si>
+  <si>
+    <t>연령대_60_이상_유동인구_수</t>
+  </si>
+  <si>
+    <t>시간대_00_06_유동인구_수</t>
+  </si>
+  <si>
+    <t>시간대_06_11_유동인구_수</t>
+  </si>
+  <si>
+    <t>시간대_11_14_유동인구_수</t>
+  </si>
+  <si>
+    <t>시간대_14_17_유동인구_수</t>
+  </si>
+  <si>
+    <t>시간대_17_21_유동인구_수</t>
+  </si>
+  <si>
+    <t>시간대_21_24_유동인구_수</t>
+  </si>
+  <si>
+    <t>월요일_유동인구_수</t>
+  </si>
+  <si>
+    <t>화요일_유동인구_수</t>
+  </si>
+  <si>
+    <t>수요일_유동인구_수</t>
+  </si>
+  <si>
+    <t>목요일_유동인구_수</t>
+  </si>
+  <si>
+    <t>금요일_유동인구_수</t>
+  </si>
+  <si>
+    <t>토요일_유동인구_수</t>
+  </si>
+  <si>
+    <t>일요일_유동인구_수</t>
+  </si>
+  <si>
+    <t>컬럼명 [행정동_코드] 이오나 [자치구_코드]의 오기로 확인됨.</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>컬럼명 [행정동_코드_명] 이오나 [자치구_코드_명]의 오기로 확인됨.</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>해당 분기(3개월) 총 매출 건수</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>해당 분기(3개월) 총 유동인구 수</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>* LL(다이나믹) : 해당 자치구 점포들의 영업기간이 서울시 평균 생존영업기간보다 낮고, 서울시 평균 폐업영업기간보다 낮은 상권
+* LH(상권확장) : 해당 자치구 점포들의 영업기간이 서울시 평균 생존영업기간보다 낮고, 서울시 평균 폐업영업기간보다 높은 상권
+* HL(상권축소) : 해당 자치구 점포들의 영업기간이 서울시 평균 생존영업기간보다 높고, 서울시 평균 폐업영업기간보다 낮은 상권
+* HH(정체) : 해당 자치구 점포들의 영업기간이 서울시 평균 생존영업기간보다 높고, 서울시 평균 폐업영업기간보다 높은 상권</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>6~24(관공서_수 ~ 버스_정거장_수)와 서울시에서 별도의 집객시설 리스트(동/식물원, 예식장 등)을 포함한 수</t>
     <phoneticPr fontId="1" type="noConversion"/>
   </si>
 </sst>
@@ -1080,7 +1570,7 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="12" x14ac:knownFonts="1">
+  <fonts count="13" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -1164,12 +1654,20 @@
     </font>
     <font>
       <sz val="11"/>
-      <color theme="1"/>
-      <name val="Calibri"/>
-      <family val="2"/>
-      <charset val="161"/>
+      <name val="맑은 고딕"/>
+      <family val="3"/>
+      <charset val="129"/>
+      <scheme val="minor"/>
     </font>
     <font>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="맑은 고딕"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
       <sz val="11"/>
       <name val="맑은 고딕"/>
       <family val="3"/>
@@ -1209,7 +1707,7 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="4">
+  <borders count="18">
     <border>
       <left/>
       <right/>
@@ -1258,16 +1756,207 @@
       </bottom>
       <diagonal/>
     </border>
+    <border>
+      <left/>
+      <right/>
+      <top/>
+      <bottom style="thin">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color indexed="64"/>
+      </left>
+      <right style="thin">
+        <color indexed="64"/>
+      </right>
+      <top style="thin">
+        <color indexed="64"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="medium">
+        <color indexed="64"/>
+      </left>
+      <right style="thin">
+        <color indexed="64"/>
+      </right>
+      <top style="medium">
+        <color indexed="64"/>
+      </top>
+      <bottom style="thin">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color indexed="64"/>
+      </left>
+      <right style="thin">
+        <color indexed="64"/>
+      </right>
+      <top style="medium">
+        <color indexed="64"/>
+      </top>
+      <bottom style="thin">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color indexed="64"/>
+      </left>
+      <right style="medium">
+        <color indexed="64"/>
+      </right>
+      <top style="medium">
+        <color indexed="64"/>
+      </top>
+      <bottom style="thin">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="medium">
+        <color indexed="64"/>
+      </left>
+      <right style="thin">
+        <color indexed="64"/>
+      </right>
+      <top style="thin">
+        <color indexed="64"/>
+      </top>
+      <bottom style="thin">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color indexed="64"/>
+      </left>
+      <right style="medium">
+        <color indexed="64"/>
+      </right>
+      <top style="thin">
+        <color indexed="64"/>
+      </top>
+      <bottom style="thin">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="medium">
+        <color indexed="64"/>
+      </left>
+      <right style="thin">
+        <color indexed="64"/>
+      </right>
+      <top style="thin">
+        <color indexed="64"/>
+      </top>
+      <bottom style="medium">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color indexed="64"/>
+      </left>
+      <right style="thin">
+        <color indexed="64"/>
+      </right>
+      <top style="thin">
+        <color indexed="64"/>
+      </top>
+      <bottom style="medium">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color indexed="64"/>
+      </left>
+      <right style="medium">
+        <color indexed="64"/>
+      </right>
+      <top style="thin">
+        <color indexed="64"/>
+      </top>
+      <bottom style="medium">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="thin">
+        <color indexed="64"/>
+      </right>
+      <top/>
+      <bottom style="thin">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="medium">
+        <color indexed="64"/>
+      </left>
+      <right style="thin">
+        <color indexed="64"/>
+      </right>
+      <top style="medium">
+        <color indexed="64"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="medium">
+        <color indexed="64"/>
+      </left>
+      <right style="thin">
+        <color indexed="64"/>
+      </right>
+      <top/>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="medium">
+        <color indexed="64"/>
+      </left>
+      <right style="thin">
+        <color indexed="64"/>
+      </right>
+      <top/>
+      <bottom style="medium">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
-  <cellStyleXfs count="2">
+  <cellStyleXfs count="3">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="45">
+  <cellXfs count="83">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0">
       <alignment vertical="center"/>
     </xf>
@@ -1376,6 +2065,12 @@
     <xf numFmtId="0" fontId="9" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="5" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="6" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
@@ -1388,24 +2083,133 @@
     <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="11" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="5" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
-    </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyBorder="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center"/>
+    <xf numFmtId="0" fontId="2" fillId="2" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="2" borderId="14" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="2" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="12" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="0" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="0" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="0" borderId="12" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="15" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="16" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="17" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="12" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="13" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="12" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="12" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="13" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="12" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="7" xfId="2" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="1" xfId="2" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="12" xfId="2" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
-  <cellStyles count="2">
+  <cellStyles count="3">
     <cellStyle name="표준" xfId="0" builtinId="0"/>
+    <cellStyle name="표준 2" xfId="2" xr:uid="{0495489C-6CC2-4726-A574-C696828E9354}"/>
     <cellStyle name="하이퍼링크" xfId="1" builtinId="8"/>
   </cellStyles>
   <dxfs count="0"/>
@@ -1427,14 +2231,14 @@
     <xdr:from>
       <xdr:col>0</xdr:col>
       <xdr:colOff>943831</xdr:colOff>
-      <xdr:row>11</xdr:row>
+      <xdr:row>10</xdr:row>
       <xdr:rowOff>174213</xdr:rowOff>
     </xdr:from>
     <xdr:to>
       <xdr:col>2</xdr:col>
       <xdr:colOff>915669</xdr:colOff>
-      <xdr:row>13</xdr:row>
-      <xdr:rowOff>1911887</xdr:rowOff>
+      <xdr:row>12</xdr:row>
+      <xdr:rowOff>1918238</xdr:rowOff>
     </xdr:to>
     <xdr:pic>
       <xdr:nvPicPr>
@@ -1474,6 +2278,22 @@
     <xdr:clientData/>
   </xdr:twoCellAnchor>
 </xdr:wsDr>
+</file>
+
+<file path=xl/externalLinks/externalLink1.xml><?xml version="1.0" encoding="utf-8"?>
+<externalLink xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:xxl21="http://schemas.microsoft.com/office/spreadsheetml/2021/extlinks2021" mc:Ignorable="x14 xxl21">
+  <externalBook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1">
+    <xxl21:alternateUrls>
+      <xxl21:absoluteUrl r:id="rId2"/>
+    </xxl21:alternateUrls>
+    <sheetNames>
+      <sheetName val="길단위인구_자치구"/>
+    </sheetNames>
+    <sheetDataSet>
+      <sheetData sheetId="0"/>
+    </sheetDataSet>
+  </externalBook>
+</externalLink>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -1895,20 +2715,20 @@
       <c r="D9" s="23"/>
     </row>
     <row r="10" spans="1:4" x14ac:dyDescent="0.45">
-      <c r="A10" s="36" t="s">
+      <c r="A10" s="38" t="s">
         <v>8</v>
       </c>
-      <c r="B10" s="37"/>
+      <c r="B10" s="39"/>
       <c r="C10" s="31">
         <v>46259.5</v>
       </c>
       <c r="D10" s="26"/>
     </row>
     <row r="11" spans="1:4" x14ac:dyDescent="0.45">
-      <c r="A11" s="36" t="s">
+      <c r="A11" s="38" t="s">
         <v>9</v>
       </c>
-      <c r="B11" s="37"/>
+      <c r="B11" s="39"/>
       <c r="C11" s="31">
         <v>46259.645833333336</v>
       </c>
@@ -2295,21 +3115,20 @@
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{41889BD0-A4A8-4188-AE8A-C708D84C89CC}">
-  <dimension ref="A1:C14"/>
+  <dimension ref="A1:C13"/>
   <sheetFormatPr defaultRowHeight="17" x14ac:dyDescent="0.45"/>
   <cols>
     <col min="1" max="1" width="28.25" customWidth="1"/>
     <col min="2" max="2" width="106.75" customWidth="1"/>
     <col min="3" max="3" width="41.9140625" customWidth="1"/>
-    <col min="4" max="16384" width="8.6640625" style="43"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:3" x14ac:dyDescent="0.45">
-      <c r="A1" s="38" t="s">
+      <c r="A1" s="40" t="s">
         <v>91</v>
       </c>
-      <c r="B1" s="38"/>
-      <c r="C1" s="38"/>
+      <c r="B1" s="40"/>
+      <c r="C1" s="40"/>
     </row>
     <row r="2" spans="1:3" ht="16.5" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A2" s="9" t="s">
@@ -2327,7 +3146,7 @@
         <v>88</v>
       </c>
       <c r="B3" s="34" t="s">
-        <v>99</v>
+        <v>98</v>
       </c>
       <c r="C3" s="2"/>
     </row>
@@ -2345,7 +3164,7 @@
         <v>95</v>
       </c>
       <c r="B5" s="34" t="s">
-        <v>101</v>
+        <v>100</v>
       </c>
       <c r="C5" s="2"/>
     </row>
@@ -2353,11 +3172,11 @@
       <c r="A6" s="3" t="s">
         <v>89</v>
       </c>
-      <c r="B6" s="40" t="s">
-        <v>100</v>
+      <c r="B6" s="36" t="s">
+        <v>99</v>
       </c>
       <c r="C6" s="34" t="s">
-        <v>104</v>
+        <v>102</v>
       </c>
     </row>
     <row r="7" spans="1:3" ht="282.5" customHeight="1" x14ac:dyDescent="0.45">
@@ -2365,57 +3184,48 @@
         <v>0</v>
       </c>
       <c r="B7" s="35" t="s">
-        <v>102</v>
+        <v>101</v>
       </c>
       <c r="C7" s="29" t="s">
         <v>103</v>
       </c>
     </row>
-    <row r="8" spans="1:3" ht="101.5" customHeight="1" x14ac:dyDescent="0.45">
+    <row r="8" spans="1:3" ht="138" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A8" s="3" t="s">
-        <v>105</v>
-      </c>
-      <c r="B8" s="35" t="s">
-        <v>106</v>
-      </c>
-      <c r="C8" s="29"/>
-    </row>
-    <row r="9" spans="1:3" ht="221" x14ac:dyDescent="0.45">
-      <c r="A9" s="3" t="s">
         <v>97</v>
       </c>
-      <c r="B9" s="41" t="s">
-        <v>98</v>
-      </c>
-      <c r="C9" s="2"/>
-    </row>
-    <row r="11" spans="1:3" x14ac:dyDescent="0.45">
-      <c r="A11" s="39" t="s">
+      <c r="B8" s="37" t="s">
+        <v>208</v>
+      </c>
+      <c r="C8" s="2"/>
+    </row>
+    <row r="10" spans="1:3" x14ac:dyDescent="0.45">
+      <c r="A10" s="41" t="s">
         <v>92</v>
       </c>
-      <c r="B11" s="39"/>
-      <c r="C11" s="39"/>
-    </row>
-    <row r="12" spans="1:3" s="44" customFormat="1" ht="162" customHeight="1" x14ac:dyDescent="0.45">
+      <c r="B10" s="41"/>
+      <c r="C10" s="41"/>
+    </row>
+    <row r="11" spans="1:3" ht="162" customHeight="1" x14ac:dyDescent="0.45">
+      <c r="A11" s="42"/>
+      <c r="B11" s="42"/>
+      <c r="C11" s="42"/>
+    </row>
+    <row r="12" spans="1:3" ht="162" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A12" s="42"/>
       <c r="B12" s="42"/>
       <c r="C12" s="42"/>
     </row>
-    <row r="13" spans="1:3" s="44" customFormat="1" ht="162" customHeight="1" x14ac:dyDescent="0.45">
+    <row r="13" spans="1:3" ht="162" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A13" s="42"/>
       <c r="B13" s="42"/>
       <c r="C13" s="42"/>
     </row>
-    <row r="14" spans="1:3" s="44" customFormat="1" ht="162" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="A14" s="42"/>
-      <c r="B14" s="42"/>
-      <c r="C14" s="42"/>
-    </row>
   </sheetData>
   <mergeCells count="3">
     <mergeCell ref="A1:C1"/>
-    <mergeCell ref="A11:C11"/>
-    <mergeCell ref="A12:C14"/>
+    <mergeCell ref="A10:C10"/>
+    <mergeCell ref="A11:C13"/>
   </mergeCells>
   <phoneticPr fontId="1" type="noConversion"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
@@ -2425,26 +3235,2921 @@
 
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{1402F3D2-E44E-49CC-8D75-9BA854A3E719}">
-  <dimension ref="A1:C1"/>
+  <dimension ref="A1:G165"/>
   <sheetFormatPr defaultRowHeight="17" x14ac:dyDescent="0.45"/>
   <cols>
-    <col min="1" max="1" width="25.9140625" customWidth="1"/>
-    <col min="2" max="2" width="63.83203125" customWidth="1"/>
-    <col min="3" max="3" width="16.25" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="23" customWidth="1"/>
+    <col min="3" max="3" width="6.33203125" customWidth="1"/>
+    <col min="4" max="4" width="25" customWidth="1"/>
+    <col min="5" max="5" width="15.6640625" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="7" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="113.4140625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3" x14ac:dyDescent="0.45">
-      <c r="A1" s="8" t="s">
+    <row r="1" spans="1:7" x14ac:dyDescent="0.45">
+      <c r="A1" s="43" t="s">
+        <v>104</v>
+      </c>
+      <c r="B1" s="43"/>
+      <c r="C1" s="43"/>
+      <c r="D1" s="43"/>
+      <c r="E1" s="43"/>
+      <c r="F1" s="43"/>
+      <c r="G1" s="47"/>
+    </row>
+    <row r="2" spans="1:7" ht="17.5" thickBot="1" x14ac:dyDescent="0.5">
+      <c r="A2" s="49" t="s">
+        <v>209</v>
+      </c>
+      <c r="B2" s="49" t="s">
+        <v>120</v>
+      </c>
+      <c r="C2" s="49" t="s">
+        <v>122</v>
+      </c>
+      <c r="D2" s="49" t="s">
+        <v>123</v>
+      </c>
+      <c r="E2" s="49" t="s">
+        <v>121</v>
+      </c>
+      <c r="F2" s="49" t="s">
+        <v>126</v>
+      </c>
+      <c r="G2" s="49" t="s">
+        <v>127</v>
+      </c>
+    </row>
+    <row r="3" spans="1:7" ht="34" x14ac:dyDescent="0.45">
+      <c r="A3" s="44">
+        <v>1</v>
+      </c>
+      <c r="B3" s="50" t="s">
+        <v>105</v>
+      </c>
+      <c r="C3" s="58">
+        <v>0</v>
+      </c>
+      <c r="D3" s="58" t="s">
+        <v>106</v>
+      </c>
+      <c r="E3" s="58">
+        <v>3250</v>
+      </c>
+      <c r="F3" s="58" t="s">
+        <v>107</v>
+      </c>
+      <c r="G3" s="59" t="s">
+        <v>128</v>
+      </c>
+    </row>
+    <row r="4" spans="1:7" x14ac:dyDescent="0.45">
+      <c r="A4" s="45"/>
+      <c r="B4" s="48"/>
+      <c r="C4" s="60">
+        <v>1</v>
+      </c>
+      <c r="D4" s="60" t="s">
+        <v>108</v>
+      </c>
+      <c r="E4" s="60">
+        <v>3250</v>
+      </c>
+      <c r="F4" s="60" t="s">
+        <v>107</v>
+      </c>
+      <c r="G4" s="61"/>
+    </row>
+    <row r="5" spans="1:7" x14ac:dyDescent="0.45">
+      <c r="A5" s="45"/>
+      <c r="B5" s="48"/>
+      <c r="C5" s="60">
+        <v>2</v>
+      </c>
+      <c r="D5" s="60" t="s">
+        <v>109</v>
+      </c>
+      <c r="E5" s="60">
+        <v>3250</v>
+      </c>
+      <c r="F5" s="60" t="s">
+        <v>110</v>
+      </c>
+      <c r="G5" s="61"/>
+    </row>
+    <row r="6" spans="1:7" ht="68" x14ac:dyDescent="0.45">
+      <c r="A6" s="45"/>
+      <c r="B6" s="48"/>
+      <c r="C6" s="60">
+        <v>3</v>
+      </c>
+      <c r="D6" s="60" t="s">
+        <v>111</v>
+      </c>
+      <c r="E6" s="60">
+        <v>3250</v>
+      </c>
+      <c r="F6" s="60" t="s">
+        <v>110</v>
+      </c>
+      <c r="G6" s="62" t="s">
+        <v>129</v>
+      </c>
+    </row>
+    <row r="7" spans="1:7" x14ac:dyDescent="0.45">
+      <c r="A7" s="45"/>
+      <c r="B7" s="48"/>
+      <c r="C7" s="60">
+        <v>4</v>
+      </c>
+      <c r="D7" s="60" t="s">
+        <v>112</v>
+      </c>
+      <c r="E7" s="60">
+        <v>3250</v>
+      </c>
+      <c r="F7" s="60" t="s">
+        <v>110</v>
+      </c>
+      <c r="G7" s="61"/>
+    </row>
+    <row r="8" spans="1:7" x14ac:dyDescent="0.45">
+      <c r="A8" s="45"/>
+      <c r="B8" s="48"/>
+      <c r="C8" s="60">
+        <v>5</v>
+      </c>
+      <c r="D8" s="60" t="s">
+        <v>113</v>
+      </c>
+      <c r="E8" s="60">
+        <v>3250</v>
+      </c>
+      <c r="F8" s="60" t="s">
+        <v>107</v>
+      </c>
+      <c r="G8" s="61" t="s">
+        <v>131</v>
+      </c>
+    </row>
+    <row r="9" spans="1:7" x14ac:dyDescent="0.45">
+      <c r="A9" s="45"/>
+      <c r="B9" s="48"/>
+      <c r="C9" s="60">
+        <v>6</v>
+      </c>
+      <c r="D9" s="60" t="s">
+        <v>114</v>
+      </c>
+      <c r="E9" s="60">
+        <v>3250</v>
+      </c>
+      <c r="F9" s="60" t="s">
+        <v>107</v>
+      </c>
+      <c r="G9" s="61"/>
+    </row>
+    <row r="10" spans="1:7" x14ac:dyDescent="0.45">
+      <c r="A10" s="45"/>
+      <c r="B10" s="48"/>
+      <c r="C10" s="60">
+        <v>7</v>
+      </c>
+      <c r="D10" s="60" t="s">
+        <v>130</v>
+      </c>
+      <c r="E10" s="60">
+        <v>3250</v>
+      </c>
+      <c r="F10" s="60" t="s">
+        <v>107</v>
+      </c>
+      <c r="G10" s="61"/>
+    </row>
+    <row r="11" spans="1:7" x14ac:dyDescent="0.45">
+      <c r="A11" s="45"/>
+      <c r="B11" s="48"/>
+      <c r="C11" s="60">
+        <v>8</v>
+      </c>
+      <c r="D11" s="60" t="s">
+        <v>116</v>
+      </c>
+      <c r="E11" s="60">
+        <v>3250</v>
+      </c>
+      <c r="F11" s="60" t="s">
+        <v>117</v>
+      </c>
+      <c r="G11" s="61"/>
+    </row>
+    <row r="12" spans="1:7" x14ac:dyDescent="0.45">
+      <c r="A12" s="45"/>
+      <c r="B12" s="48"/>
+      <c r="C12" s="60">
+        <v>9</v>
+      </c>
+      <c r="D12" s="60" t="s">
+        <v>118</v>
+      </c>
+      <c r="E12" s="60">
+        <v>3250</v>
+      </c>
+      <c r="F12" s="60" t="s">
+        <v>107</v>
+      </c>
+      <c r="G12" s="61"/>
+    </row>
+    <row r="13" spans="1:7" x14ac:dyDescent="0.45">
+      <c r="A13" s="45"/>
+      <c r="B13" s="48"/>
+      <c r="C13" s="60">
+        <v>10</v>
+      </c>
+      <c r="D13" s="60" t="s">
+        <v>119</v>
+      </c>
+      <c r="E13" s="60">
+        <v>3250</v>
+      </c>
+      <c r="F13" s="60" t="s">
+        <v>117</v>
+      </c>
+      <c r="G13" s="61"/>
+    </row>
+    <row r="14" spans="1:7" ht="17.5" thickBot="1" x14ac:dyDescent="0.5">
+      <c r="A14" s="46"/>
+      <c r="B14" s="51"/>
+      <c r="C14" s="63">
         <v>11</v>
       </c>
-      <c r="B1" s="9" t="s">
-        <v>76</v>
-      </c>
-      <c r="C1" s="9" t="s">
+      <c r="D14" s="63" t="s">
+        <v>125</v>
+      </c>
+      <c r="E14" s="63">
+        <v>3250</v>
+      </c>
+      <c r="F14" s="63" t="s">
+        <v>107</v>
+      </c>
+      <c r="G14" s="64"/>
+    </row>
+    <row r="15" spans="1:7" ht="34" x14ac:dyDescent="0.45">
+      <c r="A15" s="55">
+        <v>2</v>
+      </c>
+      <c r="B15" s="53" t="s">
+        <v>180</v>
+      </c>
+      <c r="C15" s="80">
+        <v>0</v>
+      </c>
+      <c r="D15" s="80" t="s">
+        <v>106</v>
+      </c>
+      <c r="E15" s="65">
+        <v>3250</v>
+      </c>
+      <c r="F15" s="66" t="s">
+        <v>107</v>
+      </c>
+      <c r="G15" s="67" t="s">
+        <v>128</v>
+      </c>
+    </row>
+    <row r="16" spans="1:7" x14ac:dyDescent="0.45">
+      <c r="A16" s="56"/>
+      <c r="B16" s="52"/>
+      <c r="C16" s="81">
+        <v>1</v>
+      </c>
+      <c r="D16" s="81" t="s">
+        <v>108</v>
+      </c>
+      <c r="E16" s="68">
+        <v>3250</v>
+      </c>
+      <c r="F16" s="69" t="s">
+        <v>107</v>
+      </c>
+      <c r="G16" s="70"/>
+    </row>
+    <row r="17" spans="1:7" x14ac:dyDescent="0.45">
+      <c r="A17" s="56"/>
+      <c r="B17" s="52"/>
+      <c r="C17" s="81">
+        <v>2</v>
+      </c>
+      <c r="D17" s="81" t="s">
+        <v>109</v>
+      </c>
+      <c r="E17" s="68">
+        <v>3250</v>
+      </c>
+      <c r="F17" s="69" t="s">
+        <v>110</v>
+      </c>
+      <c r="G17" s="70"/>
+    </row>
+    <row r="18" spans="1:7" ht="68" x14ac:dyDescent="0.45">
+      <c r="A18" s="56"/>
+      <c r="B18" s="52"/>
+      <c r="C18" s="81">
+        <v>3</v>
+      </c>
+      <c r="D18" s="81" t="s">
+        <v>111</v>
+      </c>
+      <c r="E18" s="68">
+        <v>3250</v>
+      </c>
+      <c r="F18" s="69" t="s">
+        <v>110</v>
+      </c>
+      <c r="G18" s="71" t="s">
+        <v>129</v>
+      </c>
+    </row>
+    <row r="19" spans="1:7" x14ac:dyDescent="0.45">
+      <c r="A19" s="56"/>
+      <c r="B19" s="52"/>
+      <c r="C19" s="81">
+        <v>4</v>
+      </c>
+      <c r="D19" s="81" t="s">
+        <v>112</v>
+      </c>
+      <c r="E19" s="68">
+        <v>3250</v>
+      </c>
+      <c r="F19" s="69" t="s">
+        <v>110</v>
+      </c>
+      <c r="G19" s="70"/>
+    </row>
+    <row r="20" spans="1:7" x14ac:dyDescent="0.45">
+      <c r="A20" s="56"/>
+      <c r="B20" s="52"/>
+      <c r="C20" s="81">
+        <v>5</v>
+      </c>
+      <c r="D20" s="81" t="s">
+        <v>132</v>
+      </c>
+      <c r="E20" s="68">
+        <v>3250</v>
+      </c>
+      <c r="F20" s="69" t="s">
+        <v>107</v>
+      </c>
+      <c r="G20" s="70" t="s">
+        <v>181</v>
+      </c>
+    </row>
+    <row r="21" spans="1:7" x14ac:dyDescent="0.45">
+      <c r="A21" s="56"/>
+      <c r="B21" s="52"/>
+      <c r="C21" s="81">
+        <v>6</v>
+      </c>
+      <c r="D21" s="81" t="s">
+        <v>133</v>
+      </c>
+      <c r="E21" s="68">
+        <v>3250</v>
+      </c>
+      <c r="F21" s="69" t="s">
+        <v>107</v>
+      </c>
+      <c r="G21" s="70" t="s">
+        <v>264</v>
+      </c>
+    </row>
+    <row r="22" spans="1:7" x14ac:dyDescent="0.45">
+      <c r="A22" s="56"/>
+      <c r="B22" s="52"/>
+      <c r="C22" s="81">
+        <v>7</v>
+      </c>
+      <c r="D22" s="81" t="s">
+        <v>134</v>
+      </c>
+      <c r="E22" s="68">
+        <v>3250</v>
+      </c>
+      <c r="F22" s="69" t="s">
+        <v>107</v>
+      </c>
+      <c r="G22" s="70"/>
+    </row>
+    <row r="23" spans="1:7" x14ac:dyDescent="0.45">
+      <c r="A23" s="56"/>
+      <c r="B23" s="52"/>
+      <c r="C23" s="81">
+        <v>8</v>
+      </c>
+      <c r="D23" s="81" t="s">
+        <v>135</v>
+      </c>
+      <c r="E23" s="68">
+        <v>3250</v>
+      </c>
+      <c r="F23" s="69" t="s">
+        <v>107</v>
+      </c>
+      <c r="G23" s="70"/>
+    </row>
+    <row r="24" spans="1:7" x14ac:dyDescent="0.45">
+      <c r="A24" s="56"/>
+      <c r="B24" s="52"/>
+      <c r="C24" s="81">
+        <v>9</v>
+      </c>
+      <c r="D24" s="81" t="s">
+        <v>136</v>
+      </c>
+      <c r="E24" s="68">
+        <v>3250</v>
+      </c>
+      <c r="F24" s="69" t="s">
+        <v>107</v>
+      </c>
+      <c r="G24" s="70"/>
+    </row>
+    <row r="25" spans="1:7" x14ac:dyDescent="0.45">
+      <c r="A25" s="56"/>
+      <c r="B25" s="52"/>
+      <c r="C25" s="81">
+        <v>10</v>
+      </c>
+      <c r="D25" s="81" t="s">
+        <v>137</v>
+      </c>
+      <c r="E25" s="68">
+        <v>3250</v>
+      </c>
+      <c r="F25" s="69" t="s">
+        <v>107</v>
+      </c>
+      <c r="G25" s="70"/>
+    </row>
+    <row r="26" spans="1:7" x14ac:dyDescent="0.45">
+      <c r="A26" s="56"/>
+      <c r="B26" s="52"/>
+      <c r="C26" s="81">
+        <v>11</v>
+      </c>
+      <c r="D26" s="81" t="s">
+        <v>138</v>
+      </c>
+      <c r="E26" s="68">
+        <v>3250</v>
+      </c>
+      <c r="F26" s="69" t="s">
+        <v>107</v>
+      </c>
+      <c r="G26" s="70"/>
+    </row>
+    <row r="27" spans="1:7" x14ac:dyDescent="0.45">
+      <c r="A27" s="56"/>
+      <c r="B27" s="52"/>
+      <c r="C27" s="81">
+        <v>12</v>
+      </c>
+      <c r="D27" s="81" t="s">
+        <v>139</v>
+      </c>
+      <c r="E27" s="68">
+        <v>3250</v>
+      </c>
+      <c r="F27" s="69" t="s">
+        <v>107</v>
+      </c>
+      <c r="G27" s="70"/>
+    </row>
+    <row r="28" spans="1:7" x14ac:dyDescent="0.45">
+      <c r="A28" s="56"/>
+      <c r="B28" s="52"/>
+      <c r="C28" s="81">
+        <v>13</v>
+      </c>
+      <c r="D28" s="81" t="s">
+        <v>140</v>
+      </c>
+      <c r="E28" s="68">
+        <v>3250</v>
+      </c>
+      <c r="F28" s="69" t="s">
+        <v>107</v>
+      </c>
+      <c r="G28" s="70"/>
+    </row>
+    <row r="29" spans="1:7" x14ac:dyDescent="0.45">
+      <c r="A29" s="56"/>
+      <c r="B29" s="52"/>
+      <c r="C29" s="81">
+        <v>14</v>
+      </c>
+      <c r="D29" s="81" t="s">
+        <v>141</v>
+      </c>
+      <c r="E29" s="68">
+        <v>3250</v>
+      </c>
+      <c r="F29" s="69" t="s">
+        <v>107</v>
+      </c>
+      <c r="G29" s="70"/>
+    </row>
+    <row r="30" spans="1:7" x14ac:dyDescent="0.45">
+      <c r="A30" s="56"/>
+      <c r="B30" s="52"/>
+      <c r="C30" s="81">
+        <v>15</v>
+      </c>
+      <c r="D30" s="81" t="s">
+        <v>142</v>
+      </c>
+      <c r="E30" s="68">
+        <v>3250</v>
+      </c>
+      <c r="F30" s="69" t="s">
+        <v>107</v>
+      </c>
+      <c r="G30" s="70"/>
+    </row>
+    <row r="31" spans="1:7" x14ac:dyDescent="0.45">
+      <c r="A31" s="56"/>
+      <c r="B31" s="52"/>
+      <c r="C31" s="81">
+        <v>16</v>
+      </c>
+      <c r="D31" s="81" t="s">
+        <v>143</v>
+      </c>
+      <c r="E31" s="68">
+        <v>3250</v>
+      </c>
+      <c r="F31" s="69" t="s">
+        <v>107</v>
+      </c>
+      <c r="G31" s="70"/>
+    </row>
+    <row r="32" spans="1:7" x14ac:dyDescent="0.45">
+      <c r="A32" s="56"/>
+      <c r="B32" s="52"/>
+      <c r="C32" s="81">
+        <v>17</v>
+      </c>
+      <c r="D32" s="81" t="s">
+        <v>144</v>
+      </c>
+      <c r="E32" s="68">
+        <v>3250</v>
+      </c>
+      <c r="F32" s="69" t="s">
+        <v>107</v>
+      </c>
+      <c r="G32" s="70"/>
+    </row>
+    <row r="33" spans="1:7" x14ac:dyDescent="0.45">
+      <c r="A33" s="56"/>
+      <c r="B33" s="52"/>
+      <c r="C33" s="81">
+        <v>18</v>
+      </c>
+      <c r="D33" s="81" t="s">
+        <v>145</v>
+      </c>
+      <c r="E33" s="68">
+        <v>3250</v>
+      </c>
+      <c r="F33" s="69" t="s">
+        <v>107</v>
+      </c>
+      <c r="G33" s="70" t="s">
+        <v>207</v>
+      </c>
+    </row>
+    <row r="34" spans="1:7" x14ac:dyDescent="0.45">
+      <c r="A34" s="56"/>
+      <c r="B34" s="52"/>
+      <c r="C34" s="81">
+        <v>19</v>
+      </c>
+      <c r="D34" s="81" t="s">
+        <v>146</v>
+      </c>
+      <c r="E34" s="68">
+        <v>3250</v>
+      </c>
+      <c r="F34" s="69" t="s">
+        <v>107</v>
+      </c>
+      <c r="G34" s="70"/>
+    </row>
+    <row r="35" spans="1:7" x14ac:dyDescent="0.45">
+      <c r="A35" s="56"/>
+      <c r="B35" s="52"/>
+      <c r="C35" s="81">
+        <v>20</v>
+      </c>
+      <c r="D35" s="81" t="s">
+        <v>147</v>
+      </c>
+      <c r="E35" s="68">
+        <v>3250</v>
+      </c>
+      <c r="F35" s="69" t="s">
+        <v>107</v>
+      </c>
+      <c r="G35" s="70"/>
+    </row>
+    <row r="36" spans="1:7" x14ac:dyDescent="0.45">
+      <c r="A36" s="56"/>
+      <c r="B36" s="52"/>
+      <c r="C36" s="81">
+        <v>21</v>
+      </c>
+      <c r="D36" s="81" t="s">
+        <v>148</v>
+      </c>
+      <c r="E36" s="68">
+        <v>3250</v>
+      </c>
+      <c r="F36" s="69" t="s">
+        <v>107</v>
+      </c>
+      <c r="G36" s="70"/>
+    </row>
+    <row r="37" spans="1:7" x14ac:dyDescent="0.45">
+      <c r="A37" s="56"/>
+      <c r="B37" s="52"/>
+      <c r="C37" s="81">
+        <v>22</v>
+      </c>
+      <c r="D37" s="81" t="s">
+        <v>149</v>
+      </c>
+      <c r="E37" s="68">
+        <v>3250</v>
+      </c>
+      <c r="F37" s="69" t="s">
+        <v>107</v>
+      </c>
+      <c r="G37" s="70"/>
+    </row>
+    <row r="38" spans="1:7" x14ac:dyDescent="0.45">
+      <c r="A38" s="56"/>
+      <c r="B38" s="52"/>
+      <c r="C38" s="81">
+        <v>23</v>
+      </c>
+      <c r="D38" s="81" t="s">
+        <v>150</v>
+      </c>
+      <c r="E38" s="68">
+        <v>3250</v>
+      </c>
+      <c r="F38" s="69" t="s">
+        <v>107</v>
+      </c>
+      <c r="G38" s="70"/>
+    </row>
+    <row r="39" spans="1:7" x14ac:dyDescent="0.45">
+      <c r="A39" s="56"/>
+      <c r="B39" s="52"/>
+      <c r="C39" s="81">
+        <v>24</v>
+      </c>
+      <c r="D39" s="81" t="s">
+        <v>151</v>
+      </c>
+      <c r="E39" s="68">
+        <v>3250</v>
+      </c>
+      <c r="F39" s="69" t="s">
+        <v>107</v>
+      </c>
+      <c r="G39" s="70"/>
+    </row>
+    <row r="40" spans="1:7" x14ac:dyDescent="0.45">
+      <c r="A40" s="56"/>
+      <c r="B40" s="52"/>
+      <c r="C40" s="81">
+        <v>25</v>
+      </c>
+      <c r="D40" s="81" t="s">
+        <v>152</v>
+      </c>
+      <c r="E40" s="68">
+        <v>3250</v>
+      </c>
+      <c r="F40" s="69" t="s">
+        <v>107</v>
+      </c>
+      <c r="G40" s="70"/>
+    </row>
+    <row r="41" spans="1:7" x14ac:dyDescent="0.45">
+      <c r="A41" s="56"/>
+      <c r="B41" s="52"/>
+      <c r="C41" s="81">
+        <v>26</v>
+      </c>
+      <c r="D41" s="81" t="s">
+        <v>153</v>
+      </c>
+      <c r="E41" s="68">
+        <v>3250</v>
+      </c>
+      <c r="F41" s="69" t="s">
+        <v>107</v>
+      </c>
+      <c r="G41" s="70"/>
+    </row>
+    <row r="42" spans="1:7" x14ac:dyDescent="0.45">
+      <c r="A42" s="56"/>
+      <c r="B42" s="52"/>
+      <c r="C42" s="81">
+        <v>27</v>
+      </c>
+      <c r="D42" s="81" t="s">
+        <v>154</v>
+      </c>
+      <c r="E42" s="68">
+        <v>3250</v>
+      </c>
+      <c r="F42" s="69" t="s">
+        <v>107</v>
+      </c>
+      <c r="G42" s="70"/>
+    </row>
+    <row r="43" spans="1:7" x14ac:dyDescent="0.45">
+      <c r="A43" s="56"/>
+      <c r="B43" s="52"/>
+      <c r="C43" s="81">
+        <v>28</v>
+      </c>
+      <c r="D43" s="81" t="s">
+        <v>155</v>
+      </c>
+      <c r="E43" s="68">
+        <v>3250</v>
+      </c>
+      <c r="F43" s="69" t="s">
+        <v>107</v>
+      </c>
+      <c r="G43" s="70"/>
+    </row>
+    <row r="44" spans="1:7" x14ac:dyDescent="0.45">
+      <c r="A44" s="56"/>
+      <c r="B44" s="52"/>
+      <c r="C44" s="81">
+        <v>29</v>
+      </c>
+      <c r="D44" s="81" t="s">
+        <v>156</v>
+      </c>
+      <c r="E44" s="68">
+        <v>3250</v>
+      </c>
+      <c r="F44" s="69" t="s">
+        <v>107</v>
+      </c>
+      <c r="G44" s="70"/>
+    </row>
+    <row r="45" spans="1:7" x14ac:dyDescent="0.45">
+      <c r="A45" s="56"/>
+      <c r="B45" s="52"/>
+      <c r="C45" s="81">
+        <v>30</v>
+      </c>
+      <c r="D45" s="81" t="s">
+        <v>157</v>
+      </c>
+      <c r="E45" s="68">
+        <v>3250</v>
+      </c>
+      <c r="F45" s="69" t="s">
+        <v>107</v>
+      </c>
+      <c r="G45" s="70"/>
+    </row>
+    <row r="46" spans="1:7" x14ac:dyDescent="0.45">
+      <c r="A46" s="56"/>
+      <c r="B46" s="52"/>
+      <c r="C46" s="81">
+        <v>31</v>
+      </c>
+      <c r="D46" s="81" t="s">
+        <v>158</v>
+      </c>
+      <c r="E46" s="68">
+        <v>3250</v>
+      </c>
+      <c r="F46" s="69" t="s">
+        <v>107</v>
+      </c>
+      <c r="G46" s="70"/>
+    </row>
+    <row r="47" spans="1:7" x14ac:dyDescent="0.45">
+      <c r="A47" s="56"/>
+      <c r="B47" s="52"/>
+      <c r="C47" s="81">
+        <v>32</v>
+      </c>
+      <c r="D47" s="81" t="s">
+        <v>159</v>
+      </c>
+      <c r="E47" s="68">
+        <v>3250</v>
+      </c>
+      <c r="F47" s="69" t="s">
+        <v>107</v>
+      </c>
+      <c r="G47" s="70"/>
+    </row>
+    <row r="48" spans="1:7" x14ac:dyDescent="0.45">
+      <c r="A48" s="56"/>
+      <c r="B48" s="52"/>
+      <c r="C48" s="81">
+        <v>33</v>
+      </c>
+      <c r="D48" s="81" t="s">
+        <v>160</v>
+      </c>
+      <c r="E48" s="68">
+        <v>3250</v>
+      </c>
+      <c r="F48" s="69" t="s">
+        <v>107</v>
+      </c>
+      <c r="G48" s="70"/>
+    </row>
+    <row r="49" spans="1:7" x14ac:dyDescent="0.45">
+      <c r="A49" s="56"/>
+      <c r="B49" s="52"/>
+      <c r="C49" s="81">
+        <v>34</v>
+      </c>
+      <c r="D49" s="81" t="s">
+        <v>161</v>
+      </c>
+      <c r="E49" s="68">
+        <v>3250</v>
+      </c>
+      <c r="F49" s="69" t="s">
+        <v>107</v>
+      </c>
+      <c r="G49" s="70"/>
+    </row>
+    <row r="50" spans="1:7" x14ac:dyDescent="0.45">
+      <c r="A50" s="56"/>
+      <c r="B50" s="52"/>
+      <c r="C50" s="81">
+        <v>35</v>
+      </c>
+      <c r="D50" s="81" t="s">
+        <v>162</v>
+      </c>
+      <c r="E50" s="68">
+        <v>3250</v>
+      </c>
+      <c r="F50" s="69" t="s">
+        <v>107</v>
+      </c>
+      <c r="G50" s="70"/>
+    </row>
+    <row r="51" spans="1:7" x14ac:dyDescent="0.45">
+      <c r="A51" s="56"/>
+      <c r="B51" s="52"/>
+      <c r="C51" s="81">
+        <v>36</v>
+      </c>
+      <c r="D51" s="81" t="s">
+        <v>163</v>
+      </c>
+      <c r="E51" s="68">
+        <v>3250</v>
+      </c>
+      <c r="F51" s="69" t="s">
+        <v>107</v>
+      </c>
+      <c r="G51" s="70"/>
+    </row>
+    <row r="52" spans="1:7" x14ac:dyDescent="0.45">
+      <c r="A52" s="56"/>
+      <c r="B52" s="52"/>
+      <c r="C52" s="81">
+        <v>37</v>
+      </c>
+      <c r="D52" s="81" t="s">
+        <v>164</v>
+      </c>
+      <c r="E52" s="68">
+        <v>3250</v>
+      </c>
+      <c r="F52" s="69" t="s">
+        <v>107</v>
+      </c>
+      <c r="G52" s="70"/>
+    </row>
+    <row r="53" spans="1:7" x14ac:dyDescent="0.45">
+      <c r="A53" s="56"/>
+      <c r="B53" s="52"/>
+      <c r="C53" s="81">
+        <v>38</v>
+      </c>
+      <c r="D53" s="81" t="s">
+        <v>165</v>
+      </c>
+      <c r="E53" s="68">
+        <v>3250</v>
+      </c>
+      <c r="F53" s="69" t="s">
+        <v>107</v>
+      </c>
+      <c r="G53" s="70"/>
+    </row>
+    <row r="54" spans="1:7" x14ac:dyDescent="0.45">
+      <c r="A54" s="56"/>
+      <c r="B54" s="52"/>
+      <c r="C54" s="81">
+        <v>39</v>
+      </c>
+      <c r="D54" s="81" t="s">
+        <v>166</v>
+      </c>
+      <c r="E54" s="68">
+        <v>3250</v>
+      </c>
+      <c r="F54" s="69" t="s">
+        <v>107</v>
+      </c>
+      <c r="G54" s="70"/>
+    </row>
+    <row r="55" spans="1:7" x14ac:dyDescent="0.45">
+      <c r="A55" s="56"/>
+      <c r="B55" s="52"/>
+      <c r="C55" s="81">
+        <v>40</v>
+      </c>
+      <c r="D55" s="81" t="s">
+        <v>167</v>
+      </c>
+      <c r="E55" s="68">
+        <v>3250</v>
+      </c>
+      <c r="F55" s="69" t="s">
+        <v>107</v>
+      </c>
+      <c r="G55" s="70"/>
+    </row>
+    <row r="56" spans="1:7" x14ac:dyDescent="0.45">
+      <c r="A56" s="56"/>
+      <c r="B56" s="52"/>
+      <c r="C56" s="81">
+        <v>41</v>
+      </c>
+      <c r="D56" s="81" t="s">
+        <v>168</v>
+      </c>
+      <c r="E56" s="68">
+        <v>3250</v>
+      </c>
+      <c r="F56" s="69" t="s">
+        <v>107</v>
+      </c>
+      <c r="G56" s="70"/>
+    </row>
+    <row r="57" spans="1:7" x14ac:dyDescent="0.45">
+      <c r="A57" s="56"/>
+      <c r="B57" s="52"/>
+      <c r="C57" s="81">
+        <v>42</v>
+      </c>
+      <c r="D57" s="81" t="s">
+        <v>169</v>
+      </c>
+      <c r="E57" s="68">
+        <v>3250</v>
+      </c>
+      <c r="F57" s="69" t="s">
+        <v>107</v>
+      </c>
+      <c r="G57" s="70"/>
+    </row>
+    <row r="58" spans="1:7" x14ac:dyDescent="0.45">
+      <c r="A58" s="56"/>
+      <c r="B58" s="52"/>
+      <c r="C58" s="81">
+        <v>43</v>
+      </c>
+      <c r="D58" s="81" t="s">
+        <v>170</v>
+      </c>
+      <c r="E58" s="68">
+        <v>3250</v>
+      </c>
+      <c r="F58" s="69" t="s">
+        <v>107</v>
+      </c>
+      <c r="G58" s="70"/>
+    </row>
+    <row r="59" spans="1:7" x14ac:dyDescent="0.45">
+      <c r="A59" s="56"/>
+      <c r="B59" s="52"/>
+      <c r="C59" s="81">
+        <v>44</v>
+      </c>
+      <c r="D59" s="81" t="s">
+        <v>171</v>
+      </c>
+      <c r="E59" s="68">
+        <v>3250</v>
+      </c>
+      <c r="F59" s="69" t="s">
+        <v>107</v>
+      </c>
+      <c r="G59" s="70"/>
+    </row>
+    <row r="60" spans="1:7" x14ac:dyDescent="0.45">
+      <c r="A60" s="56"/>
+      <c r="B60" s="52"/>
+      <c r="C60" s="81">
+        <v>45</v>
+      </c>
+      <c r="D60" s="81" t="s">
+        <v>172</v>
+      </c>
+      <c r="E60" s="68">
+        <v>3250</v>
+      </c>
+      <c r="F60" s="69" t="s">
+        <v>107</v>
+      </c>
+      <c r="G60" s="70"/>
+    </row>
+    <row r="61" spans="1:7" x14ac:dyDescent="0.45">
+      <c r="A61" s="56"/>
+      <c r="B61" s="52"/>
+      <c r="C61" s="81">
+        <v>46</v>
+      </c>
+      <c r="D61" s="81" t="s">
+        <v>173</v>
+      </c>
+      <c r="E61" s="68">
+        <v>3250</v>
+      </c>
+      <c r="F61" s="69" t="s">
+        <v>107</v>
+      </c>
+      <c r="G61" s="70"/>
+    </row>
+    <row r="62" spans="1:7" x14ac:dyDescent="0.45">
+      <c r="A62" s="56"/>
+      <c r="B62" s="52"/>
+      <c r="C62" s="81">
+        <v>47</v>
+      </c>
+      <c r="D62" s="81" t="s">
+        <v>174</v>
+      </c>
+      <c r="E62" s="68">
+        <v>3250</v>
+      </c>
+      <c r="F62" s="69" t="s">
+        <v>107</v>
+      </c>
+      <c r="G62" s="70"/>
+    </row>
+    <row r="63" spans="1:7" x14ac:dyDescent="0.45">
+      <c r="A63" s="56"/>
+      <c r="B63" s="52"/>
+      <c r="C63" s="81">
         <v>48</v>
       </c>
+      <c r="D63" s="81" t="s">
+        <v>175</v>
+      </c>
+      <c r="E63" s="68">
+        <v>3250</v>
+      </c>
+      <c r="F63" s="69" t="s">
+        <v>107</v>
+      </c>
+      <c r="G63" s="70"/>
+    </row>
+    <row r="64" spans="1:7" x14ac:dyDescent="0.45">
+      <c r="A64" s="56"/>
+      <c r="B64" s="52"/>
+      <c r="C64" s="81">
+        <v>49</v>
+      </c>
+      <c r="D64" s="81" t="s">
+        <v>176</v>
+      </c>
+      <c r="E64" s="68">
+        <v>3250</v>
+      </c>
+      <c r="F64" s="69" t="s">
+        <v>107</v>
+      </c>
+      <c r="G64" s="70"/>
+    </row>
+    <row r="65" spans="1:7" x14ac:dyDescent="0.45">
+      <c r="A65" s="56"/>
+      <c r="B65" s="52"/>
+      <c r="C65" s="81">
+        <v>50</v>
+      </c>
+      <c r="D65" s="81" t="s">
+        <v>177</v>
+      </c>
+      <c r="E65" s="68">
+        <v>3250</v>
+      </c>
+      <c r="F65" s="69" t="s">
+        <v>107</v>
+      </c>
+      <c r="G65" s="70"/>
+    </row>
+    <row r="66" spans="1:7" x14ac:dyDescent="0.45">
+      <c r="A66" s="56"/>
+      <c r="B66" s="52"/>
+      <c r="C66" s="81">
+        <v>51</v>
+      </c>
+      <c r="D66" s="81" t="s">
+        <v>178</v>
+      </c>
+      <c r="E66" s="68">
+        <v>3250</v>
+      </c>
+      <c r="F66" s="69" t="s">
+        <v>107</v>
+      </c>
+      <c r="G66" s="70"/>
+    </row>
+    <row r="67" spans="1:7" ht="17.5" thickBot="1" x14ac:dyDescent="0.5">
+      <c r="A67" s="57"/>
+      <c r="B67" s="54"/>
+      <c r="C67" s="82">
+        <v>52</v>
+      </c>
+      <c r="D67" s="82" t="s">
+        <v>179</v>
+      </c>
+      <c r="E67" s="72">
+        <v>3250</v>
+      </c>
+      <c r="F67" s="73" t="s">
+        <v>107</v>
+      </c>
+      <c r="G67" s="74"/>
+    </row>
+    <row r="68" spans="1:7" ht="34" x14ac:dyDescent="0.45">
+      <c r="A68" s="44">
+        <v>3</v>
+      </c>
+      <c r="B68" s="50" t="s">
+        <v>226</v>
+      </c>
+      <c r="C68" s="58">
+        <v>0</v>
+      </c>
+      <c r="D68" s="58" t="s">
+        <v>106</v>
+      </c>
+      <c r="E68" s="58">
+        <v>325</v>
+      </c>
+      <c r="F68" s="58" t="s">
+        <v>107</v>
+      </c>
+      <c r="G68" s="59" t="s">
+        <v>227</v>
+      </c>
+    </row>
+    <row r="69" spans="1:7" x14ac:dyDescent="0.45">
+      <c r="A69" s="45"/>
+      <c r="B69" s="48"/>
+      <c r="C69" s="60">
+        <v>1</v>
+      </c>
+      <c r="D69" s="60" t="s">
+        <v>213</v>
+      </c>
+      <c r="E69" s="60">
+        <v>325</v>
+      </c>
+      <c r="F69" s="60" t="s">
+        <v>107</v>
+      </c>
+      <c r="G69" s="61" t="s">
+        <v>262</v>
+      </c>
+    </row>
+    <row r="70" spans="1:7" x14ac:dyDescent="0.45">
+      <c r="A70" s="45"/>
+      <c r="B70" s="48"/>
+      <c r="C70" s="60">
+        <v>2</v>
+      </c>
+      <c r="D70" s="60" t="s">
+        <v>214</v>
+      </c>
+      <c r="E70" s="60">
+        <v>325</v>
+      </c>
+      <c r="F70" s="60" t="s">
+        <v>110</v>
+      </c>
+      <c r="G70" s="61" t="s">
+        <v>263</v>
+      </c>
+    </row>
+    <row r="71" spans="1:7" x14ac:dyDescent="0.45">
+      <c r="A71" s="45"/>
+      <c r="B71" s="48"/>
+      <c r="C71" s="60">
+        <v>3</v>
+      </c>
+      <c r="D71" s="60" t="s">
+        <v>215</v>
+      </c>
+      <c r="E71" s="60">
+        <v>325</v>
+      </c>
+      <c r="F71" s="60" t="s">
+        <v>107</v>
+      </c>
+      <c r="G71" s="70" t="s">
+        <v>181</v>
+      </c>
+    </row>
+    <row r="72" spans="1:7" x14ac:dyDescent="0.45">
+      <c r="A72" s="45"/>
+      <c r="B72" s="48"/>
+      <c r="C72" s="60">
+        <v>4</v>
+      </c>
+      <c r="D72" s="60" t="s">
+        <v>216</v>
+      </c>
+      <c r="E72" s="60">
+        <v>325</v>
+      </c>
+      <c r="F72" s="60" t="s">
+        <v>107</v>
+      </c>
+      <c r="G72" s="61"/>
+    </row>
+    <row r="73" spans="1:7" x14ac:dyDescent="0.45">
+      <c r="A73" s="45"/>
+      <c r="B73" s="48"/>
+      <c r="C73" s="60">
+        <v>5</v>
+      </c>
+      <c r="D73" s="60" t="s">
+        <v>217</v>
+      </c>
+      <c r="E73" s="60">
+        <v>325</v>
+      </c>
+      <c r="F73" s="60" t="s">
+        <v>107</v>
+      </c>
+      <c r="G73" s="61"/>
+    </row>
+    <row r="74" spans="1:7" x14ac:dyDescent="0.45">
+      <c r="A74" s="45"/>
+      <c r="B74" s="48"/>
+      <c r="C74" s="60">
+        <v>6</v>
+      </c>
+      <c r="D74" s="60" t="s">
+        <v>218</v>
+      </c>
+      <c r="E74" s="60">
+        <v>325</v>
+      </c>
+      <c r="F74" s="60" t="s">
+        <v>107</v>
+      </c>
+      <c r="G74" s="61"/>
+    </row>
+    <row r="75" spans="1:7" x14ac:dyDescent="0.45">
+      <c r="A75" s="45"/>
+      <c r="B75" s="48"/>
+      <c r="C75" s="60">
+        <v>7</v>
+      </c>
+      <c r="D75" s="60" t="s">
+        <v>219</v>
+      </c>
+      <c r="E75" s="60">
+        <v>325</v>
+      </c>
+      <c r="F75" s="60" t="s">
+        <v>107</v>
+      </c>
+      <c r="G75" s="61"/>
+    </row>
+    <row r="76" spans="1:7" x14ac:dyDescent="0.45">
+      <c r="A76" s="45"/>
+      <c r="B76" s="48"/>
+      <c r="C76" s="60">
+        <v>8</v>
+      </c>
+      <c r="D76" s="60" t="s">
+        <v>220</v>
+      </c>
+      <c r="E76" s="60">
+        <v>325</v>
+      </c>
+      <c r="F76" s="60" t="s">
+        <v>107</v>
+      </c>
+      <c r="G76" s="61"/>
+    </row>
+    <row r="77" spans="1:7" x14ac:dyDescent="0.45">
+      <c r="A77" s="45"/>
+      <c r="B77" s="48"/>
+      <c r="C77" s="60">
+        <v>9</v>
+      </c>
+      <c r="D77" s="60" t="s">
+        <v>221</v>
+      </c>
+      <c r="E77" s="60">
+        <v>325</v>
+      </c>
+      <c r="F77" s="60" t="s">
+        <v>107</v>
+      </c>
+      <c r="G77" s="61"/>
+    </row>
+    <row r="78" spans="1:7" x14ac:dyDescent="0.45">
+      <c r="A78" s="45"/>
+      <c r="B78" s="48"/>
+      <c r="C78" s="60">
+        <v>10</v>
+      </c>
+      <c r="D78" s="60" t="s">
+        <v>222</v>
+      </c>
+      <c r="E78" s="60">
+        <v>325</v>
+      </c>
+      <c r="F78" s="60" t="s">
+        <v>107</v>
+      </c>
+      <c r="G78" s="61"/>
+    </row>
+    <row r="79" spans="1:7" x14ac:dyDescent="0.45">
+      <c r="A79" s="45"/>
+      <c r="B79" s="48"/>
+      <c r="C79" s="60">
+        <v>11</v>
+      </c>
+      <c r="D79" s="60" t="s">
+        <v>223</v>
+      </c>
+      <c r="E79" s="60">
+        <v>325</v>
+      </c>
+      <c r="F79" s="60" t="s">
+        <v>107</v>
+      </c>
+      <c r="G79" s="61"/>
+    </row>
+    <row r="80" spans="1:7" x14ac:dyDescent="0.45">
+      <c r="A80" s="45"/>
+      <c r="B80" s="48"/>
+      <c r="C80" s="60">
+        <v>12</v>
+      </c>
+      <c r="D80" s="60" t="s">
+        <v>224</v>
+      </c>
+      <c r="E80" s="60">
+        <v>325</v>
+      </c>
+      <c r="F80" s="60" t="s">
+        <v>107</v>
+      </c>
+      <c r="G80" s="61"/>
+    </row>
+    <row r="81" spans="1:7" ht="17.5" thickBot="1" x14ac:dyDescent="0.5">
+      <c r="A81" s="46"/>
+      <c r="B81" s="51"/>
+      <c r="C81" s="63">
+        <v>13</v>
+      </c>
+      <c r="D81" s="63" t="s">
+        <v>225</v>
+      </c>
+      <c r="E81" s="63">
+        <v>325</v>
+      </c>
+      <c r="F81" s="63" t="s">
+        <v>107</v>
+      </c>
+      <c r="G81" s="64"/>
+    </row>
+    <row r="82" spans="1:7" ht="16.5" customHeight="1" x14ac:dyDescent="0.45">
+      <c r="A82" s="44">
+        <v>4</v>
+      </c>
+      <c r="B82" s="75" t="s">
+        <v>229</v>
+      </c>
+      <c r="C82" s="58">
+        <v>0</v>
+      </c>
+      <c r="D82" s="58" t="s">
+        <v>182</v>
+      </c>
+      <c r="E82" s="58">
+        <v>1650</v>
+      </c>
+      <c r="F82" s="76" t="s">
+        <v>110</v>
+      </c>
+      <c r="G82" s="77"/>
+    </row>
+    <row r="83" spans="1:7" x14ac:dyDescent="0.45">
+      <c r="A83" s="45"/>
+      <c r="B83" s="78"/>
+      <c r="C83" s="60">
+        <v>1</v>
+      </c>
+      <c r="D83" s="60" t="s">
+        <v>183</v>
+      </c>
+      <c r="E83" s="60">
+        <v>1650</v>
+      </c>
+      <c r="F83" s="60" t="s">
+        <v>110</v>
+      </c>
+      <c r="G83" s="61"/>
+    </row>
+    <row r="84" spans="1:7" x14ac:dyDescent="0.45">
+      <c r="A84" s="45"/>
+      <c r="B84" s="78"/>
+      <c r="C84" s="60">
+        <v>2</v>
+      </c>
+      <c r="D84" s="60" t="s">
+        <v>184</v>
+      </c>
+      <c r="E84" s="60">
+        <v>1650</v>
+      </c>
+      <c r="F84" s="60" t="s">
+        <v>107</v>
+      </c>
+      <c r="G84" s="61"/>
+    </row>
+    <row r="85" spans="1:7" x14ac:dyDescent="0.45">
+      <c r="A85" s="45"/>
+      <c r="B85" s="78"/>
+      <c r="C85" s="60">
+        <v>3</v>
+      </c>
+      <c r="D85" s="60" t="s">
+        <v>185</v>
+      </c>
+      <c r="E85" s="60">
+        <v>1650</v>
+      </c>
+      <c r="F85" s="60" t="s">
+        <v>110</v>
+      </c>
+      <c r="G85" s="61"/>
+    </row>
+    <row r="86" spans="1:7" x14ac:dyDescent="0.45">
+      <c r="A86" s="45"/>
+      <c r="B86" s="78"/>
+      <c r="C86" s="60">
+        <v>4</v>
+      </c>
+      <c r="D86" s="60" t="s">
+        <v>230</v>
+      </c>
+      <c r="E86" s="60">
+        <v>1650</v>
+      </c>
+      <c r="F86" s="60" t="s">
+        <v>107</v>
+      </c>
+      <c r="G86" s="61"/>
+    </row>
+    <row r="87" spans="1:7" x14ac:dyDescent="0.45">
+      <c r="A87" s="45"/>
+      <c r="B87" s="78"/>
+      <c r="C87" s="60">
+        <v>5</v>
+      </c>
+      <c r="D87" s="60" t="s">
+        <v>231</v>
+      </c>
+      <c r="E87" s="60">
+        <v>1650</v>
+      </c>
+      <c r="F87" s="60" t="s">
+        <v>107</v>
+      </c>
+      <c r="G87" s="61"/>
+    </row>
+    <row r="88" spans="1:7" x14ac:dyDescent="0.45">
+      <c r="A88" s="45"/>
+      <c r="B88" s="78"/>
+      <c r="C88" s="60">
+        <v>6</v>
+      </c>
+      <c r="D88" s="60" t="s">
+        <v>108</v>
+      </c>
+      <c r="E88" s="60">
+        <v>1650</v>
+      </c>
+      <c r="F88" s="60" t="s">
+        <v>107</v>
+      </c>
+      <c r="G88" s="61"/>
+    </row>
+    <row r="89" spans="1:7" x14ac:dyDescent="0.45">
+      <c r="A89" s="45"/>
+      <c r="B89" s="78"/>
+      <c r="C89" s="60">
+        <v>7</v>
+      </c>
+      <c r="D89" s="60" t="s">
+        <v>109</v>
+      </c>
+      <c r="E89" s="60">
+        <v>1650</v>
+      </c>
+      <c r="F89" s="60" t="s">
+        <v>110</v>
+      </c>
+      <c r="G89" s="61"/>
+    </row>
+    <row r="90" spans="1:7" x14ac:dyDescent="0.45">
+      <c r="A90" s="45"/>
+      <c r="B90" s="78"/>
+      <c r="C90" s="60">
+        <v>8</v>
+      </c>
+      <c r="D90" s="60" t="s">
+        <v>213</v>
+      </c>
+      <c r="E90" s="60">
+        <v>1650</v>
+      </c>
+      <c r="F90" s="60" t="s">
+        <v>107</v>
+      </c>
+      <c r="G90" s="61"/>
+    </row>
+    <row r="91" spans="1:7" x14ac:dyDescent="0.45">
+      <c r="A91" s="45"/>
+      <c r="B91" s="78"/>
+      <c r="C91" s="60">
+        <v>9</v>
+      </c>
+      <c r="D91" s="60" t="s">
+        <v>214</v>
+      </c>
+      <c r="E91" s="60">
+        <v>1650</v>
+      </c>
+      <c r="F91" s="60" t="s">
+        <v>110</v>
+      </c>
+      <c r="G91" s="61"/>
+    </row>
+    <row r="92" spans="1:7" ht="17.5" thickBot="1" x14ac:dyDescent="0.5">
+      <c r="A92" s="46"/>
+      <c r="B92" s="79"/>
+      <c r="C92" s="63">
+        <v>10</v>
+      </c>
+      <c r="D92" s="63" t="s">
+        <v>232</v>
+      </c>
+      <c r="E92" s="63">
+        <v>1650</v>
+      </c>
+      <c r="F92" s="63" t="s">
+        <v>107</v>
+      </c>
+      <c r="G92" s="64"/>
+    </row>
+    <row r="93" spans="1:7" ht="34" x14ac:dyDescent="0.45">
+      <c r="A93" s="44">
+        <v>5</v>
+      </c>
+      <c r="B93" s="50" t="s">
+        <v>210</v>
+      </c>
+      <c r="C93" s="58">
+        <v>0</v>
+      </c>
+      <c r="D93" s="58" t="s">
+        <v>106</v>
+      </c>
+      <c r="E93" s="58">
+        <v>160352</v>
+      </c>
+      <c r="F93" s="58" t="s">
+        <v>107</v>
+      </c>
+      <c r="G93" s="59" t="s">
+        <v>128</v>
+      </c>
+    </row>
+    <row r="94" spans="1:7" x14ac:dyDescent="0.45">
+      <c r="A94" s="45"/>
+      <c r="B94" s="48"/>
+      <c r="C94" s="60">
+        <v>1</v>
+      </c>
+      <c r="D94" s="60" t="s">
+        <v>182</v>
+      </c>
+      <c r="E94" s="60">
+        <v>160352</v>
+      </c>
+      <c r="F94" s="60" t="s">
+        <v>110</v>
+      </c>
+      <c r="G94" s="61"/>
+    </row>
+    <row r="95" spans="1:7" x14ac:dyDescent="0.45">
+      <c r="A95" s="45"/>
+      <c r="B95" s="48"/>
+      <c r="C95" s="60">
+        <v>2</v>
+      </c>
+      <c r="D95" s="60" t="s">
+        <v>183</v>
+      </c>
+      <c r="E95" s="60">
+        <v>160352</v>
+      </c>
+      <c r="F95" s="60" t="s">
+        <v>110</v>
+      </c>
+      <c r="G95" s="61"/>
+    </row>
+    <row r="96" spans="1:7" x14ac:dyDescent="0.45">
+      <c r="A96" s="45"/>
+      <c r="B96" s="48"/>
+      <c r="C96" s="60">
+        <v>3</v>
+      </c>
+      <c r="D96" s="60" t="s">
+        <v>184</v>
+      </c>
+      <c r="E96" s="60">
+        <v>160352</v>
+      </c>
+      <c r="F96" s="60" t="s">
+        <v>107</v>
+      </c>
+      <c r="G96" s="61"/>
+    </row>
+    <row r="97" spans="1:7" x14ac:dyDescent="0.45">
+      <c r="A97" s="45"/>
+      <c r="B97" s="48"/>
+      <c r="C97" s="60">
+        <v>4</v>
+      </c>
+      <c r="D97" s="60" t="s">
+        <v>185</v>
+      </c>
+      <c r="E97" s="60">
+        <v>160352</v>
+      </c>
+      <c r="F97" s="60" t="s">
+        <v>110</v>
+      </c>
+      <c r="G97" s="61"/>
+    </row>
+    <row r="98" spans="1:7" ht="68" x14ac:dyDescent="0.45">
+      <c r="A98" s="45"/>
+      <c r="B98" s="48"/>
+      <c r="C98" s="60">
+        <v>5</v>
+      </c>
+      <c r="D98" s="60" t="s">
+        <v>111</v>
+      </c>
+      <c r="E98" s="60">
+        <v>160352</v>
+      </c>
+      <c r="F98" s="60" t="s">
+        <v>110</v>
+      </c>
+      <c r="G98" s="62" t="s">
+        <v>129</v>
+      </c>
+    </row>
+    <row r="99" spans="1:7" x14ac:dyDescent="0.45">
+      <c r="A99" s="45"/>
+      <c r="B99" s="48"/>
+      <c r="C99" s="60">
+        <v>6</v>
+      </c>
+      <c r="D99" s="60" t="s">
+        <v>112</v>
+      </c>
+      <c r="E99" s="60">
+        <v>160352</v>
+      </c>
+      <c r="F99" s="60" t="s">
+        <v>110</v>
+      </c>
+      <c r="G99" s="61"/>
+    </row>
+    <row r="100" spans="1:7" ht="34" x14ac:dyDescent="0.45">
+      <c r="A100" s="45"/>
+      <c r="B100" s="48"/>
+      <c r="C100" s="60">
+        <v>7</v>
+      </c>
+      <c r="D100" s="60" t="s">
+        <v>114</v>
+      </c>
+      <c r="E100" s="60">
+        <v>160352</v>
+      </c>
+      <c r="F100" s="60" t="s">
+        <v>107</v>
+      </c>
+      <c r="G100" s="62" t="s">
+        <v>211</v>
+      </c>
+    </row>
+    <row r="101" spans="1:7" ht="68" x14ac:dyDescent="0.45">
+      <c r="A101" s="45"/>
+      <c r="B101" s="48"/>
+      <c r="C101" s="60">
+        <v>8</v>
+      </c>
+      <c r="D101" s="60" t="s">
+        <v>113</v>
+      </c>
+      <c r="E101" s="60">
+        <v>160352</v>
+      </c>
+      <c r="F101" s="60" t="s">
+        <v>107</v>
+      </c>
+      <c r="G101" s="62" t="s">
+        <v>212</v>
+      </c>
+    </row>
+    <row r="102" spans="1:7" x14ac:dyDescent="0.45">
+      <c r="A102" s="45"/>
+      <c r="B102" s="48"/>
+      <c r="C102" s="60">
+        <v>9</v>
+      </c>
+      <c r="D102" s="60" t="s">
+        <v>116</v>
+      </c>
+      <c r="E102" s="60">
+        <v>160352</v>
+      </c>
+      <c r="F102" s="60" t="s">
+        <v>107</v>
+      </c>
+      <c r="G102" s="61"/>
+    </row>
+    <row r="103" spans="1:7" x14ac:dyDescent="0.45">
+      <c r="A103" s="45"/>
+      <c r="B103" s="48"/>
+      <c r="C103" s="60">
+        <v>10</v>
+      </c>
+      <c r="D103" s="60" t="s">
+        <v>118</v>
+      </c>
+      <c r="E103" s="60">
+        <v>160352</v>
+      </c>
+      <c r="F103" s="60" t="s">
+        <v>107</v>
+      </c>
+      <c r="G103" s="61"/>
+    </row>
+    <row r="104" spans="1:7" x14ac:dyDescent="0.45">
+      <c r="A104" s="45"/>
+      <c r="B104" s="48"/>
+      <c r="C104" s="60">
+        <v>11</v>
+      </c>
+      <c r="D104" s="60" t="s">
+        <v>119</v>
+      </c>
+      <c r="E104" s="60">
+        <v>160352</v>
+      </c>
+      <c r="F104" s="60" t="s">
+        <v>107</v>
+      </c>
+      <c r="G104" s="61"/>
+    </row>
+    <row r="105" spans="1:7" x14ac:dyDescent="0.45">
+      <c r="A105" s="45"/>
+      <c r="B105" s="48"/>
+      <c r="C105" s="60">
+        <v>12</v>
+      </c>
+      <c r="D105" s="60" t="s">
+        <v>124</v>
+      </c>
+      <c r="E105" s="60">
+        <v>160352</v>
+      </c>
+      <c r="F105" s="60" t="s">
+        <v>107</v>
+      </c>
+      <c r="G105" s="61"/>
+    </row>
+    <row r="106" spans="1:7" ht="17.5" thickBot="1" x14ac:dyDescent="0.5">
+      <c r="A106" s="46"/>
+      <c r="B106" s="51"/>
+      <c r="C106" s="63">
+        <v>13</v>
+      </c>
+      <c r="D106" s="63" t="s">
+        <v>115</v>
+      </c>
+      <c r="E106" s="63">
+        <v>160352</v>
+      </c>
+      <c r="F106" s="63" t="s">
+        <v>107</v>
+      </c>
+      <c r="G106" s="64"/>
+    </row>
+    <row r="107" spans="1:7" ht="34" x14ac:dyDescent="0.45">
+      <c r="A107" s="44">
+        <v>6</v>
+      </c>
+      <c r="B107" s="50" t="s">
+        <v>206</v>
+      </c>
+      <c r="C107" s="58">
+        <v>0</v>
+      </c>
+      <c r="D107" s="58" t="s">
+        <v>106</v>
+      </c>
+      <c r="E107" s="58">
+        <v>20514</v>
+      </c>
+      <c r="F107" s="58" t="s">
+        <v>107</v>
+      </c>
+      <c r="G107" s="59" t="s">
+        <v>128</v>
+      </c>
+    </row>
+    <row r="108" spans="1:7" x14ac:dyDescent="0.45">
+      <c r="A108" s="45"/>
+      <c r="B108" s="48"/>
+      <c r="C108" s="60">
+        <v>1</v>
+      </c>
+      <c r="D108" s="60" t="s">
+        <v>182</v>
+      </c>
+      <c r="E108" s="60">
+        <v>20514</v>
+      </c>
+      <c r="F108" s="60" t="s">
+        <v>110</v>
+      </c>
+      <c r="G108" s="61"/>
+    </row>
+    <row r="109" spans="1:7" x14ac:dyDescent="0.45">
+      <c r="A109" s="45"/>
+      <c r="B109" s="48"/>
+      <c r="C109" s="60">
+        <v>2</v>
+      </c>
+      <c r="D109" s="60" t="s">
+        <v>183</v>
+      </c>
+      <c r="E109" s="60">
+        <v>20514</v>
+      </c>
+      <c r="F109" s="60" t="s">
+        <v>110</v>
+      </c>
+      <c r="G109" s="61"/>
+    </row>
+    <row r="110" spans="1:7" x14ac:dyDescent="0.45">
+      <c r="A110" s="45"/>
+      <c r="B110" s="48"/>
+      <c r="C110" s="60">
+        <v>3</v>
+      </c>
+      <c r="D110" s="60" t="s">
+        <v>184</v>
+      </c>
+      <c r="E110" s="60">
+        <v>20514</v>
+      </c>
+      <c r="F110" s="60" t="s">
+        <v>107</v>
+      </c>
+      <c r="G110" s="61"/>
+    </row>
+    <row r="111" spans="1:7" x14ac:dyDescent="0.45">
+      <c r="A111" s="45"/>
+      <c r="B111" s="48"/>
+      <c r="C111" s="60">
+        <v>4</v>
+      </c>
+      <c r="D111" s="60" t="s">
+        <v>185</v>
+      </c>
+      <c r="E111" s="60">
+        <v>20514</v>
+      </c>
+      <c r="F111" s="60" t="s">
+        <v>110</v>
+      </c>
+      <c r="G111" s="61"/>
+    </row>
+    <row r="112" spans="1:7" x14ac:dyDescent="0.45">
+      <c r="A112" s="45"/>
+      <c r="B112" s="48"/>
+      <c r="C112" s="60">
+        <v>5</v>
+      </c>
+      <c r="D112" s="60" t="s">
+        <v>186</v>
+      </c>
+      <c r="E112" s="60">
+        <v>20514</v>
+      </c>
+      <c r="F112" s="60" t="s">
+        <v>107</v>
+      </c>
+      <c r="G112" s="61" t="s">
+        <v>267</v>
+      </c>
+    </row>
+    <row r="113" spans="1:7" x14ac:dyDescent="0.45">
+      <c r="A113" s="45"/>
+      <c r="B113" s="48"/>
+      <c r="C113" s="60">
+        <v>6</v>
+      </c>
+      <c r="D113" s="60" t="s">
+        <v>187</v>
+      </c>
+      <c r="E113" s="60">
+        <v>20514</v>
+      </c>
+      <c r="F113" s="60" t="s">
+        <v>117</v>
+      </c>
+      <c r="G113" s="61"/>
+    </row>
+    <row r="114" spans="1:7" x14ac:dyDescent="0.45">
+      <c r="A114" s="45"/>
+      <c r="B114" s="48"/>
+      <c r="C114" s="60">
+        <v>7</v>
+      </c>
+      <c r="D114" s="60" t="s">
+        <v>188</v>
+      </c>
+      <c r="E114" s="60">
+        <v>20514</v>
+      </c>
+      <c r="F114" s="60" t="s">
+        <v>117</v>
+      </c>
+      <c r="G114" s="61"/>
+    </row>
+    <row r="115" spans="1:7" x14ac:dyDescent="0.45">
+      <c r="A115" s="45"/>
+      <c r="B115" s="48"/>
+      <c r="C115" s="60">
+        <v>8</v>
+      </c>
+      <c r="D115" s="60" t="s">
+        <v>189</v>
+      </c>
+      <c r="E115" s="60">
+        <v>20514</v>
+      </c>
+      <c r="F115" s="60" t="s">
+        <v>117</v>
+      </c>
+      <c r="G115" s="61"/>
+    </row>
+    <row r="116" spans="1:7" x14ac:dyDescent="0.45">
+      <c r="A116" s="45"/>
+      <c r="B116" s="48"/>
+      <c r="C116" s="60">
+        <v>9</v>
+      </c>
+      <c r="D116" s="60" t="s">
+        <v>190</v>
+      </c>
+      <c r="E116" s="60">
+        <v>20514</v>
+      </c>
+      <c r="F116" s="60" t="s">
+        <v>117</v>
+      </c>
+      <c r="G116" s="61"/>
+    </row>
+    <row r="117" spans="1:7" x14ac:dyDescent="0.45">
+      <c r="A117" s="45"/>
+      <c r="B117" s="48"/>
+      <c r="C117" s="60">
+        <v>10</v>
+      </c>
+      <c r="D117" s="60" t="s">
+        <v>191</v>
+      </c>
+      <c r="E117" s="60">
+        <v>20514</v>
+      </c>
+      <c r="F117" s="60" t="s">
+        <v>117</v>
+      </c>
+      <c r="G117" s="61"/>
+    </row>
+    <row r="118" spans="1:7" x14ac:dyDescent="0.45">
+      <c r="A118" s="45"/>
+      <c r="B118" s="48"/>
+      <c r="C118" s="60">
+        <v>11</v>
+      </c>
+      <c r="D118" s="60" t="s">
+        <v>192</v>
+      </c>
+      <c r="E118" s="60">
+        <v>20514</v>
+      </c>
+      <c r="F118" s="60" t="s">
+        <v>117</v>
+      </c>
+      <c r="G118" s="61"/>
+    </row>
+    <row r="119" spans="1:7" x14ac:dyDescent="0.45">
+      <c r="A119" s="45"/>
+      <c r="B119" s="48"/>
+      <c r="C119" s="60">
+        <v>12</v>
+      </c>
+      <c r="D119" s="60" t="s">
+        <v>193</v>
+      </c>
+      <c r="E119" s="60">
+        <v>20514</v>
+      </c>
+      <c r="F119" s="60" t="s">
+        <v>117</v>
+      </c>
+      <c r="G119" s="61"/>
+    </row>
+    <row r="120" spans="1:7" x14ac:dyDescent="0.45">
+      <c r="A120" s="45"/>
+      <c r="B120" s="48"/>
+      <c r="C120" s="60">
+        <v>13</v>
+      </c>
+      <c r="D120" s="60" t="s">
+        <v>194</v>
+      </c>
+      <c r="E120" s="60">
+        <v>20514</v>
+      </c>
+      <c r="F120" s="60" t="s">
+        <v>117</v>
+      </c>
+      <c r="G120" s="61"/>
+    </row>
+    <row r="121" spans="1:7" x14ac:dyDescent="0.45">
+      <c r="A121" s="45"/>
+      <c r="B121" s="48"/>
+      <c r="C121" s="60">
+        <v>14</v>
+      </c>
+      <c r="D121" s="60" t="s">
+        <v>195</v>
+      </c>
+      <c r="E121" s="60">
+        <v>20514</v>
+      </c>
+      <c r="F121" s="60" t="s">
+        <v>117</v>
+      </c>
+      <c r="G121" s="61"/>
+    </row>
+    <row r="122" spans="1:7" x14ac:dyDescent="0.45">
+      <c r="A122" s="45"/>
+      <c r="B122" s="48"/>
+      <c r="C122" s="60">
+        <v>15</v>
+      </c>
+      <c r="D122" s="60" t="s">
+        <v>196</v>
+      </c>
+      <c r="E122" s="60">
+        <v>20514</v>
+      </c>
+      <c r="F122" s="60" t="s">
+        <v>117</v>
+      </c>
+      <c r="G122" s="61"/>
+    </row>
+    <row r="123" spans="1:7" x14ac:dyDescent="0.45">
+      <c r="A123" s="45"/>
+      <c r="B123" s="48"/>
+      <c r="C123" s="60">
+        <v>16</v>
+      </c>
+      <c r="D123" s="60" t="s">
+        <v>197</v>
+      </c>
+      <c r="E123" s="60">
+        <v>20514</v>
+      </c>
+      <c r="F123" s="60" t="s">
+        <v>117</v>
+      </c>
+      <c r="G123" s="61"/>
+    </row>
+    <row r="124" spans="1:7" x14ac:dyDescent="0.45">
+      <c r="A124" s="45"/>
+      <c r="B124" s="48"/>
+      <c r="C124" s="60">
+        <v>17</v>
+      </c>
+      <c r="D124" s="60" t="s">
+        <v>198</v>
+      </c>
+      <c r="E124" s="60">
+        <v>20514</v>
+      </c>
+      <c r="F124" s="60" t="s">
+        <v>117</v>
+      </c>
+      <c r="G124" s="61"/>
+    </row>
+    <row r="125" spans="1:7" x14ac:dyDescent="0.45">
+      <c r="A125" s="45"/>
+      <c r="B125" s="48"/>
+      <c r="C125" s="60">
+        <v>18</v>
+      </c>
+      <c r="D125" s="60" t="s">
+        <v>199</v>
+      </c>
+      <c r="E125" s="60">
+        <v>20514</v>
+      </c>
+      <c r="F125" s="60" t="s">
+        <v>117</v>
+      </c>
+      <c r="G125" s="61"/>
+    </row>
+    <row r="126" spans="1:7" x14ac:dyDescent="0.45">
+      <c r="A126" s="45"/>
+      <c r="B126" s="48"/>
+      <c r="C126" s="60">
+        <v>19</v>
+      </c>
+      <c r="D126" s="60" t="s">
+        <v>200</v>
+      </c>
+      <c r="E126" s="60">
+        <v>20514</v>
+      </c>
+      <c r="F126" s="60" t="s">
+        <v>117</v>
+      </c>
+      <c r="G126" s="61"/>
+    </row>
+    <row r="127" spans="1:7" x14ac:dyDescent="0.45">
+      <c r="A127" s="45"/>
+      <c r="B127" s="48"/>
+      <c r="C127" s="60">
+        <v>20</v>
+      </c>
+      <c r="D127" s="60" t="s">
+        <v>201</v>
+      </c>
+      <c r="E127" s="60">
+        <v>20514</v>
+      </c>
+      <c r="F127" s="60" t="s">
+        <v>117</v>
+      </c>
+      <c r="G127" s="61"/>
+    </row>
+    <row r="128" spans="1:7" x14ac:dyDescent="0.45">
+      <c r="A128" s="45"/>
+      <c r="B128" s="48"/>
+      <c r="C128" s="60">
+        <v>21</v>
+      </c>
+      <c r="D128" s="60" t="s">
+        <v>202</v>
+      </c>
+      <c r="E128" s="60">
+        <v>20514</v>
+      </c>
+      <c r="F128" s="60" t="s">
+        <v>117</v>
+      </c>
+      <c r="G128" s="61"/>
+    </row>
+    <row r="129" spans="1:7" x14ac:dyDescent="0.45">
+      <c r="A129" s="45"/>
+      <c r="B129" s="48"/>
+      <c r="C129" s="60">
+        <v>22</v>
+      </c>
+      <c r="D129" s="60" t="s">
+        <v>203</v>
+      </c>
+      <c r="E129" s="60">
+        <v>20514</v>
+      </c>
+      <c r="F129" s="60" t="s">
+        <v>117</v>
+      </c>
+      <c r="G129" s="61"/>
+    </row>
+    <row r="130" spans="1:7" x14ac:dyDescent="0.45">
+      <c r="A130" s="45"/>
+      <c r="B130" s="48"/>
+      <c r="C130" s="60">
+        <v>23</v>
+      </c>
+      <c r="D130" s="60" t="s">
+        <v>204</v>
+      </c>
+      <c r="E130" s="60">
+        <v>20514</v>
+      </c>
+      <c r="F130" s="60" t="s">
+        <v>117</v>
+      </c>
+      <c r="G130" s="61"/>
+    </row>
+    <row r="131" spans="1:7" ht="17.5" thickBot="1" x14ac:dyDescent="0.5">
+      <c r="A131" s="46"/>
+      <c r="B131" s="51"/>
+      <c r="C131" s="63">
+        <v>24</v>
+      </c>
+      <c r="D131" s="63" t="s">
+        <v>205</v>
+      </c>
+      <c r="E131" s="63">
+        <v>20514</v>
+      </c>
+      <c r="F131" s="63" t="s">
+        <v>117</v>
+      </c>
+      <c r="G131" s="64"/>
+    </row>
+    <row r="132" spans="1:7" ht="34" x14ac:dyDescent="0.45">
+      <c r="A132" s="44">
+        <v>7</v>
+      </c>
+      <c r="B132" s="75" t="s">
+        <v>228</v>
+      </c>
+      <c r="C132" s="58">
+        <v>0</v>
+      </c>
+      <c r="D132" s="58" t="s">
+        <v>106</v>
+      </c>
+      <c r="E132" s="58">
+        <v>325</v>
+      </c>
+      <c r="F132" s="58" t="s">
+        <v>107</v>
+      </c>
+      <c r="G132" s="59" t="s">
+        <v>128</v>
+      </c>
+    </row>
+    <row r="133" spans="1:7" x14ac:dyDescent="0.45">
+      <c r="A133" s="45"/>
+      <c r="B133" s="78"/>
+      <c r="C133" s="60">
+        <v>1</v>
+      </c>
+      <c r="D133" s="60" t="s">
+        <v>108</v>
+      </c>
+      <c r="E133" s="60">
+        <v>325</v>
+      </c>
+      <c r="F133" s="60" t="s">
+        <v>107</v>
+      </c>
+      <c r="G133" s="61"/>
+    </row>
+    <row r="134" spans="1:7" x14ac:dyDescent="0.45">
+      <c r="A134" s="45"/>
+      <c r="B134" s="78"/>
+      <c r="C134" s="60">
+        <v>2</v>
+      </c>
+      <c r="D134" s="60" t="s">
+        <v>109</v>
+      </c>
+      <c r="E134" s="60">
+        <v>325</v>
+      </c>
+      <c r="F134" s="60" t="s">
+        <v>110</v>
+      </c>
+      <c r="G134" s="61"/>
+    </row>
+    <row r="135" spans="1:7" x14ac:dyDescent="0.45">
+      <c r="A135" s="45"/>
+      <c r="B135" s="78"/>
+      <c r="C135" s="60">
+        <v>3</v>
+      </c>
+      <c r="D135" s="60" t="s">
+        <v>240</v>
+      </c>
+      <c r="E135" s="60">
+        <v>325</v>
+      </c>
+      <c r="F135" s="60" t="s">
+        <v>107</v>
+      </c>
+      <c r="G135" s="61" t="s">
+        <v>265</v>
+      </c>
+    </row>
+    <row r="136" spans="1:7" x14ac:dyDescent="0.45">
+      <c r="A136" s="45"/>
+      <c r="B136" s="78"/>
+      <c r="C136" s="60">
+        <v>4</v>
+      </c>
+      <c r="D136" s="60" t="s">
+        <v>241</v>
+      </c>
+      <c r="E136" s="60">
+        <v>325</v>
+      </c>
+      <c r="F136" s="60" t="s">
+        <v>107</v>
+      </c>
+      <c r="G136" s="61"/>
+    </row>
+    <row r="137" spans="1:7" x14ac:dyDescent="0.45">
+      <c r="A137" s="45"/>
+      <c r="B137" s="78"/>
+      <c r="C137" s="60">
+        <v>5</v>
+      </c>
+      <c r="D137" s="60" t="s">
+        <v>242</v>
+      </c>
+      <c r="E137" s="60">
+        <v>325</v>
+      </c>
+      <c r="F137" s="60" t="s">
+        <v>107</v>
+      </c>
+      <c r="G137" s="61"/>
+    </row>
+    <row r="138" spans="1:7" x14ac:dyDescent="0.45">
+      <c r="A138" s="45"/>
+      <c r="B138" s="78"/>
+      <c r="C138" s="60">
+        <v>6</v>
+      </c>
+      <c r="D138" s="60" t="s">
+        <v>243</v>
+      </c>
+      <c r="E138" s="60">
+        <v>325</v>
+      </c>
+      <c r="F138" s="60" t="s">
+        <v>107</v>
+      </c>
+      <c r="G138" s="61"/>
+    </row>
+    <row r="139" spans="1:7" x14ac:dyDescent="0.45">
+      <c r="A139" s="45"/>
+      <c r="B139" s="78"/>
+      <c r="C139" s="60">
+        <v>7</v>
+      </c>
+      <c r="D139" s="60" t="s">
+        <v>244</v>
+      </c>
+      <c r="E139" s="60">
+        <v>325</v>
+      </c>
+      <c r="F139" s="60" t="s">
+        <v>107</v>
+      </c>
+      <c r="G139" s="61"/>
+    </row>
+    <row r="140" spans="1:7" x14ac:dyDescent="0.45">
+      <c r="A140" s="45"/>
+      <c r="B140" s="78"/>
+      <c r="C140" s="60">
+        <v>8</v>
+      </c>
+      <c r="D140" s="60" t="s">
+        <v>245</v>
+      </c>
+      <c r="E140" s="60">
+        <v>325</v>
+      </c>
+      <c r="F140" s="60" t="s">
+        <v>107</v>
+      </c>
+      <c r="G140" s="61"/>
+    </row>
+    <row r="141" spans="1:7" x14ac:dyDescent="0.45">
+      <c r="A141" s="45"/>
+      <c r="B141" s="78"/>
+      <c r="C141" s="60">
+        <v>9</v>
+      </c>
+      <c r="D141" s="60" t="s">
+        <v>246</v>
+      </c>
+      <c r="E141" s="60">
+        <v>325</v>
+      </c>
+      <c r="F141" s="60" t="s">
+        <v>107</v>
+      </c>
+      <c r="G141" s="61"/>
+    </row>
+    <row r="142" spans="1:7" x14ac:dyDescent="0.45">
+      <c r="A142" s="45"/>
+      <c r="B142" s="78"/>
+      <c r="C142" s="60">
+        <v>10</v>
+      </c>
+      <c r="D142" s="60" t="s">
+        <v>247</v>
+      </c>
+      <c r="E142" s="60">
+        <v>325</v>
+      </c>
+      <c r="F142" s="60" t="s">
+        <v>107</v>
+      </c>
+      <c r="G142" s="61"/>
+    </row>
+    <row r="143" spans="1:7" x14ac:dyDescent="0.45">
+      <c r="A143" s="45"/>
+      <c r="B143" s="78"/>
+      <c r="C143" s="60">
+        <v>11</v>
+      </c>
+      <c r="D143" s="60" t="s">
+        <v>248</v>
+      </c>
+      <c r="E143" s="60">
+        <v>325</v>
+      </c>
+      <c r="F143" s="60" t="s">
+        <v>107</v>
+      </c>
+      <c r="G143" s="61"/>
+    </row>
+    <row r="144" spans="1:7" x14ac:dyDescent="0.45">
+      <c r="A144" s="45"/>
+      <c r="B144" s="78"/>
+      <c r="C144" s="60">
+        <v>12</v>
+      </c>
+      <c r="D144" s="60" t="s">
+        <v>249</v>
+      </c>
+      <c r="E144" s="60">
+        <v>325</v>
+      </c>
+      <c r="F144" s="60" t="s">
+        <v>107</v>
+      </c>
+      <c r="G144" s="61"/>
+    </row>
+    <row r="145" spans="1:7" x14ac:dyDescent="0.45">
+      <c r="A145" s="45"/>
+      <c r="B145" s="78"/>
+      <c r="C145" s="60">
+        <v>13</v>
+      </c>
+      <c r="D145" s="60" t="s">
+        <v>250</v>
+      </c>
+      <c r="E145" s="60">
+        <v>325</v>
+      </c>
+      <c r="F145" s="60" t="s">
+        <v>107</v>
+      </c>
+      <c r="G145" s="61"/>
+    </row>
+    <row r="146" spans="1:7" x14ac:dyDescent="0.45">
+      <c r="A146" s="45"/>
+      <c r="B146" s="78"/>
+      <c r="C146" s="60">
+        <v>14</v>
+      </c>
+      <c r="D146" s="60" t="s">
+        <v>251</v>
+      </c>
+      <c r="E146" s="60">
+        <v>325</v>
+      </c>
+      <c r="F146" s="60" t="s">
+        <v>107</v>
+      </c>
+      <c r="G146" s="61"/>
+    </row>
+    <row r="147" spans="1:7" x14ac:dyDescent="0.45">
+      <c r="A147" s="45"/>
+      <c r="B147" s="78"/>
+      <c r="C147" s="60">
+        <v>15</v>
+      </c>
+      <c r="D147" s="60" t="s">
+        <v>252</v>
+      </c>
+      <c r="E147" s="60">
+        <v>325</v>
+      </c>
+      <c r="F147" s="60" t="s">
+        <v>107</v>
+      </c>
+      <c r="G147" s="61"/>
+    </row>
+    <row r="148" spans="1:7" x14ac:dyDescent="0.45">
+      <c r="A148" s="45"/>
+      <c r="B148" s="78"/>
+      <c r="C148" s="60">
+        <v>16</v>
+      </c>
+      <c r="D148" s="60" t="s">
+        <v>253</v>
+      </c>
+      <c r="E148" s="60">
+        <v>325</v>
+      </c>
+      <c r="F148" s="60" t="s">
+        <v>107</v>
+      </c>
+      <c r="G148" s="61"/>
+    </row>
+    <row r="149" spans="1:7" x14ac:dyDescent="0.45">
+      <c r="A149" s="45"/>
+      <c r="B149" s="78"/>
+      <c r="C149" s="60">
+        <v>17</v>
+      </c>
+      <c r="D149" s="60" t="s">
+        <v>254</v>
+      </c>
+      <c r="E149" s="60">
+        <v>325</v>
+      </c>
+      <c r="F149" s="60" t="s">
+        <v>107</v>
+      </c>
+      <c r="G149" s="61"/>
+    </row>
+    <row r="150" spans="1:7" x14ac:dyDescent="0.45">
+      <c r="A150" s="45"/>
+      <c r="B150" s="78"/>
+      <c r="C150" s="60">
+        <v>18</v>
+      </c>
+      <c r="D150" s="60" t="s">
+        <v>255</v>
+      </c>
+      <c r="E150" s="60">
+        <v>325</v>
+      </c>
+      <c r="F150" s="60" t="s">
+        <v>107</v>
+      </c>
+      <c r="G150" s="61"/>
+    </row>
+    <row r="151" spans="1:7" x14ac:dyDescent="0.45">
+      <c r="A151" s="45"/>
+      <c r="B151" s="78"/>
+      <c r="C151" s="60">
+        <v>19</v>
+      </c>
+      <c r="D151" s="60" t="s">
+        <v>256</v>
+      </c>
+      <c r="E151" s="60">
+        <v>325</v>
+      </c>
+      <c r="F151" s="60" t="s">
+        <v>107</v>
+      </c>
+      <c r="G151" s="61"/>
+    </row>
+    <row r="152" spans="1:7" x14ac:dyDescent="0.45">
+      <c r="A152" s="45"/>
+      <c r="B152" s="78"/>
+      <c r="C152" s="60">
+        <v>20</v>
+      </c>
+      <c r="D152" s="60" t="s">
+        <v>257</v>
+      </c>
+      <c r="E152" s="60">
+        <v>325</v>
+      </c>
+      <c r="F152" s="60" t="s">
+        <v>107</v>
+      </c>
+      <c r="G152" s="61"/>
+    </row>
+    <row r="153" spans="1:7" x14ac:dyDescent="0.45">
+      <c r="A153" s="45"/>
+      <c r="B153" s="78"/>
+      <c r="C153" s="60">
+        <v>21</v>
+      </c>
+      <c r="D153" s="60" t="s">
+        <v>258</v>
+      </c>
+      <c r="E153" s="60">
+        <v>325</v>
+      </c>
+      <c r="F153" s="60" t="s">
+        <v>107</v>
+      </c>
+      <c r="G153" s="61"/>
+    </row>
+    <row r="154" spans="1:7" x14ac:dyDescent="0.45">
+      <c r="A154" s="45"/>
+      <c r="B154" s="78"/>
+      <c r="C154" s="60">
+        <v>22</v>
+      </c>
+      <c r="D154" s="60" t="s">
+        <v>259</v>
+      </c>
+      <c r="E154" s="60">
+        <v>325</v>
+      </c>
+      <c r="F154" s="60" t="s">
+        <v>107</v>
+      </c>
+      <c r="G154" s="61"/>
+    </row>
+    <row r="155" spans="1:7" x14ac:dyDescent="0.45">
+      <c r="A155" s="45"/>
+      <c r="B155" s="78"/>
+      <c r="C155" s="60">
+        <v>23</v>
+      </c>
+      <c r="D155" s="60" t="s">
+        <v>260</v>
+      </c>
+      <c r="E155" s="60">
+        <v>325</v>
+      </c>
+      <c r="F155" s="60" t="s">
+        <v>107</v>
+      </c>
+      <c r="G155" s="61"/>
+    </row>
+    <row r="156" spans="1:7" ht="17.5" thickBot="1" x14ac:dyDescent="0.5">
+      <c r="A156" s="46"/>
+      <c r="B156" s="79"/>
+      <c r="C156" s="63">
+        <v>24</v>
+      </c>
+      <c r="D156" s="63" t="s">
+        <v>261</v>
+      </c>
+      <c r="E156" s="63">
+        <v>325</v>
+      </c>
+      <c r="F156" s="63" t="s">
+        <v>107</v>
+      </c>
+      <c r="G156" s="64"/>
+    </row>
+    <row r="157" spans="1:7" ht="34" x14ac:dyDescent="0.45">
+      <c r="A157" s="44">
+        <v>8</v>
+      </c>
+      <c r="B157" s="75" t="s">
+        <v>233</v>
+      </c>
+      <c r="C157" s="58">
+        <v>0</v>
+      </c>
+      <c r="D157" s="58" t="s">
+        <v>106</v>
+      </c>
+      <c r="E157" s="58">
+        <v>325</v>
+      </c>
+      <c r="F157" s="58" t="s">
+        <v>107</v>
+      </c>
+      <c r="G157" s="59" t="s">
+        <v>128</v>
+      </c>
+    </row>
+    <row r="158" spans="1:7" x14ac:dyDescent="0.45">
+      <c r="A158" s="45"/>
+      <c r="B158" s="78"/>
+      <c r="C158" s="60">
+        <v>1</v>
+      </c>
+      <c r="D158" s="60" t="s">
+        <v>108</v>
+      </c>
+      <c r="E158" s="60">
+        <v>325</v>
+      </c>
+      <c r="F158" s="60" t="s">
+        <v>107</v>
+      </c>
+      <c r="G158" s="61"/>
+    </row>
+    <row r="159" spans="1:7" x14ac:dyDescent="0.45">
+      <c r="A159" s="45"/>
+      <c r="B159" s="78"/>
+      <c r="C159" s="60">
+        <v>2</v>
+      </c>
+      <c r="D159" s="60" t="s">
+        <v>109</v>
+      </c>
+      <c r="E159" s="60">
+        <v>325</v>
+      </c>
+      <c r="F159" s="60" t="s">
+        <v>110</v>
+      </c>
+      <c r="G159" s="61"/>
+    </row>
+    <row r="160" spans="1:7" ht="68" x14ac:dyDescent="0.45">
+      <c r="A160" s="45"/>
+      <c r="B160" s="78"/>
+      <c r="C160" s="60">
+        <v>3</v>
+      </c>
+      <c r="D160" s="60" t="s">
+        <v>234</v>
+      </c>
+      <c r="E160" s="60">
+        <v>325</v>
+      </c>
+      <c r="F160" s="60" t="s">
+        <v>110</v>
+      </c>
+      <c r="G160" s="62" t="s">
+        <v>266</v>
+      </c>
+    </row>
+    <row r="161" spans="1:7" x14ac:dyDescent="0.45">
+      <c r="A161" s="45"/>
+      <c r="B161" s="78"/>
+      <c r="C161" s="60">
+        <v>4</v>
+      </c>
+      <c r="D161" s="60" t="s">
+        <v>235</v>
+      </c>
+      <c r="E161" s="60">
+        <v>325</v>
+      </c>
+      <c r="F161" s="60" t="s">
+        <v>110</v>
+      </c>
+      <c r="G161" s="61"/>
+    </row>
+    <row r="162" spans="1:7" x14ac:dyDescent="0.45">
+      <c r="A162" s="45"/>
+      <c r="B162" s="78"/>
+      <c r="C162" s="60">
+        <v>5</v>
+      </c>
+      <c r="D162" s="60" t="s">
+        <v>236</v>
+      </c>
+      <c r="E162" s="60">
+        <v>325</v>
+      </c>
+      <c r="F162" s="60" t="s">
+        <v>107</v>
+      </c>
+      <c r="G162" s="61"/>
+    </row>
+    <row r="163" spans="1:7" x14ac:dyDescent="0.45">
+      <c r="A163" s="45"/>
+      <c r="B163" s="78"/>
+      <c r="C163" s="60">
+        <v>6</v>
+      </c>
+      <c r="D163" s="60" t="s">
+        <v>237</v>
+      </c>
+      <c r="E163" s="60">
+        <v>325</v>
+      </c>
+      <c r="F163" s="60" t="s">
+        <v>107</v>
+      </c>
+      <c r="G163" s="61"/>
+    </row>
+    <row r="164" spans="1:7" x14ac:dyDescent="0.45">
+      <c r="A164" s="45"/>
+      <c r="B164" s="78"/>
+      <c r="C164" s="60">
+        <v>7</v>
+      </c>
+      <c r="D164" s="60" t="s">
+        <v>238</v>
+      </c>
+      <c r="E164" s="60">
+        <v>325</v>
+      </c>
+      <c r="F164" s="60" t="s">
+        <v>107</v>
+      </c>
+      <c r="G164" s="61"/>
+    </row>
+    <row r="165" spans="1:7" ht="17.5" thickBot="1" x14ac:dyDescent="0.5">
+      <c r="A165" s="46"/>
+      <c r="B165" s="79"/>
+      <c r="C165" s="63">
+        <v>8</v>
+      </c>
+      <c r="D165" s="63" t="s">
+        <v>239</v>
+      </c>
+      <c r="E165" s="63">
+        <v>325</v>
+      </c>
+      <c r="F165" s="63" t="s">
+        <v>107</v>
+      </c>
+      <c r="G165" s="64"/>
     </row>
   </sheetData>
+  <autoFilter ref="B2:G2" xr:uid="{1402F3D2-E44E-49CC-8D75-9BA854A3E719}">
+    <filterColumn colId="3" showButton="0"/>
+  </autoFilter>
+  <mergeCells count="17">
+    <mergeCell ref="A82:A92"/>
+    <mergeCell ref="B82:B92"/>
+    <mergeCell ref="B157:B165"/>
+    <mergeCell ref="A157:A165"/>
+    <mergeCell ref="B132:B156"/>
+    <mergeCell ref="A132:A156"/>
+    <mergeCell ref="B107:B131"/>
+    <mergeCell ref="A1:G1"/>
+    <mergeCell ref="A3:A14"/>
+    <mergeCell ref="A107:A131"/>
+    <mergeCell ref="B93:B106"/>
+    <mergeCell ref="A93:A106"/>
+    <mergeCell ref="A68:A81"/>
+    <mergeCell ref="B68:B81"/>
+    <mergeCell ref="B15:B67"/>
+    <mergeCell ref="A15:A67"/>
+    <mergeCell ref="B3:B14"/>
+  </mergeCells>
   <phoneticPr fontId="1" type="noConversion"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>

<commit_message>
project 관련 파일 업로드_20260824_3
</commit_message>
<xml_diff>
--- a/Project_1/Project Status.xlsx
+++ b/Project_1/Project Status.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\pyostry\workspace\aiffel\ai-data-bootcamp\Project_1\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{799EF382-2A9F-474C-9390-D0B75A541E90}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6CF4EE9F-A8AE-4280-A76A-14A19917807E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="30612" yWindow="-108" windowWidth="30936" windowHeight="16776" activeTab="5" xr2:uid="{6B636699-A6E6-472F-A92F-8A8168DF527A}"/>
+    <workbookView xWindow="-110" yWindow="-110" windowWidth="25820" windowHeight="15500" activeTab="3" xr2:uid="{6B636699-A6E6-472F-A92F-8A8168DF527A}"/>
   </bookViews>
   <sheets>
     <sheet name="0. Status" sheetId="3" r:id="rId1"/>
@@ -52,9 +52,6 @@
   </si>
   <si>
     <t>5. 인사이트(Insight) — 발견이 비즈니스 맥락에서 갖는 의미, 왜 그런 패턴이 나타나는가</t>
-  </si>
-  <si>
-    <t>6. 비즈니스 제언(Recommendation) — 최소 2개. 각 제언은 누가 / 무엇을 / 언제 + 기대 효과 형식</t>
   </si>
   <si>
     <t>7. 한계 및 후속 분석 제안 — 이 분석이 답하지 못한 것, 다음에 필요한 데이터</t>
@@ -1654,6 +1651,10 @@
   </si>
   <si>
     <t>폐업_률</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>6. 비즈니스 제언(Recommendation) — 최소 2개. 각 제언은 누가 / 무엇을 / 언제 + 기대 효과 형식</t>
     <phoneticPr fontId="1" type="noConversion"/>
   </si>
 </sst>
@@ -2246,30 +2247,39 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="12" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="12" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="2" fillId="2" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="2" borderId="14" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="12" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="12" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
@@ -2287,15 +2297,6 @@
     </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="17" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="0" borderId="12" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="6" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
@@ -2682,16 +2683,16 @@
   <sheetData>
     <row r="1" spans="1:4">
       <c r="A1" s="8" t="s">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="B1" s="9" t="s">
-        <v>76</v>
+        <v>75</v>
       </c>
       <c r="C1" s="9" t="s">
-        <v>48</v>
+        <v>47</v>
       </c>
       <c r="D1" s="9" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
     </row>
     <row r="2" spans="1:4">
@@ -2699,33 +2700,33 @@
         <v>0</v>
       </c>
       <c r="B2" s="28" t="s">
-        <v>77</v>
+        <v>76</v>
       </c>
       <c r="C2" s="24">
         <v>46254</v>
       </c>
       <c r="D2" s="23" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
     </row>
     <row r="3" spans="1:4">
       <c r="A3" s="21" t="s">
-        <v>83</v>
+        <v>82</v>
       </c>
       <c r="B3" s="28"/>
       <c r="C3" s="24">
         <v>46254</v>
       </c>
       <c r="D3" s="23" t="s">
-        <v>84</v>
+        <v>83</v>
       </c>
     </row>
     <row r="4" spans="1:4" ht="64">
       <c r="A4" s="21" t="s">
-        <v>49</v>
+        <v>48</v>
       </c>
       <c r="B4" s="19" t="s">
-        <v>54</v>
+        <v>53</v>
       </c>
       <c r="C4" s="24">
         <v>46254</v>
@@ -2734,22 +2735,22 @@
     </row>
     <row r="5" spans="1:4" ht="112">
       <c r="A5" s="22" t="s">
-        <v>50</v>
+        <v>49</v>
       </c>
       <c r="B5" s="20" t="s">
-        <v>60</v>
+        <v>59</v>
       </c>
       <c r="C5" s="24" t="s">
-        <v>82</v>
+        <v>81</v>
       </c>
       <c r="D5" s="23"/>
     </row>
     <row r="6" spans="1:4" ht="48">
       <c r="A6" s="22" t="s">
-        <v>51</v>
+        <v>50</v>
       </c>
       <c r="B6" s="20" t="s">
-        <v>55</v>
+        <v>54</v>
       </c>
       <c r="C6" s="30">
         <v>46255</v>
@@ -2758,10 +2759,10 @@
     </row>
     <row r="7" spans="1:4" ht="64">
       <c r="A7" s="22" t="s">
-        <v>52</v>
+        <v>51</v>
       </c>
       <c r="B7" s="20" t="s">
-        <v>56</v>
+        <v>55</v>
       </c>
       <c r="C7" s="30">
         <v>46258</v>
@@ -2770,10 +2771,10 @@
     </row>
     <row r="8" spans="1:4" ht="80">
       <c r="A8" s="22" t="s">
-        <v>53</v>
+        <v>52</v>
       </c>
       <c r="B8" s="20" t="s">
-        <v>57</v>
+        <v>56</v>
       </c>
       <c r="C8" s="30">
         <v>46258</v>
@@ -2782,10 +2783,10 @@
     </row>
     <row r="9" spans="1:4" ht="80">
       <c r="A9" s="22" t="s">
-        <v>59</v>
+        <v>58</v>
       </c>
       <c r="B9" s="20" t="s">
-        <v>58</v>
+        <v>57</v>
       </c>
       <c r="C9" s="30">
         <v>46259</v>
@@ -2794,7 +2795,7 @@
     </row>
     <row r="10" spans="1:4">
       <c r="A10" s="61" t="s">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="B10" s="62"/>
       <c r="C10" s="31">
@@ -2804,7 +2805,7 @@
     </row>
     <row r="11" spans="1:4">
       <c r="A11" s="61" t="s">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="B11" s="62"/>
       <c r="C11" s="31">
@@ -2839,31 +2840,31 @@
   <sheetData>
     <row r="1" spans="1:9">
       <c r="A1" s="13" t="s">
+        <v>18</v>
+      </c>
+      <c r="B1" s="13" t="s">
         <v>19</v>
       </c>
-      <c r="B1" s="13" t="s">
+      <c r="C1" s="13" t="s">
         <v>20</v>
       </c>
-      <c r="C1" s="13" t="s">
-        <v>21</v>
-      </c>
       <c r="D1" s="13" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="E1" s="14" t="s">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="F1" s="14" t="s">
+        <v>43</v>
+      </c>
+      <c r="G1" s="14" t="s">
         <v>44</v>
       </c>
-      <c r="G1" s="14" t="s">
+      <c r="H1" s="14" t="s">
         <v>45</v>
       </c>
-      <c r="H1" s="14" t="s">
+      <c r="I1" s="14" t="s">
         <v>46</v>
-      </c>
-      <c r="I1" s="14" t="s">
-        <v>47</v>
       </c>
     </row>
     <row r="2" spans="1:9" ht="51">
@@ -2871,19 +2872,19 @@
         <v>1</v>
       </c>
       <c r="B2" s="12" t="s">
+        <v>21</v>
+      </c>
+      <c r="C2" s="10" t="s">
         <v>22</v>
       </c>
-      <c r="C2" s="10" t="s">
-        <v>23</v>
-      </c>
       <c r="D2" s="10" t="s">
-        <v>35</v>
+        <v>34</v>
       </c>
       <c r="E2" s="4"/>
       <c r="F2" s="4"/>
       <c r="G2" s="15"/>
       <c r="H2" s="15" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="I2" s="4"/>
     </row>
@@ -2892,19 +2893,19 @@
         <v>2</v>
       </c>
       <c r="B3" s="12" t="s">
+        <v>23</v>
+      </c>
+      <c r="C3" s="10" t="s">
         <v>24</v>
       </c>
-      <c r="C3" s="10" t="s">
-        <v>25</v>
-      </c>
       <c r="D3" s="10" t="s">
-        <v>36</v>
+        <v>35</v>
       </c>
       <c r="E3" s="4"/>
       <c r="F3" s="4"/>
       <c r="G3" s="15"/>
       <c r="H3" s="15" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="I3" s="4"/>
     </row>
@@ -2913,18 +2914,18 @@
         <v>3</v>
       </c>
       <c r="B4" s="12" t="s">
-        <v>26</v>
+        <v>25</v>
       </c>
       <c r="C4" s="10" t="s">
-        <v>25</v>
+        <v>24</v>
       </c>
       <c r="D4" s="10" t="s">
-        <v>37</v>
+        <v>36</v>
       </c>
       <c r="E4" s="4"/>
       <c r="F4" s="4"/>
       <c r="G4" s="15" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="H4" s="4"/>
       <c r="I4" s="4"/>
@@ -2934,13 +2935,13 @@
         <v>4</v>
       </c>
       <c r="B5" s="12" t="s">
+        <v>26</v>
+      </c>
+      <c r="C5" s="10" t="s">
         <v>27</v>
       </c>
-      <c r="C5" s="10" t="s">
-        <v>28</v>
-      </c>
       <c r="D5" s="10" t="s">
-        <v>38</v>
+        <v>37</v>
       </c>
       <c r="E5" s="4"/>
       <c r="F5" s="4"/>
@@ -2953,17 +2954,17 @@
         <v>5</v>
       </c>
       <c r="B6" s="12" t="s">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="C6" s="10" t="s">
-        <v>28</v>
+        <v>27</v>
       </c>
       <c r="D6" s="10" t="s">
-        <v>39</v>
+        <v>38</v>
       </c>
       <c r="E6" s="4"/>
       <c r="F6" s="15" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="G6" s="4"/>
       <c r="H6" s="4"/>
@@ -2974,13 +2975,13 @@
         <v>6</v>
       </c>
       <c r="B7" s="12" t="s">
-        <v>30</v>
+        <v>29</v>
       </c>
       <c r="C7" s="10" t="s">
-        <v>28</v>
+        <v>27</v>
       </c>
       <c r="D7" s="10" t="s">
-        <v>40</v>
+        <v>39</v>
       </c>
       <c r="E7" s="4"/>
       <c r="F7" s="4"/>
@@ -2993,20 +2994,20 @@
         <v>7</v>
       </c>
       <c r="B8" s="12" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="C8" s="10" t="s">
-        <v>28</v>
+        <v>27</v>
       </c>
       <c r="D8" s="10" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="E8" s="15" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="F8" s="4"/>
       <c r="G8" s="15" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="H8" s="4"/>
       <c r="I8" s="4"/>
@@ -3016,25 +3017,25 @@
         <v>8</v>
       </c>
       <c r="B9" s="17" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="C9" s="18" t="s">
-        <v>28</v>
+        <v>27</v>
       </c>
       <c r="D9" s="18" t="s">
+        <v>41</v>
+      </c>
+      <c r="E9" s="15" t="s">
         <v>42</v>
       </c>
-      <c r="E9" s="15" t="s">
-        <v>43</v>
-      </c>
       <c r="F9" s="15" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="G9" s="15" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="H9" s="15" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="I9" s="4"/>
     </row>
@@ -3043,13 +3044,13 @@
         <v>9</v>
       </c>
       <c r="B10" s="12" t="s">
-        <v>16</v>
+        <v>15</v>
       </c>
       <c r="C10" s="10" t="s">
+        <v>30</v>
+      </c>
+      <c r="D10" s="10" t="s">
         <v>31</v>
-      </c>
-      <c r="D10" s="10" t="s">
-        <v>32</v>
       </c>
       <c r="E10" s="15"/>
       <c r="F10" s="4"/>
@@ -3062,19 +3063,19 @@
         <v>10</v>
       </c>
       <c r="B11" s="12" t="s">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="C11" s="10" t="s">
+        <v>32</v>
+      </c>
+      <c r="D11" s="10" t="s">
         <v>33</v>
       </c>
-      <c r="D11" s="10" t="s">
-        <v>34</v>
-      </c>
       <c r="E11" s="15" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="F11" s="15" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="G11" s="4"/>
       <c r="H11" s="4"/>
@@ -3110,71 +3111,71 @@
   <sheetData>
     <row r="1" spans="1:3">
       <c r="A1" s="8" t="s">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="B1" s="9" t="s">
-        <v>76</v>
+        <v>75</v>
       </c>
       <c r="C1" s="9" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
     </row>
     <row r="2" spans="1:3" ht="64">
       <c r="A2" s="32" t="s">
-        <v>49</v>
+        <v>48</v>
       </c>
       <c r="B2" s="19" t="s">
-        <v>54</v>
+        <v>53</v>
       </c>
       <c r="C2" s="2"/>
     </row>
     <row r="3" spans="1:3" ht="101.5" customHeight="1">
       <c r="A3" s="14" t="s">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="B3" s="25" t="s">
-        <v>80</v>
+        <v>79</v>
       </c>
       <c r="C3" s="33" t="s">
-        <v>93</v>
+        <v>92</v>
       </c>
     </row>
     <row r="4" spans="1:3" ht="299.5" customHeight="1">
       <c r="A4" s="14" t="s">
-        <v>44</v>
+        <v>43</v>
       </c>
       <c r="B4" s="29" t="s">
-        <v>78</v>
+        <v>77</v>
       </c>
       <c r="C4" s="33" t="s">
-        <v>87</v>
+        <v>86</v>
       </c>
     </row>
     <row r="5" spans="1:3" ht="409.6" customHeight="1">
       <c r="A5" s="14" t="s">
-        <v>45</v>
+        <v>44</v>
       </c>
       <c r="B5" s="29" t="s">
-        <v>79</v>
+        <v>78</v>
       </c>
       <c r="C5" s="33" t="s">
-        <v>86</v>
+        <v>85</v>
       </c>
     </row>
     <row r="6" spans="1:3" ht="287.5" customHeight="1">
       <c r="A6" s="14" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
       <c r="B6" s="19" t="s">
-        <v>81</v>
+        <v>80</v>
       </c>
       <c r="C6" s="25" t="s">
-        <v>85</v>
+        <v>84</v>
       </c>
     </row>
     <row r="7" spans="1:3" ht="101.5" customHeight="1">
       <c r="A7" s="14" t="s">
-        <v>47</v>
+        <v>46</v>
       </c>
       <c r="B7" s="19"/>
       <c r="C7" s="2"/>
@@ -3203,58 +3204,58 @@
   <sheetData>
     <row r="1" spans="1:3">
       <c r="A1" s="63" t="s">
-        <v>91</v>
+        <v>90</v>
       </c>
       <c r="B1" s="63"/>
       <c r="C1" s="63"/>
     </row>
     <row r="2" spans="1:3" ht="16.5" customHeight="1">
       <c r="A2" s="9" t="s">
-        <v>90</v>
+        <v>89</v>
       </c>
       <c r="B2" s="9" t="s">
-        <v>76</v>
+        <v>75</v>
       </c>
       <c r="C2" s="9" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
     </row>
     <row r="3" spans="1:3" ht="207.5" customHeight="1">
       <c r="A3" s="3" t="s">
-        <v>88</v>
+        <v>87</v>
       </c>
       <c r="B3" s="34" t="s">
-        <v>98</v>
+        <v>97</v>
       </c>
       <c r="C3" s="2"/>
     </row>
     <row r="4" spans="1:3" ht="25" customHeight="1">
       <c r="A4" s="3" t="s">
-        <v>94</v>
+        <v>93</v>
       </c>
       <c r="B4" s="34" t="s">
-        <v>96</v>
+        <v>95</v>
       </c>
       <c r="C4" s="2"/>
     </row>
     <row r="5" spans="1:3" ht="34">
       <c r="A5" s="3" t="s">
-        <v>95</v>
+        <v>94</v>
       </c>
       <c r="B5" s="34" t="s">
-        <v>100</v>
+        <v>99</v>
       </c>
       <c r="C5" s="2"/>
     </row>
     <row r="6" spans="1:3" ht="34">
       <c r="A6" s="3" t="s">
-        <v>89</v>
+        <v>88</v>
       </c>
       <c r="B6" s="36" t="s">
-        <v>99</v>
+        <v>98</v>
       </c>
       <c r="C6" s="34" t="s">
-        <v>102</v>
+        <v>101</v>
       </c>
     </row>
     <row r="7" spans="1:3" ht="294.5" customHeight="1">
@@ -3262,24 +3263,24 @@
         <v>0</v>
       </c>
       <c r="B7" s="35" t="s">
-        <v>101</v>
+        <v>100</v>
       </c>
       <c r="C7" s="29" t="s">
-        <v>103</v>
+        <v>102</v>
       </c>
     </row>
     <row r="8" spans="1:3" ht="138" customHeight="1">
       <c r="A8" s="3" t="s">
-        <v>97</v>
+        <v>96</v>
       </c>
       <c r="B8" s="37" t="s">
-        <v>207</v>
+        <v>206</v>
       </c>
       <c r="C8" s="2"/>
     </row>
     <row r="10" spans="1:3">
       <c r="A10" s="64" t="s">
-        <v>92</v>
+        <v>91</v>
       </c>
       <c r="B10" s="64"/>
       <c r="C10" s="64"/>
@@ -3325,2891 +3326,2891 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:7">
-      <c r="A1" s="66" t="s">
-        <v>104</v>
-      </c>
-      <c r="B1" s="66"/>
-      <c r="C1" s="66"/>
-      <c r="D1" s="66"/>
-      <c r="E1" s="66"/>
-      <c r="F1" s="66"/>
-      <c r="G1" s="67"/>
+      <c r="A1" s="75" t="s">
+        <v>103</v>
+      </c>
+      <c r="B1" s="75"/>
+      <c r="C1" s="75"/>
+      <c r="D1" s="75"/>
+      <c r="E1" s="75"/>
+      <c r="F1" s="75"/>
+      <c r="G1" s="76"/>
     </row>
     <row r="2" spans="1:7" ht="17.5" thickBot="1">
       <c r="A2" s="38" t="s">
-        <v>208</v>
+        <v>207</v>
       </c>
       <c r="B2" s="38" t="s">
+        <v>119</v>
+      </c>
+      <c r="C2" s="38" t="s">
+        <v>121</v>
+      </c>
+      <c r="D2" s="38" t="s">
+        <v>122</v>
+      </c>
+      <c r="E2" s="38" t="s">
         <v>120</v>
       </c>
-      <c r="C2" s="38" t="s">
-        <v>122</v>
-      </c>
-      <c r="D2" s="38" t="s">
-        <v>123</v>
-      </c>
-      <c r="E2" s="38" t="s">
-        <v>121</v>
-      </c>
       <c r="F2" s="38" t="s">
+        <v>125</v>
+      </c>
+      <c r="G2" s="38" t="s">
         <v>126</v>
       </c>
-      <c r="G2" s="38" t="s">
-        <v>127</v>
-      </c>
     </row>
     <row r="3" spans="1:7">
-      <c r="A3" s="68">
+      <c r="A3" s="69">
         <v>1</v>
       </c>
-      <c r="B3" s="71" t="s">
-        <v>105</v>
+      <c r="B3" s="72" t="s">
+        <v>104</v>
       </c>
       <c r="C3" s="39">
         <v>0</v>
       </c>
       <c r="D3" s="39" t="s">
-        <v>272</v>
+        <v>271</v>
       </c>
       <c r="E3" s="39">
         <v>3250</v>
       </c>
       <c r="F3" s="39" t="s">
-        <v>107</v>
+        <v>106</v>
       </c>
       <c r="G3" s="40" t="s">
-        <v>226</v>
+        <v>225</v>
       </c>
     </row>
     <row r="4" spans="1:7">
-      <c r="A4" s="69"/>
-      <c r="B4" s="72"/>
+      <c r="A4" s="70"/>
+      <c r="B4" s="73"/>
       <c r="C4" s="41">
         <v>1</v>
       </c>
       <c r="D4" s="41" t="s">
-        <v>108</v>
+        <v>107</v>
       </c>
       <c r="E4" s="41">
         <v>3250</v>
       </c>
       <c r="F4" s="41" t="s">
-        <v>107</v>
+        <v>106</v>
       </c>
       <c r="G4" s="42"/>
     </row>
     <row r="5" spans="1:7">
-      <c r="A5" s="69"/>
-      <c r="B5" s="72"/>
+      <c r="A5" s="70"/>
+      <c r="B5" s="73"/>
       <c r="C5" s="41">
         <v>2</v>
       </c>
       <c r="D5" s="41" t="s">
-        <v>109</v>
+        <v>108</v>
       </c>
       <c r="E5" s="41">
         <v>3250</v>
       </c>
       <c r="F5" s="41" t="s">
-        <v>110</v>
+        <v>109</v>
       </c>
       <c r="G5" s="42"/>
     </row>
     <row r="6" spans="1:7" ht="51">
-      <c r="A6" s="69"/>
-      <c r="B6" s="72"/>
+      <c r="A6" s="70"/>
+      <c r="B6" s="73"/>
       <c r="C6" s="41">
         <v>3</v>
       </c>
       <c r="D6" s="41" t="s">
-        <v>277</v>
+        <v>276</v>
       </c>
       <c r="E6" s="41">
         <v>3250</v>
       </c>
       <c r="F6" s="41" t="s">
-        <v>110</v>
+        <v>109</v>
       </c>
       <c r="G6" s="43" t="s">
-        <v>128</v>
+        <v>127</v>
       </c>
     </row>
     <row r="7" spans="1:7">
-      <c r="A7" s="69"/>
-      <c r="B7" s="72"/>
+      <c r="A7" s="70"/>
+      <c r="B7" s="73"/>
       <c r="C7" s="41">
         <v>4</v>
       </c>
       <c r="D7" s="41" t="s">
-        <v>112</v>
+        <v>111</v>
       </c>
       <c r="E7" s="41">
         <v>3250</v>
       </c>
       <c r="F7" s="41" t="s">
-        <v>110</v>
+        <v>109</v>
       </c>
       <c r="G7" s="42"/>
     </row>
     <row r="8" spans="1:7">
-      <c r="A8" s="69"/>
-      <c r="B8" s="72"/>
+      <c r="A8" s="70"/>
+      <c r="B8" s="73"/>
       <c r="C8" s="41">
         <v>5</v>
       </c>
       <c r="D8" s="41" t="s">
-        <v>113</v>
+        <v>112</v>
       </c>
       <c r="E8" s="41">
         <v>3250</v>
       </c>
       <c r="F8" s="41" t="s">
-        <v>107</v>
+        <v>106</v>
       </c>
       <c r="G8" s="42" t="s">
-        <v>130</v>
+        <v>129</v>
       </c>
     </row>
     <row r="9" spans="1:7">
-      <c r="A9" s="69"/>
-      <c r="B9" s="72"/>
+      <c r="A9" s="70"/>
+      <c r="B9" s="73"/>
       <c r="C9" s="41">
         <v>6</v>
       </c>
       <c r="D9" s="41" t="s">
-        <v>114</v>
+        <v>113</v>
       </c>
       <c r="E9" s="41">
         <v>3250</v>
       </c>
       <c r="F9" s="41" t="s">
-        <v>107</v>
+        <v>106</v>
       </c>
       <c r="G9" s="42"/>
     </row>
     <row r="10" spans="1:7">
-      <c r="A10" s="69"/>
-      <c r="B10" s="72"/>
+      <c r="A10" s="70"/>
+      <c r="B10" s="73"/>
       <c r="C10" s="41">
         <v>7</v>
       </c>
       <c r="D10" s="41" t="s">
-        <v>129</v>
+        <v>128</v>
       </c>
       <c r="E10" s="41">
         <v>3250</v>
       </c>
       <c r="F10" s="41" t="s">
-        <v>107</v>
+        <v>106</v>
       </c>
       <c r="G10" s="42"/>
     </row>
     <row r="11" spans="1:7">
-      <c r="A11" s="69"/>
-      <c r="B11" s="72"/>
+      <c r="A11" s="70"/>
+      <c r="B11" s="73"/>
       <c r="C11" s="41">
         <v>8</v>
       </c>
       <c r="D11" s="41" t="s">
-        <v>116</v>
+        <v>115</v>
       </c>
       <c r="E11" s="41">
         <v>3250</v>
       </c>
       <c r="F11" s="41" t="s">
-        <v>117</v>
+        <v>116</v>
       </c>
       <c r="G11" s="42" t="s">
-        <v>267</v>
+        <v>266</v>
       </c>
     </row>
     <row r="12" spans="1:7">
-      <c r="A12" s="69"/>
-      <c r="B12" s="72"/>
+      <c r="A12" s="70"/>
+      <c r="B12" s="73"/>
       <c r="C12" s="41">
         <v>9</v>
       </c>
       <c r="D12" s="41" t="s">
-        <v>118</v>
+        <v>117</v>
       </c>
       <c r="E12" s="41">
         <v>3250</v>
       </c>
       <c r="F12" s="41" t="s">
-        <v>107</v>
+        <v>106</v>
       </c>
       <c r="G12" s="42"/>
     </row>
     <row r="13" spans="1:7">
-      <c r="A13" s="69"/>
-      <c r="B13" s="72"/>
+      <c r="A13" s="70"/>
+      <c r="B13" s="73"/>
       <c r="C13" s="41">
         <v>10</v>
       </c>
       <c r="D13" s="41" t="s">
-        <v>119</v>
+        <v>118</v>
       </c>
       <c r="E13" s="41">
         <v>3250</v>
       </c>
       <c r="F13" s="41" t="s">
-        <v>117</v>
+        <v>116</v>
       </c>
       <c r="G13" s="42" t="s">
-        <v>268</v>
+        <v>267</v>
       </c>
     </row>
     <row r="14" spans="1:7" ht="17.5" thickBot="1">
-      <c r="A14" s="70"/>
-      <c r="B14" s="73"/>
+      <c r="A14" s="71"/>
+      <c r="B14" s="74"/>
       <c r="C14" s="44">
         <v>11</v>
       </c>
       <c r="D14" s="44" t="s">
-        <v>125</v>
+        <v>124</v>
       </c>
       <c r="E14" s="44">
         <v>3250</v>
       </c>
       <c r="F14" s="44" t="s">
-        <v>107</v>
+        <v>106</v>
       </c>
       <c r="G14" s="45"/>
     </row>
     <row r="15" spans="1:7">
-      <c r="A15" s="77">
+      <c r="A15" s="80">
         <v>2</v>
       </c>
-      <c r="B15" s="74" t="s">
-        <v>179</v>
+      <c r="B15" s="77" t="s">
+        <v>178</v>
       </c>
       <c r="C15" s="54">
         <v>0</v>
       </c>
       <c r="D15" s="54" t="s">
-        <v>106</v>
+        <v>105</v>
       </c>
       <c r="E15" s="46">
         <v>3250</v>
       </c>
       <c r="F15" s="46" t="s">
-        <v>107</v>
+        <v>106</v>
       </c>
       <c r="G15" s="40" t="s">
-        <v>226</v>
+        <v>225</v>
       </c>
     </row>
     <row r="16" spans="1:7">
-      <c r="A16" s="78"/>
-      <c r="B16" s="75"/>
+      <c r="A16" s="81"/>
+      <c r="B16" s="78"/>
       <c r="C16" s="55">
         <v>1</v>
       </c>
       <c r="D16" s="55" t="s">
-        <v>108</v>
+        <v>107</v>
       </c>
       <c r="E16" s="47">
         <v>3250</v>
       </c>
       <c r="F16" s="47" t="s">
-        <v>107</v>
+        <v>106</v>
       </c>
       <c r="G16" s="48"/>
     </row>
     <row r="17" spans="1:7">
-      <c r="A17" s="78"/>
-      <c r="B17" s="75"/>
+      <c r="A17" s="81"/>
+      <c r="B17" s="78"/>
       <c r="C17" s="55">
         <v>2</v>
       </c>
       <c r="D17" s="55" t="s">
-        <v>109</v>
+        <v>108</v>
       </c>
       <c r="E17" s="47">
         <v>3250</v>
       </c>
       <c r="F17" s="47" t="s">
-        <v>110</v>
+        <v>109</v>
       </c>
       <c r="G17" s="48"/>
     </row>
     <row r="18" spans="1:7" ht="51">
-      <c r="A18" s="78"/>
-      <c r="B18" s="75"/>
+      <c r="A18" s="81"/>
+      <c r="B18" s="78"/>
       <c r="C18" s="55">
         <v>3</v>
       </c>
       <c r="D18" s="55" t="s">
-        <v>111</v>
+        <v>110</v>
       </c>
       <c r="E18" s="47">
         <v>3250</v>
       </c>
       <c r="F18" s="47" t="s">
-        <v>110</v>
+        <v>109</v>
       </c>
       <c r="G18" s="49" t="s">
-        <v>128</v>
+        <v>127</v>
       </c>
     </row>
     <row r="19" spans="1:7">
-      <c r="A19" s="78"/>
-      <c r="B19" s="75"/>
+      <c r="A19" s="81"/>
+      <c r="B19" s="78"/>
       <c r="C19" s="55">
         <v>4</v>
       </c>
       <c r="D19" s="55" t="s">
-        <v>112</v>
+        <v>111</v>
       </c>
       <c r="E19" s="47">
         <v>3250</v>
       </c>
       <c r="F19" s="47" t="s">
-        <v>110</v>
+        <v>109</v>
       </c>
       <c r="G19" s="48"/>
     </row>
     <row r="20" spans="1:7">
-      <c r="A20" s="78"/>
-      <c r="B20" s="75"/>
+      <c r="A20" s="81"/>
+      <c r="B20" s="78"/>
       <c r="C20" s="55">
         <v>5</v>
       </c>
       <c r="D20" s="55" t="s">
-        <v>131</v>
+        <v>130</v>
       </c>
       <c r="E20" s="47">
         <v>3250</v>
       </c>
       <c r="F20" s="47" t="s">
-        <v>107</v>
+        <v>106</v>
       </c>
       <c r="G20" s="48" t="s">
-        <v>180</v>
+        <v>179</v>
       </c>
     </row>
     <row r="21" spans="1:7">
-      <c r="A21" s="78"/>
-      <c r="B21" s="75"/>
+      <c r="A21" s="81"/>
+      <c r="B21" s="78"/>
       <c r="C21" s="55">
         <v>6</v>
       </c>
       <c r="D21" s="55" t="s">
-        <v>132</v>
+        <v>131</v>
       </c>
       <c r="E21" s="47">
         <v>3250</v>
       </c>
       <c r="F21" s="47" t="s">
-        <v>107</v>
+        <v>106</v>
       </c>
       <c r="G21" s="48" t="s">
-        <v>263</v>
+        <v>262</v>
       </c>
     </row>
     <row r="22" spans="1:7">
-      <c r="A22" s="78"/>
-      <c r="B22" s="75"/>
+      <c r="A22" s="81"/>
+      <c r="B22" s="78"/>
       <c r="C22" s="55">
         <v>7</v>
       </c>
       <c r="D22" s="55" t="s">
-        <v>133</v>
+        <v>132</v>
       </c>
       <c r="E22" s="47">
         <v>3250</v>
       </c>
       <c r="F22" s="47" t="s">
-        <v>107</v>
+        <v>106</v>
       </c>
       <c r="G22" s="48"/>
     </row>
     <row r="23" spans="1:7">
-      <c r="A23" s="78"/>
-      <c r="B23" s="75"/>
+      <c r="A23" s="81"/>
+      <c r="B23" s="78"/>
       <c r="C23" s="55">
         <v>8</v>
       </c>
       <c r="D23" s="55" t="s">
-        <v>134</v>
+        <v>133</v>
       </c>
       <c r="E23" s="47">
         <v>3250</v>
       </c>
       <c r="F23" s="47" t="s">
-        <v>107</v>
+        <v>106</v>
       </c>
       <c r="G23" s="48"/>
     </row>
     <row r="24" spans="1:7">
-      <c r="A24" s="78"/>
-      <c r="B24" s="75"/>
+      <c r="A24" s="81"/>
+      <c r="B24" s="78"/>
       <c r="C24" s="55">
         <v>9</v>
       </c>
       <c r="D24" s="55" t="s">
-        <v>135</v>
+        <v>134</v>
       </c>
       <c r="E24" s="47">
         <v>3250</v>
       </c>
       <c r="F24" s="47" t="s">
-        <v>107</v>
+        <v>106</v>
       </c>
       <c r="G24" s="48"/>
     </row>
     <row r="25" spans="1:7">
-      <c r="A25" s="78"/>
-      <c r="B25" s="75"/>
+      <c r="A25" s="81"/>
+      <c r="B25" s="78"/>
       <c r="C25" s="55">
         <v>10</v>
       </c>
       <c r="D25" s="55" t="s">
-        <v>136</v>
+        <v>135</v>
       </c>
       <c r="E25" s="47">
         <v>3250</v>
       </c>
       <c r="F25" s="47" t="s">
-        <v>107</v>
+        <v>106</v>
       </c>
       <c r="G25" s="48"/>
     </row>
     <row r="26" spans="1:7">
-      <c r="A26" s="78"/>
-      <c r="B26" s="75"/>
+      <c r="A26" s="81"/>
+      <c r="B26" s="78"/>
       <c r="C26" s="55">
         <v>11</v>
       </c>
       <c r="D26" s="55" t="s">
-        <v>137</v>
+        <v>136</v>
       </c>
       <c r="E26" s="47">
         <v>3250</v>
       </c>
       <c r="F26" s="47" t="s">
-        <v>107</v>
+        <v>106</v>
       </c>
       <c r="G26" s="48"/>
     </row>
     <row r="27" spans="1:7">
-      <c r="A27" s="78"/>
-      <c r="B27" s="75"/>
+      <c r="A27" s="81"/>
+      <c r="B27" s="78"/>
       <c r="C27" s="55">
         <v>12</v>
       </c>
       <c r="D27" s="55" t="s">
-        <v>138</v>
+        <v>137</v>
       </c>
       <c r="E27" s="47">
         <v>3250</v>
       </c>
       <c r="F27" s="47" t="s">
-        <v>107</v>
+        <v>106</v>
       </c>
       <c r="G27" s="48"/>
     </row>
     <row r="28" spans="1:7">
-      <c r="A28" s="78"/>
-      <c r="B28" s="75"/>
+      <c r="A28" s="81"/>
+      <c r="B28" s="78"/>
       <c r="C28" s="55">
         <v>13</v>
       </c>
       <c r="D28" s="55" t="s">
-        <v>139</v>
+        <v>138</v>
       </c>
       <c r="E28" s="47">
         <v>3250</v>
       </c>
       <c r="F28" s="47" t="s">
-        <v>107</v>
+        <v>106</v>
       </c>
       <c r="G28" s="48"/>
     </row>
     <row r="29" spans="1:7">
-      <c r="A29" s="78"/>
-      <c r="B29" s="75"/>
+      <c r="A29" s="81"/>
+      <c r="B29" s="78"/>
       <c r="C29" s="55">
         <v>14</v>
       </c>
       <c r="D29" s="55" t="s">
-        <v>140</v>
+        <v>139</v>
       </c>
       <c r="E29" s="47">
         <v>3250</v>
       </c>
       <c r="F29" s="47" t="s">
-        <v>107</v>
+        <v>106</v>
       </c>
       <c r="G29" s="48"/>
     </row>
     <row r="30" spans="1:7">
-      <c r="A30" s="78"/>
-      <c r="B30" s="75"/>
+      <c r="A30" s="81"/>
+      <c r="B30" s="78"/>
       <c r="C30" s="55">
         <v>15</v>
       </c>
       <c r="D30" s="55" t="s">
-        <v>141</v>
+        <v>140</v>
       </c>
       <c r="E30" s="47">
         <v>3250</v>
       </c>
       <c r="F30" s="47" t="s">
-        <v>107</v>
+        <v>106</v>
       </c>
       <c r="G30" s="48"/>
     </row>
     <row r="31" spans="1:7">
-      <c r="A31" s="78"/>
-      <c r="B31" s="75"/>
+      <c r="A31" s="81"/>
+      <c r="B31" s="78"/>
       <c r="C31" s="55">
         <v>16</v>
       </c>
       <c r="D31" s="55" t="s">
-        <v>142</v>
+        <v>141</v>
       </c>
       <c r="E31" s="47">
         <v>3250</v>
       </c>
       <c r="F31" s="47" t="s">
-        <v>107</v>
+        <v>106</v>
       </c>
       <c r="G31" s="48"/>
     </row>
     <row r="32" spans="1:7">
-      <c r="A32" s="78"/>
-      <c r="B32" s="75"/>
+      <c r="A32" s="81"/>
+      <c r="B32" s="78"/>
       <c r="C32" s="55">
         <v>17</v>
       </c>
       <c r="D32" s="55" t="s">
-        <v>143</v>
+        <v>142</v>
       </c>
       <c r="E32" s="47">
         <v>3250</v>
       </c>
       <c r="F32" s="47" t="s">
-        <v>107</v>
+        <v>106</v>
       </c>
       <c r="G32" s="48"/>
     </row>
     <row r="33" spans="1:7">
-      <c r="A33" s="78"/>
-      <c r="B33" s="75"/>
+      <c r="A33" s="81"/>
+      <c r="B33" s="78"/>
       <c r="C33" s="55">
         <v>18</v>
       </c>
       <c r="D33" s="55" t="s">
-        <v>144</v>
+        <v>143</v>
       </c>
       <c r="E33" s="47">
         <v>3250</v>
       </c>
       <c r="F33" s="47" t="s">
-        <v>107</v>
+        <v>106</v>
       </c>
       <c r="G33" s="48" t="s">
-        <v>206</v>
+        <v>205</v>
       </c>
     </row>
     <row r="34" spans="1:7">
-      <c r="A34" s="78"/>
-      <c r="B34" s="75"/>
+      <c r="A34" s="81"/>
+      <c r="B34" s="78"/>
       <c r="C34" s="55">
         <v>19</v>
       </c>
       <c r="D34" s="55" t="s">
-        <v>145</v>
+        <v>144</v>
       </c>
       <c r="E34" s="47">
         <v>3250</v>
       </c>
       <c r="F34" s="47" t="s">
-        <v>107</v>
+        <v>106</v>
       </c>
       <c r="G34" s="48"/>
     </row>
     <row r="35" spans="1:7">
-      <c r="A35" s="78"/>
-      <c r="B35" s="75"/>
+      <c r="A35" s="81"/>
+      <c r="B35" s="78"/>
       <c r="C35" s="55">
         <v>20</v>
       </c>
       <c r="D35" s="55" t="s">
-        <v>146</v>
+        <v>145</v>
       </c>
       <c r="E35" s="47">
         <v>3250</v>
       </c>
       <c r="F35" s="47" t="s">
-        <v>107</v>
+        <v>106</v>
       </c>
       <c r="G35" s="48"/>
     </row>
     <row r="36" spans="1:7">
-      <c r="A36" s="78"/>
-      <c r="B36" s="75"/>
+      <c r="A36" s="81"/>
+      <c r="B36" s="78"/>
       <c r="C36" s="55">
         <v>21</v>
       </c>
       <c r="D36" s="55" t="s">
-        <v>147</v>
+        <v>146</v>
       </c>
       <c r="E36" s="47">
         <v>3250</v>
       </c>
       <c r="F36" s="47" t="s">
-        <v>107</v>
+        <v>106</v>
       </c>
       <c r="G36" s="48"/>
     </row>
     <row r="37" spans="1:7">
-      <c r="A37" s="78"/>
-      <c r="B37" s="75"/>
+      <c r="A37" s="81"/>
+      <c r="B37" s="78"/>
       <c r="C37" s="55">
         <v>22</v>
       </c>
       <c r="D37" s="55" t="s">
-        <v>148</v>
+        <v>147</v>
       </c>
       <c r="E37" s="47">
         <v>3250</v>
       </c>
       <c r="F37" s="47" t="s">
-        <v>107</v>
+        <v>106</v>
       </c>
       <c r="G37" s="48"/>
     </row>
     <row r="38" spans="1:7">
-      <c r="A38" s="78"/>
-      <c r="B38" s="75"/>
+      <c r="A38" s="81"/>
+      <c r="B38" s="78"/>
       <c r="C38" s="55">
         <v>23</v>
       </c>
       <c r="D38" s="55" t="s">
-        <v>149</v>
+        <v>148</v>
       </c>
       <c r="E38" s="47">
         <v>3250</v>
       </c>
       <c r="F38" s="47" t="s">
-        <v>107</v>
+        <v>106</v>
       </c>
       <c r="G38" s="48"/>
     </row>
     <row r="39" spans="1:7">
-      <c r="A39" s="78"/>
-      <c r="B39" s="75"/>
+      <c r="A39" s="81"/>
+      <c r="B39" s="78"/>
       <c r="C39" s="55">
         <v>24</v>
       </c>
       <c r="D39" s="55" t="s">
-        <v>150</v>
+        <v>149</v>
       </c>
       <c r="E39" s="47">
         <v>3250</v>
       </c>
       <c r="F39" s="47" t="s">
-        <v>107</v>
+        <v>106</v>
       </c>
       <c r="G39" s="48"/>
     </row>
     <row r="40" spans="1:7">
-      <c r="A40" s="78"/>
-      <c r="B40" s="75"/>
+      <c r="A40" s="81"/>
+      <c r="B40" s="78"/>
       <c r="C40" s="55">
         <v>25</v>
       </c>
       <c r="D40" s="55" t="s">
-        <v>151</v>
+        <v>150</v>
       </c>
       <c r="E40" s="47">
         <v>3250</v>
       </c>
       <c r="F40" s="47" t="s">
-        <v>107</v>
+        <v>106</v>
       </c>
       <c r="G40" s="48"/>
     </row>
     <row r="41" spans="1:7">
-      <c r="A41" s="78"/>
-      <c r="B41" s="75"/>
+      <c r="A41" s="81"/>
+      <c r="B41" s="78"/>
       <c r="C41" s="55">
         <v>26</v>
       </c>
       <c r="D41" s="55" t="s">
-        <v>152</v>
+        <v>151</v>
       </c>
       <c r="E41" s="47">
         <v>3250</v>
       </c>
       <c r="F41" s="47" t="s">
-        <v>107</v>
+        <v>106</v>
       </c>
       <c r="G41" s="48"/>
     </row>
     <row r="42" spans="1:7">
-      <c r="A42" s="78"/>
-      <c r="B42" s="75"/>
+      <c r="A42" s="81"/>
+      <c r="B42" s="78"/>
       <c r="C42" s="55">
         <v>27</v>
       </c>
       <c r="D42" s="55" t="s">
-        <v>153</v>
+        <v>152</v>
       </c>
       <c r="E42" s="47">
         <v>3250</v>
       </c>
       <c r="F42" s="47" t="s">
-        <v>107</v>
+        <v>106</v>
       </c>
       <c r="G42" s="48"/>
     </row>
     <row r="43" spans="1:7">
-      <c r="A43" s="78"/>
-      <c r="B43" s="75"/>
+      <c r="A43" s="81"/>
+      <c r="B43" s="78"/>
       <c r="C43" s="55">
         <v>28</v>
       </c>
       <c r="D43" s="55" t="s">
-        <v>154</v>
+        <v>153</v>
       </c>
       <c r="E43" s="47">
         <v>3250</v>
       </c>
       <c r="F43" s="47" t="s">
-        <v>107</v>
+        <v>106</v>
       </c>
       <c r="G43" s="48"/>
     </row>
     <row r="44" spans="1:7">
-      <c r="A44" s="78"/>
-      <c r="B44" s="75"/>
+      <c r="A44" s="81"/>
+      <c r="B44" s="78"/>
       <c r="C44" s="55">
         <v>29</v>
       </c>
       <c r="D44" s="55" t="s">
-        <v>155</v>
+        <v>154</v>
       </c>
       <c r="E44" s="47">
         <v>3250</v>
       </c>
       <c r="F44" s="47" t="s">
-        <v>107</v>
+        <v>106</v>
       </c>
       <c r="G44" s="48"/>
     </row>
     <row r="45" spans="1:7">
-      <c r="A45" s="78"/>
-      <c r="B45" s="75"/>
+      <c r="A45" s="81"/>
+      <c r="B45" s="78"/>
       <c r="C45" s="55">
         <v>30</v>
       </c>
       <c r="D45" s="55" t="s">
-        <v>156</v>
+        <v>155</v>
       </c>
       <c r="E45" s="47">
         <v>3250</v>
       </c>
       <c r="F45" s="47" t="s">
-        <v>107</v>
+        <v>106</v>
       </c>
       <c r="G45" s="48"/>
     </row>
     <row r="46" spans="1:7">
-      <c r="A46" s="78"/>
-      <c r="B46" s="75"/>
+      <c r="A46" s="81"/>
+      <c r="B46" s="78"/>
       <c r="C46" s="55">
         <v>31</v>
       </c>
       <c r="D46" s="55" t="s">
-        <v>157</v>
+        <v>156</v>
       </c>
       <c r="E46" s="47">
         <v>3250</v>
       </c>
       <c r="F46" s="47" t="s">
-        <v>107</v>
+        <v>106</v>
       </c>
       <c r="G46" s="48"/>
     </row>
     <row r="47" spans="1:7">
-      <c r="A47" s="78"/>
-      <c r="B47" s="75"/>
+      <c r="A47" s="81"/>
+      <c r="B47" s="78"/>
       <c r="C47" s="55">
         <v>32</v>
       </c>
       <c r="D47" s="55" t="s">
-        <v>158</v>
+        <v>157</v>
       </c>
       <c r="E47" s="47">
         <v>3250</v>
       </c>
       <c r="F47" s="47" t="s">
-        <v>107</v>
+        <v>106</v>
       </c>
       <c r="G47" s="48"/>
     </row>
     <row r="48" spans="1:7">
-      <c r="A48" s="78"/>
-      <c r="B48" s="75"/>
+      <c r="A48" s="81"/>
+      <c r="B48" s="78"/>
       <c r="C48" s="55">
         <v>33</v>
       </c>
       <c r="D48" s="55" t="s">
-        <v>159</v>
+        <v>158</v>
       </c>
       <c r="E48" s="47">
         <v>3250</v>
       </c>
       <c r="F48" s="47" t="s">
-        <v>107</v>
+        <v>106</v>
       </c>
       <c r="G48" s="48"/>
     </row>
     <row r="49" spans="1:7">
-      <c r="A49" s="78"/>
-      <c r="B49" s="75"/>
+      <c r="A49" s="81"/>
+      <c r="B49" s="78"/>
       <c r="C49" s="55">
         <v>34</v>
       </c>
       <c r="D49" s="55" t="s">
-        <v>160</v>
+        <v>159</v>
       </c>
       <c r="E49" s="47">
         <v>3250</v>
       </c>
       <c r="F49" s="47" t="s">
-        <v>107</v>
+        <v>106</v>
       </c>
       <c r="G49" s="48"/>
     </row>
     <row r="50" spans="1:7">
-      <c r="A50" s="78"/>
-      <c r="B50" s="75"/>
+      <c r="A50" s="81"/>
+      <c r="B50" s="78"/>
       <c r="C50" s="55">
         <v>35</v>
       </c>
       <c r="D50" s="55" t="s">
-        <v>161</v>
+        <v>160</v>
       </c>
       <c r="E50" s="47">
         <v>3250</v>
       </c>
       <c r="F50" s="47" t="s">
-        <v>107</v>
+        <v>106</v>
       </c>
       <c r="G50" s="48"/>
     </row>
     <row r="51" spans="1:7">
-      <c r="A51" s="78"/>
-      <c r="B51" s="75"/>
+      <c r="A51" s="81"/>
+      <c r="B51" s="78"/>
       <c r="C51" s="55">
         <v>36</v>
       </c>
       <c r="D51" s="55" t="s">
-        <v>162</v>
+        <v>161</v>
       </c>
       <c r="E51" s="47">
         <v>3250</v>
       </c>
       <c r="F51" s="47" t="s">
-        <v>107</v>
+        <v>106</v>
       </c>
       <c r="G51" s="48"/>
     </row>
     <row r="52" spans="1:7">
-      <c r="A52" s="78"/>
-      <c r="B52" s="75"/>
+      <c r="A52" s="81"/>
+      <c r="B52" s="78"/>
       <c r="C52" s="55">
         <v>37</v>
       </c>
       <c r="D52" s="55" t="s">
-        <v>163</v>
+        <v>162</v>
       </c>
       <c r="E52" s="47">
         <v>3250</v>
       </c>
       <c r="F52" s="47" t="s">
-        <v>107</v>
+        <v>106</v>
       </c>
       <c r="G52" s="48"/>
     </row>
     <row r="53" spans="1:7">
-      <c r="A53" s="78"/>
-      <c r="B53" s="75"/>
+      <c r="A53" s="81"/>
+      <c r="B53" s="78"/>
       <c r="C53" s="55">
         <v>38</v>
       </c>
       <c r="D53" s="55" t="s">
-        <v>164</v>
+        <v>163</v>
       </c>
       <c r="E53" s="47">
         <v>3250</v>
       </c>
       <c r="F53" s="47" t="s">
-        <v>107</v>
+        <v>106</v>
       </c>
       <c r="G53" s="48"/>
     </row>
     <row r="54" spans="1:7">
-      <c r="A54" s="78"/>
-      <c r="B54" s="75"/>
+      <c r="A54" s="81"/>
+      <c r="B54" s="78"/>
       <c r="C54" s="55">
         <v>39</v>
       </c>
       <c r="D54" s="55" t="s">
-        <v>165</v>
+        <v>164</v>
       </c>
       <c r="E54" s="47">
         <v>3250</v>
       </c>
       <c r="F54" s="47" t="s">
-        <v>107</v>
+        <v>106</v>
       </c>
       <c r="G54" s="48"/>
     </row>
     <row r="55" spans="1:7">
-      <c r="A55" s="78"/>
-      <c r="B55" s="75"/>
+      <c r="A55" s="81"/>
+      <c r="B55" s="78"/>
       <c r="C55" s="55">
         <v>40</v>
       </c>
       <c r="D55" s="55" t="s">
-        <v>166</v>
+        <v>165</v>
       </c>
       <c r="E55" s="47">
         <v>3250</v>
       </c>
       <c r="F55" s="47" t="s">
-        <v>107</v>
+        <v>106</v>
       </c>
       <c r="G55" s="48"/>
     </row>
     <row r="56" spans="1:7">
-      <c r="A56" s="78"/>
-      <c r="B56" s="75"/>
+      <c r="A56" s="81"/>
+      <c r="B56" s="78"/>
       <c r="C56" s="55">
         <v>41</v>
       </c>
       <c r="D56" s="55" t="s">
-        <v>167</v>
+        <v>166</v>
       </c>
       <c r="E56" s="47">
         <v>3250</v>
       </c>
       <c r="F56" s="47" t="s">
-        <v>107</v>
+        <v>106</v>
       </c>
       <c r="G56" s="48"/>
     </row>
     <row r="57" spans="1:7">
-      <c r="A57" s="78"/>
-      <c r="B57" s="75"/>
+      <c r="A57" s="81"/>
+      <c r="B57" s="78"/>
       <c r="C57" s="55">
         <v>42</v>
       </c>
       <c r="D57" s="55" t="s">
-        <v>168</v>
+        <v>167</v>
       </c>
       <c r="E57" s="47">
         <v>3250</v>
       </c>
       <c r="F57" s="47" t="s">
-        <v>107</v>
+        <v>106</v>
       </c>
       <c r="G57" s="48"/>
     </row>
     <row r="58" spans="1:7">
-      <c r="A58" s="78"/>
-      <c r="B58" s="75"/>
+      <c r="A58" s="81"/>
+      <c r="B58" s="78"/>
       <c r="C58" s="55">
         <v>43</v>
       </c>
       <c r="D58" s="55" t="s">
-        <v>169</v>
+        <v>168</v>
       </c>
       <c r="E58" s="47">
         <v>3250</v>
       </c>
       <c r="F58" s="47" t="s">
-        <v>107</v>
+        <v>106</v>
       </c>
       <c r="G58" s="48"/>
     </row>
     <row r="59" spans="1:7">
-      <c r="A59" s="78"/>
-      <c r="B59" s="75"/>
+      <c r="A59" s="81"/>
+      <c r="B59" s="78"/>
       <c r="C59" s="55">
         <v>44</v>
       </c>
       <c r="D59" s="55" t="s">
-        <v>170</v>
+        <v>169</v>
       </c>
       <c r="E59" s="47">
         <v>3250</v>
       </c>
       <c r="F59" s="47" t="s">
-        <v>107</v>
+        <v>106</v>
       </c>
       <c r="G59" s="48"/>
     </row>
     <row r="60" spans="1:7">
-      <c r="A60" s="78"/>
-      <c r="B60" s="75"/>
+      <c r="A60" s="81"/>
+      <c r="B60" s="78"/>
       <c r="C60" s="55">
         <v>45</v>
       </c>
       <c r="D60" s="55" t="s">
-        <v>171</v>
+        <v>170</v>
       </c>
       <c r="E60" s="47">
         <v>3250</v>
       </c>
       <c r="F60" s="47" t="s">
-        <v>107</v>
+        <v>106</v>
       </c>
       <c r="G60" s="48"/>
     </row>
     <row r="61" spans="1:7">
-      <c r="A61" s="78"/>
-      <c r="B61" s="75"/>
+      <c r="A61" s="81"/>
+      <c r="B61" s="78"/>
       <c r="C61" s="55">
         <v>46</v>
       </c>
       <c r="D61" s="55" t="s">
-        <v>172</v>
+        <v>171</v>
       </c>
       <c r="E61" s="47">
         <v>3250</v>
       </c>
       <c r="F61" s="47" t="s">
-        <v>107</v>
+        <v>106</v>
       </c>
       <c r="G61" s="48"/>
     </row>
     <row r="62" spans="1:7">
-      <c r="A62" s="78"/>
-      <c r="B62" s="75"/>
+      <c r="A62" s="81"/>
+      <c r="B62" s="78"/>
       <c r="C62" s="55">
         <v>47</v>
       </c>
       <c r="D62" s="55" t="s">
-        <v>173</v>
+        <v>172</v>
       </c>
       <c r="E62" s="47">
         <v>3250</v>
       </c>
       <c r="F62" s="47" t="s">
-        <v>107</v>
+        <v>106</v>
       </c>
       <c r="G62" s="48"/>
     </row>
     <row r="63" spans="1:7">
-      <c r="A63" s="78"/>
-      <c r="B63" s="75"/>
+      <c r="A63" s="81"/>
+      <c r="B63" s="78"/>
       <c r="C63" s="55">
         <v>48</v>
       </c>
       <c r="D63" s="55" t="s">
-        <v>174</v>
+        <v>173</v>
       </c>
       <c r="E63" s="47">
         <v>3250</v>
       </c>
       <c r="F63" s="47" t="s">
-        <v>107</v>
+        <v>106</v>
       </c>
       <c r="G63" s="48"/>
     </row>
     <row r="64" spans="1:7">
-      <c r="A64" s="78"/>
-      <c r="B64" s="75"/>
+      <c r="A64" s="81"/>
+      <c r="B64" s="78"/>
       <c r="C64" s="55">
         <v>49</v>
       </c>
       <c r="D64" s="55" t="s">
-        <v>175</v>
+        <v>174</v>
       </c>
       <c r="E64" s="47">
         <v>3250</v>
       </c>
       <c r="F64" s="47" t="s">
-        <v>107</v>
+        <v>106</v>
       </c>
       <c r="G64" s="48"/>
     </row>
     <row r="65" spans="1:7">
-      <c r="A65" s="78"/>
-      <c r="B65" s="75"/>
+      <c r="A65" s="81"/>
+      <c r="B65" s="78"/>
       <c r="C65" s="55">
         <v>50</v>
       </c>
       <c r="D65" s="55" t="s">
-        <v>176</v>
+        <v>175</v>
       </c>
       <c r="E65" s="47">
         <v>3250</v>
       </c>
       <c r="F65" s="47" t="s">
-        <v>107</v>
+        <v>106</v>
       </c>
       <c r="G65" s="48"/>
     </row>
     <row r="66" spans="1:7">
-      <c r="A66" s="78"/>
-      <c r="B66" s="75"/>
+      <c r="A66" s="81"/>
+      <c r="B66" s="78"/>
       <c r="C66" s="55">
         <v>51</v>
       </c>
       <c r="D66" s="55" t="s">
-        <v>177</v>
+        <v>176</v>
       </c>
       <c r="E66" s="47">
         <v>3250</v>
       </c>
       <c r="F66" s="47" t="s">
-        <v>107</v>
+        <v>106</v>
       </c>
       <c r="G66" s="48"/>
     </row>
     <row r="67" spans="1:7" ht="17.5" thickBot="1">
-      <c r="A67" s="79"/>
-      <c r="B67" s="76"/>
+      <c r="A67" s="82"/>
+      <c r="B67" s="79"/>
       <c r="C67" s="56">
         <v>52</v>
       </c>
       <c r="D67" s="56" t="s">
-        <v>178</v>
+        <v>177</v>
       </c>
       <c r="E67" s="50">
         <v>3250</v>
       </c>
       <c r="F67" s="50" t="s">
-        <v>107</v>
+        <v>106</v>
       </c>
       <c r="G67" s="51"/>
     </row>
     <row r="68" spans="1:7">
-      <c r="A68" s="68">
+      <c r="A68" s="69">
         <v>3</v>
       </c>
-      <c r="B68" s="71" t="s">
-        <v>225</v>
+      <c r="B68" s="72" t="s">
+        <v>224</v>
       </c>
       <c r="C68" s="39">
         <v>0</v>
       </c>
       <c r="D68" s="39" t="s">
-        <v>106</v>
+        <v>105</v>
       </c>
       <c r="E68" s="39">
         <v>325</v>
       </c>
       <c r="F68" s="39" t="s">
-        <v>107</v>
+        <v>106</v>
       </c>
       <c r="G68" s="40" t="s">
-        <v>226</v>
+        <v>225</v>
       </c>
     </row>
     <row r="69" spans="1:7">
-      <c r="A69" s="69"/>
-      <c r="B69" s="72"/>
+      <c r="A69" s="70"/>
+      <c r="B69" s="73"/>
       <c r="C69" s="41">
         <v>1</v>
       </c>
       <c r="D69" s="41" t="s">
-        <v>212</v>
+        <v>211</v>
       </c>
       <c r="E69" s="41">
         <v>325</v>
       </c>
       <c r="F69" s="41" t="s">
-        <v>107</v>
+        <v>106</v>
       </c>
       <c r="G69" s="42" t="s">
-        <v>261</v>
+        <v>260</v>
       </c>
     </row>
     <row r="70" spans="1:7">
-      <c r="A70" s="69"/>
-      <c r="B70" s="72"/>
+      <c r="A70" s="70"/>
+      <c r="B70" s="73"/>
       <c r="C70" s="41">
         <v>2</v>
       </c>
       <c r="D70" s="41" t="s">
-        <v>213</v>
+        <v>212</v>
       </c>
       <c r="E70" s="41">
         <v>325</v>
       </c>
       <c r="F70" s="41" t="s">
-        <v>110</v>
+        <v>109</v>
       </c>
       <c r="G70" s="42" t="s">
-        <v>262</v>
+        <v>261</v>
       </c>
     </row>
     <row r="71" spans="1:7">
-      <c r="A71" s="69"/>
-      <c r="B71" s="72"/>
+      <c r="A71" s="70"/>
+      <c r="B71" s="73"/>
       <c r="C71" s="41">
         <v>3</v>
       </c>
       <c r="D71" s="41" t="s">
-        <v>214</v>
+        <v>213</v>
       </c>
       <c r="E71" s="41">
         <v>325</v>
       </c>
       <c r="F71" s="41" t="s">
-        <v>107</v>
+        <v>106</v>
       </c>
       <c r="G71" s="48" t="s">
-        <v>180</v>
+        <v>179</v>
       </c>
     </row>
     <row r="72" spans="1:7">
-      <c r="A72" s="69"/>
-      <c r="B72" s="72"/>
+      <c r="A72" s="70"/>
+      <c r="B72" s="73"/>
       <c r="C72" s="41">
         <v>4</v>
       </c>
       <c r="D72" s="41" t="s">
-        <v>215</v>
+        <v>214</v>
       </c>
       <c r="E72" s="41">
         <v>325</v>
       </c>
       <c r="F72" s="41" t="s">
-        <v>107</v>
+        <v>106</v>
       </c>
       <c r="G72" s="42"/>
     </row>
     <row r="73" spans="1:7">
-      <c r="A73" s="69"/>
-      <c r="B73" s="72"/>
+      <c r="A73" s="70"/>
+      <c r="B73" s="73"/>
       <c r="C73" s="41">
         <v>5</v>
       </c>
       <c r="D73" s="41" t="s">
-        <v>216</v>
+        <v>215</v>
       </c>
       <c r="E73" s="41">
         <v>325</v>
       </c>
       <c r="F73" s="41" t="s">
-        <v>107</v>
+        <v>106</v>
       </c>
       <c r="G73" s="42"/>
     </row>
     <row r="74" spans="1:7">
-      <c r="A74" s="69"/>
-      <c r="B74" s="72"/>
+      <c r="A74" s="70"/>
+      <c r="B74" s="73"/>
       <c r="C74" s="41">
         <v>6</v>
       </c>
       <c r="D74" s="41" t="s">
-        <v>217</v>
+        <v>216</v>
       </c>
       <c r="E74" s="41">
         <v>325</v>
       </c>
       <c r="F74" s="41" t="s">
-        <v>107</v>
+        <v>106</v>
       </c>
       <c r="G74" s="42"/>
     </row>
     <row r="75" spans="1:7">
-      <c r="A75" s="69"/>
-      <c r="B75" s="72"/>
+      <c r="A75" s="70"/>
+      <c r="B75" s="73"/>
       <c r="C75" s="41">
         <v>7</v>
       </c>
       <c r="D75" s="41" t="s">
-        <v>218</v>
+        <v>217</v>
       </c>
       <c r="E75" s="41">
         <v>325</v>
       </c>
       <c r="F75" s="41" t="s">
-        <v>107</v>
+        <v>106</v>
       </c>
       <c r="G75" s="42"/>
     </row>
     <row r="76" spans="1:7">
-      <c r="A76" s="69"/>
-      <c r="B76" s="72"/>
+      <c r="A76" s="70"/>
+      <c r="B76" s="73"/>
       <c r="C76" s="41">
         <v>8</v>
       </c>
       <c r="D76" s="41" t="s">
-        <v>219</v>
+        <v>218</v>
       </c>
       <c r="E76" s="41">
         <v>325</v>
       </c>
       <c r="F76" s="41" t="s">
-        <v>107</v>
+        <v>106</v>
       </c>
       <c r="G76" s="42"/>
     </row>
     <row r="77" spans="1:7">
-      <c r="A77" s="69"/>
-      <c r="B77" s="72"/>
+      <c r="A77" s="70"/>
+      <c r="B77" s="73"/>
       <c r="C77" s="41">
         <v>9</v>
       </c>
       <c r="D77" s="41" t="s">
-        <v>220</v>
+        <v>219</v>
       </c>
       <c r="E77" s="41">
         <v>325</v>
       </c>
       <c r="F77" s="41" t="s">
-        <v>107</v>
+        <v>106</v>
       </c>
       <c r="G77" s="42"/>
     </row>
     <row r="78" spans="1:7">
-      <c r="A78" s="69"/>
-      <c r="B78" s="72"/>
+      <c r="A78" s="70"/>
+      <c r="B78" s="73"/>
       <c r="C78" s="41">
         <v>10</v>
       </c>
       <c r="D78" s="41" t="s">
-        <v>221</v>
+        <v>220</v>
       </c>
       <c r="E78" s="41">
         <v>325</v>
       </c>
       <c r="F78" s="41" t="s">
-        <v>107</v>
+        <v>106</v>
       </c>
       <c r="G78" s="42"/>
     </row>
     <row r="79" spans="1:7">
-      <c r="A79" s="69"/>
-      <c r="B79" s="72"/>
+      <c r="A79" s="70"/>
+      <c r="B79" s="73"/>
       <c r="C79" s="41">
         <v>11</v>
       </c>
       <c r="D79" s="41" t="s">
-        <v>222</v>
+        <v>221</v>
       </c>
       <c r="E79" s="41">
         <v>325</v>
       </c>
       <c r="F79" s="41" t="s">
-        <v>107</v>
+        <v>106</v>
       </c>
       <c r="G79" s="42"/>
     </row>
     <row r="80" spans="1:7">
-      <c r="A80" s="69"/>
-      <c r="B80" s="72"/>
+      <c r="A80" s="70"/>
+      <c r="B80" s="73"/>
       <c r="C80" s="41">
         <v>12</v>
       </c>
       <c r="D80" s="41" t="s">
-        <v>223</v>
+        <v>222</v>
       </c>
       <c r="E80" s="41">
         <v>325</v>
       </c>
       <c r="F80" s="41" t="s">
-        <v>107</v>
+        <v>106</v>
       </c>
       <c r="G80" s="42"/>
     </row>
     <row r="81" spans="1:7" ht="17.5" thickBot="1">
-      <c r="A81" s="70"/>
-      <c r="B81" s="73"/>
+      <c r="A81" s="71"/>
+      <c r="B81" s="74"/>
       <c r="C81" s="44">
         <v>13</v>
       </c>
       <c r="D81" s="44" t="s">
-        <v>224</v>
+        <v>223</v>
       </c>
       <c r="E81" s="44">
         <v>325</v>
       </c>
       <c r="F81" s="44" t="s">
-        <v>107</v>
+        <v>106</v>
       </c>
       <c r="G81" s="45"/>
     </row>
     <row r="82" spans="1:7" ht="16.5" customHeight="1">
-      <c r="A82" s="68">
+      <c r="A82" s="69">
         <v>4</v>
       </c>
-      <c r="B82" s="80" t="s">
-        <v>228</v>
+      <c r="B82" s="66" t="s">
+        <v>227</v>
       </c>
       <c r="C82" s="39">
         <v>0</v>
       </c>
       <c r="D82" s="39" t="s">
-        <v>181</v>
+        <v>180</v>
       </c>
       <c r="E82" s="39">
         <v>1650</v>
       </c>
       <c r="F82" s="52" t="s">
-        <v>110</v>
+        <v>109</v>
       </c>
       <c r="G82" s="53"/>
     </row>
     <row r="83" spans="1:7">
-      <c r="A83" s="69"/>
-      <c r="B83" s="81"/>
+      <c r="A83" s="70"/>
+      <c r="B83" s="67"/>
       <c r="C83" s="41">
         <v>1</v>
       </c>
       <c r="D83" s="41" t="s">
-        <v>182</v>
+        <v>181</v>
       </c>
       <c r="E83" s="41">
         <v>1650</v>
       </c>
       <c r="F83" s="41" t="s">
-        <v>110</v>
+        <v>109</v>
       </c>
       <c r="G83" s="42"/>
     </row>
     <row r="84" spans="1:7">
-      <c r="A84" s="69"/>
-      <c r="B84" s="81"/>
+      <c r="A84" s="70"/>
+      <c r="B84" s="67"/>
       <c r="C84" s="41">
         <v>2</v>
       </c>
       <c r="D84" s="41" t="s">
-        <v>183</v>
+        <v>182</v>
       </c>
       <c r="E84" s="41">
         <v>1650</v>
       </c>
       <c r="F84" s="41" t="s">
-        <v>107</v>
+        <v>106</v>
       </c>
       <c r="G84" s="42"/>
     </row>
     <row r="85" spans="1:7">
-      <c r="A85" s="69"/>
-      <c r="B85" s="81"/>
+      <c r="A85" s="70"/>
+      <c r="B85" s="67"/>
       <c r="C85" s="41">
         <v>3</v>
       </c>
       <c r="D85" s="41" t="s">
-        <v>184</v>
+        <v>183</v>
       </c>
       <c r="E85" s="41">
         <v>1650</v>
       </c>
       <c r="F85" s="41" t="s">
-        <v>110</v>
+        <v>109</v>
       </c>
       <c r="G85" s="42"/>
     </row>
     <row r="86" spans="1:7">
-      <c r="A86" s="69"/>
-      <c r="B86" s="81"/>
+      <c r="A86" s="70"/>
+      <c r="B86" s="67"/>
       <c r="C86" s="41">
         <v>4</v>
       </c>
       <c r="D86" s="41" t="s">
-        <v>229</v>
+        <v>228</v>
       </c>
       <c r="E86" s="41">
         <v>1650</v>
       </c>
       <c r="F86" s="41" t="s">
-        <v>107</v>
+        <v>106</v>
       </c>
       <c r="G86" s="42"/>
     </row>
     <row r="87" spans="1:7">
-      <c r="A87" s="69"/>
-      <c r="B87" s="81"/>
+      <c r="A87" s="70"/>
+      <c r="B87" s="67"/>
       <c r="C87" s="41">
         <v>5</v>
       </c>
       <c r="D87" s="41" t="s">
-        <v>230</v>
+        <v>229</v>
       </c>
       <c r="E87" s="41">
         <v>1650</v>
       </c>
       <c r="F87" s="41" t="s">
-        <v>107</v>
+        <v>106</v>
       </c>
       <c r="G87" s="42"/>
     </row>
     <row r="88" spans="1:7">
-      <c r="A88" s="69"/>
-      <c r="B88" s="81"/>
+      <c r="A88" s="70"/>
+      <c r="B88" s="67"/>
       <c r="C88" s="41">
         <v>6</v>
       </c>
       <c r="D88" s="41" t="s">
-        <v>108</v>
+        <v>107</v>
       </c>
       <c r="E88" s="41">
         <v>1650</v>
       </c>
       <c r="F88" s="41" t="s">
-        <v>107</v>
+        <v>106</v>
       </c>
       <c r="G88" s="42"/>
     </row>
     <row r="89" spans="1:7">
-      <c r="A89" s="69"/>
-      <c r="B89" s="81"/>
+      <c r="A89" s="70"/>
+      <c r="B89" s="67"/>
       <c r="C89" s="41">
         <v>7</v>
       </c>
       <c r="D89" s="41" t="s">
-        <v>109</v>
+        <v>108</v>
       </c>
       <c r="E89" s="41">
         <v>1650</v>
       </c>
       <c r="F89" s="41" t="s">
-        <v>110</v>
+        <v>109</v>
       </c>
       <c r="G89" s="42"/>
     </row>
     <row r="90" spans="1:7">
-      <c r="A90" s="69"/>
-      <c r="B90" s="81"/>
+      <c r="A90" s="70"/>
+      <c r="B90" s="67"/>
       <c r="C90" s="41">
         <v>8</v>
       </c>
       <c r="D90" s="41" t="s">
-        <v>212</v>
+        <v>211</v>
       </c>
       <c r="E90" s="41">
         <v>1650</v>
       </c>
       <c r="F90" s="41" t="s">
-        <v>107</v>
+        <v>106</v>
       </c>
       <c r="G90" s="42"/>
     </row>
     <row r="91" spans="1:7">
-      <c r="A91" s="69"/>
-      <c r="B91" s="81"/>
+      <c r="A91" s="70"/>
+      <c r="B91" s="67"/>
       <c r="C91" s="41">
         <v>9</v>
       </c>
       <c r="D91" s="41" t="s">
-        <v>213</v>
+        <v>212</v>
       </c>
       <c r="E91" s="41">
         <v>1650</v>
       </c>
       <c r="F91" s="41" t="s">
-        <v>110</v>
+        <v>109</v>
       </c>
       <c r="G91" s="42"/>
     </row>
     <row r="92" spans="1:7" ht="17.5" thickBot="1">
-      <c r="A92" s="70"/>
-      <c r="B92" s="82"/>
+      <c r="A92" s="71"/>
+      <c r="B92" s="68"/>
       <c r="C92" s="44">
         <v>10</v>
       </c>
       <c r="D92" s="44" t="s">
-        <v>231</v>
+        <v>230</v>
       </c>
       <c r="E92" s="44">
         <v>1650</v>
       </c>
       <c r="F92" s="44" t="s">
-        <v>107</v>
+        <v>106</v>
       </c>
       <c r="G92" s="45"/>
     </row>
     <row r="93" spans="1:7">
-      <c r="A93" s="68">
+      <c r="A93" s="69">
         <v>5</v>
       </c>
-      <c r="B93" s="71" t="s">
-        <v>209</v>
+      <c r="B93" s="72" t="s">
+        <v>208</v>
       </c>
       <c r="C93" s="39">
         <v>0</v>
       </c>
       <c r="D93" s="39" t="s">
-        <v>106</v>
+        <v>105</v>
       </c>
       <c r="E93" s="39">
         <v>160352</v>
       </c>
       <c r="F93" s="39" t="s">
-        <v>107</v>
+        <v>106</v>
       </c>
       <c r="G93" s="40" t="s">
-        <v>226</v>
+        <v>225</v>
       </c>
     </row>
     <row r="94" spans="1:7">
-      <c r="A94" s="69"/>
-      <c r="B94" s="72"/>
+      <c r="A94" s="70"/>
+      <c r="B94" s="73"/>
       <c r="C94" s="41">
         <v>1</v>
       </c>
       <c r="D94" s="41" t="s">
-        <v>181</v>
+        <v>180</v>
       </c>
       <c r="E94" s="41">
         <v>160352</v>
       </c>
       <c r="F94" s="41" t="s">
-        <v>110</v>
+        <v>109</v>
       </c>
       <c r="G94" s="42"/>
     </row>
     <row r="95" spans="1:7">
-      <c r="A95" s="69"/>
-      <c r="B95" s="72"/>
+      <c r="A95" s="70"/>
+      <c r="B95" s="73"/>
       <c r="C95" s="41">
         <v>2</v>
       </c>
       <c r="D95" s="41" t="s">
-        <v>182</v>
+        <v>181</v>
       </c>
       <c r="E95" s="41">
         <v>160352</v>
       </c>
       <c r="F95" s="41" t="s">
-        <v>110</v>
+        <v>109</v>
       </c>
       <c r="G95" s="42"/>
     </row>
     <row r="96" spans="1:7">
-      <c r="A96" s="69"/>
-      <c r="B96" s="72"/>
+      <c r="A96" s="70"/>
+      <c r="B96" s="73"/>
       <c r="C96" s="41">
         <v>3</v>
       </c>
       <c r="D96" s="41" t="s">
-        <v>183</v>
+        <v>182</v>
       </c>
       <c r="E96" s="41">
         <v>160352</v>
       </c>
       <c r="F96" s="41" t="s">
-        <v>107</v>
+        <v>106</v>
       </c>
       <c r="G96" s="42"/>
     </row>
     <row r="97" spans="1:7">
-      <c r="A97" s="69"/>
-      <c r="B97" s="72"/>
+      <c r="A97" s="70"/>
+      <c r="B97" s="73"/>
       <c r="C97" s="41">
         <v>4</v>
       </c>
       <c r="D97" s="41" t="s">
-        <v>184</v>
+        <v>183</v>
       </c>
       <c r="E97" s="41">
         <v>160352</v>
       </c>
       <c r="F97" s="41" t="s">
-        <v>110</v>
+        <v>109</v>
       </c>
       <c r="G97" s="42"/>
     </row>
     <row r="98" spans="1:7" ht="51">
-      <c r="A98" s="69"/>
-      <c r="B98" s="72"/>
+      <c r="A98" s="70"/>
+      <c r="B98" s="73"/>
       <c r="C98" s="41">
         <v>5</v>
       </c>
       <c r="D98" s="41" t="s">
-        <v>111</v>
+        <v>110</v>
       </c>
       <c r="E98" s="41">
         <v>160352</v>
       </c>
       <c r="F98" s="41" t="s">
-        <v>110</v>
+        <v>109</v>
       </c>
       <c r="G98" s="43" t="s">
-        <v>128</v>
+        <v>127</v>
       </c>
     </row>
     <row r="99" spans="1:7">
-      <c r="A99" s="69"/>
-      <c r="B99" s="72"/>
+      <c r="A99" s="70"/>
+      <c r="B99" s="73"/>
       <c r="C99" s="41">
         <v>6</v>
       </c>
       <c r="D99" s="41" t="s">
-        <v>112</v>
+        <v>111</v>
       </c>
       <c r="E99" s="41">
         <v>160352</v>
       </c>
       <c r="F99" s="41" t="s">
-        <v>110</v>
+        <v>109</v>
       </c>
       <c r="G99" s="42"/>
     </row>
     <row r="100" spans="1:7">
-      <c r="A100" s="69"/>
-      <c r="B100" s="72"/>
+      <c r="A100" s="70"/>
+      <c r="B100" s="73"/>
       <c r="C100" s="41">
         <v>7</v>
       </c>
       <c r="D100" s="41" t="s">
-        <v>114</v>
+        <v>113</v>
       </c>
       <c r="E100" s="41">
         <v>160352</v>
       </c>
       <c r="F100" s="41" t="s">
-        <v>107</v>
+        <v>106</v>
       </c>
       <c r="G100" s="43" t="s">
-        <v>210</v>
+        <v>209</v>
       </c>
     </row>
     <row r="101" spans="1:7" ht="51">
-      <c r="A101" s="69"/>
-      <c r="B101" s="72"/>
+      <c r="A101" s="70"/>
+      <c r="B101" s="73"/>
       <c r="C101" s="41">
         <v>8</v>
       </c>
       <c r="D101" s="41" t="s">
-        <v>113</v>
+        <v>112</v>
       </c>
       <c r="E101" s="41">
         <v>160352</v>
       </c>
       <c r="F101" s="41" t="s">
-        <v>107</v>
+        <v>106</v>
       </c>
       <c r="G101" s="43" t="s">
-        <v>211</v>
+        <v>210</v>
       </c>
     </row>
     <row r="102" spans="1:7">
-      <c r="A102" s="69"/>
-      <c r="B102" s="72"/>
+      <c r="A102" s="70"/>
+      <c r="B102" s="73"/>
       <c r="C102" s="41">
         <v>9</v>
       </c>
       <c r="D102" s="41" t="s">
-        <v>116</v>
+        <v>115</v>
       </c>
       <c r="E102" s="41">
         <v>160352</v>
       </c>
       <c r="F102" s="41" t="s">
-        <v>107</v>
+        <v>106</v>
       </c>
       <c r="G102" s="42" t="s">
-        <v>267</v>
+        <v>266</v>
       </c>
     </row>
     <row r="103" spans="1:7">
-      <c r="A103" s="69"/>
-      <c r="B103" s="72"/>
+      <c r="A103" s="70"/>
+      <c r="B103" s="73"/>
       <c r="C103" s="41">
         <v>10</v>
       </c>
       <c r="D103" s="41" t="s">
-        <v>118</v>
+        <v>117</v>
       </c>
       <c r="E103" s="41">
         <v>160352</v>
       </c>
       <c r="F103" s="41" t="s">
-        <v>107</v>
+        <v>106</v>
       </c>
       <c r="G103" s="42"/>
     </row>
     <row r="104" spans="1:7">
-      <c r="A104" s="69"/>
-      <c r="B104" s="72"/>
+      <c r="A104" s="70"/>
+      <c r="B104" s="73"/>
       <c r="C104" s="41">
         <v>11</v>
       </c>
       <c r="D104" s="41" t="s">
-        <v>286</v>
+        <v>285</v>
       </c>
       <c r="E104" s="41">
         <v>160352</v>
       </c>
       <c r="F104" s="41" t="s">
-        <v>107</v>
+        <v>106</v>
       </c>
       <c r="G104" s="42" t="s">
-        <v>268</v>
+        <v>267</v>
       </c>
     </row>
     <row r="105" spans="1:7">
-      <c r="A105" s="69"/>
-      <c r="B105" s="72"/>
+      <c r="A105" s="70"/>
+      <c r="B105" s="73"/>
       <c r="C105" s="41">
         <v>12</v>
       </c>
       <c r="D105" s="41" t="s">
-        <v>124</v>
+        <v>123</v>
       </c>
       <c r="E105" s="41">
         <v>160352</v>
       </c>
       <c r="F105" s="41" t="s">
-        <v>107</v>
+        <v>106</v>
       </c>
       <c r="G105" s="42"/>
     </row>
     <row r="106" spans="1:7" ht="17.5" thickBot="1">
-      <c r="A106" s="70"/>
-      <c r="B106" s="73"/>
+      <c r="A106" s="71"/>
+      <c r="B106" s="74"/>
       <c r="C106" s="44">
         <v>13</v>
       </c>
       <c r="D106" s="44" t="s">
-        <v>115</v>
+        <v>114</v>
       </c>
       <c r="E106" s="44">
         <v>160352</v>
       </c>
       <c r="F106" s="44" t="s">
-        <v>107</v>
+        <v>106</v>
       </c>
       <c r="G106" s="45"/>
     </row>
     <row r="107" spans="1:7">
-      <c r="A107" s="68">
+      <c r="A107" s="69">
         <v>6</v>
       </c>
-      <c r="B107" s="71" t="s">
-        <v>205</v>
+      <c r="B107" s="72" t="s">
+        <v>204</v>
       </c>
       <c r="C107" s="39">
         <v>0</v>
       </c>
       <c r="D107" s="39" t="s">
-        <v>106</v>
+        <v>105</v>
       </c>
       <c r="E107" s="39">
         <v>20514</v>
       </c>
       <c r="F107" s="39" t="s">
-        <v>107</v>
+        <v>106</v>
       </c>
       <c r="G107" s="40" t="s">
-        <v>226</v>
+        <v>225</v>
       </c>
     </row>
     <row r="108" spans="1:7">
-      <c r="A108" s="69"/>
-      <c r="B108" s="72"/>
+      <c r="A108" s="70"/>
+      <c r="B108" s="73"/>
       <c r="C108" s="41">
         <v>1</v>
       </c>
       <c r="D108" s="41" t="s">
-        <v>181</v>
+        <v>180</v>
       </c>
       <c r="E108" s="41">
         <v>20514</v>
       </c>
       <c r="F108" s="41" t="s">
-        <v>110</v>
+        <v>109</v>
       </c>
       <c r="G108" s="42"/>
     </row>
     <row r="109" spans="1:7">
-      <c r="A109" s="69"/>
-      <c r="B109" s="72"/>
+      <c r="A109" s="70"/>
+      <c r="B109" s="73"/>
       <c r="C109" s="41">
         <v>2</v>
       </c>
       <c r="D109" s="41" t="s">
-        <v>182</v>
+        <v>181</v>
       </c>
       <c r="E109" s="41">
         <v>20514</v>
       </c>
       <c r="F109" s="41" t="s">
-        <v>110</v>
+        <v>109</v>
       </c>
       <c r="G109" s="42"/>
     </row>
     <row r="110" spans="1:7">
-      <c r="A110" s="69"/>
-      <c r="B110" s="72"/>
+      <c r="A110" s="70"/>
+      <c r="B110" s="73"/>
       <c r="C110" s="41">
         <v>3</v>
       </c>
       <c r="D110" s="41" t="s">
-        <v>183</v>
+        <v>182</v>
       </c>
       <c r="E110" s="41">
         <v>20514</v>
       </c>
       <c r="F110" s="41" t="s">
-        <v>107</v>
+        <v>106</v>
       </c>
       <c r="G110" s="42"/>
     </row>
     <row r="111" spans="1:7">
-      <c r="A111" s="69"/>
-      <c r="B111" s="72"/>
+      <c r="A111" s="70"/>
+      <c r="B111" s="73"/>
       <c r="C111" s="41">
         <v>4</v>
       </c>
       <c r="D111" s="41" t="s">
-        <v>184</v>
+        <v>183</v>
       </c>
       <c r="E111" s="41">
         <v>20514</v>
       </c>
       <c r="F111" s="41" t="s">
-        <v>110</v>
+        <v>109</v>
       </c>
       <c r="G111" s="42"/>
     </row>
     <row r="112" spans="1:7">
-      <c r="A112" s="69"/>
-      <c r="B112" s="72"/>
+      <c r="A112" s="70"/>
+      <c r="B112" s="73"/>
       <c r="C112" s="41">
         <v>5</v>
       </c>
       <c r="D112" s="41" t="s">
-        <v>185</v>
+        <v>184</v>
       </c>
       <c r="E112" s="41">
         <v>20514</v>
       </c>
       <c r="F112" s="41" t="s">
-        <v>107</v>
+        <v>106</v>
       </c>
       <c r="G112" s="42" t="s">
-        <v>266</v>
+        <v>265</v>
       </c>
     </row>
     <row r="113" spans="1:7">
-      <c r="A113" s="69"/>
-      <c r="B113" s="72"/>
+      <c r="A113" s="70"/>
+      <c r="B113" s="73"/>
       <c r="C113" s="41">
         <v>6</v>
       </c>
       <c r="D113" s="41" t="s">
-        <v>186</v>
+        <v>185</v>
       </c>
       <c r="E113" s="41">
         <v>20514</v>
       </c>
       <c r="F113" s="41" t="s">
-        <v>117</v>
+        <v>116</v>
       </c>
       <c r="G113" s="42"/>
     </row>
     <row r="114" spans="1:7">
-      <c r="A114" s="69"/>
-      <c r="B114" s="72"/>
+      <c r="A114" s="70"/>
+      <c r="B114" s="73"/>
       <c r="C114" s="41">
         <v>7</v>
       </c>
       <c r="D114" s="41" t="s">
-        <v>187</v>
+        <v>186</v>
       </c>
       <c r="E114" s="41">
         <v>20514</v>
       </c>
       <c r="F114" s="41" t="s">
-        <v>117</v>
+        <v>116</v>
       </c>
       <c r="G114" s="42"/>
     </row>
     <row r="115" spans="1:7">
-      <c r="A115" s="69"/>
-      <c r="B115" s="72"/>
+      <c r="A115" s="70"/>
+      <c r="B115" s="73"/>
       <c r="C115" s="41">
         <v>8</v>
       </c>
       <c r="D115" s="41" t="s">
-        <v>188</v>
+        <v>187</v>
       </c>
       <c r="E115" s="41">
         <v>20514</v>
       </c>
       <c r="F115" s="41" t="s">
-        <v>117</v>
+        <v>116</v>
       </c>
       <c r="G115" s="42"/>
     </row>
     <row r="116" spans="1:7">
-      <c r="A116" s="69"/>
-      <c r="B116" s="72"/>
+      <c r="A116" s="70"/>
+      <c r="B116" s="73"/>
       <c r="C116" s="41">
         <v>9</v>
       </c>
       <c r="D116" s="41" t="s">
-        <v>189</v>
+        <v>188</v>
       </c>
       <c r="E116" s="41">
         <v>20514</v>
       </c>
       <c r="F116" s="41" t="s">
-        <v>117</v>
+        <v>116</v>
       </c>
       <c r="G116" s="42"/>
     </row>
     <row r="117" spans="1:7">
-      <c r="A117" s="69"/>
-      <c r="B117" s="72"/>
+      <c r="A117" s="70"/>
+      <c r="B117" s="73"/>
       <c r="C117" s="41">
         <v>10</v>
       </c>
       <c r="D117" s="41" t="s">
-        <v>190</v>
+        <v>189</v>
       </c>
       <c r="E117" s="41">
         <v>20514</v>
       </c>
       <c r="F117" s="41" t="s">
-        <v>117</v>
+        <v>116</v>
       </c>
       <c r="G117" s="42"/>
     </row>
     <row r="118" spans="1:7">
-      <c r="A118" s="69"/>
-      <c r="B118" s="72"/>
+      <c r="A118" s="70"/>
+      <c r="B118" s="73"/>
       <c r="C118" s="41">
         <v>11</v>
       </c>
       <c r="D118" s="41" t="s">
-        <v>191</v>
+        <v>190</v>
       </c>
       <c r="E118" s="41">
         <v>20514</v>
       </c>
       <c r="F118" s="41" t="s">
-        <v>117</v>
+        <v>116</v>
       </c>
       <c r="G118" s="42"/>
     </row>
     <row r="119" spans="1:7">
-      <c r="A119" s="69"/>
-      <c r="B119" s="72"/>
+      <c r="A119" s="70"/>
+      <c r="B119" s="73"/>
       <c r="C119" s="41">
         <v>12</v>
       </c>
       <c r="D119" s="41" t="s">
-        <v>192</v>
+        <v>191</v>
       </c>
       <c r="E119" s="41">
         <v>20514</v>
       </c>
       <c r="F119" s="41" t="s">
-        <v>117</v>
+        <v>116</v>
       </c>
       <c r="G119" s="42"/>
     </row>
     <row r="120" spans="1:7">
-      <c r="A120" s="69"/>
-      <c r="B120" s="72"/>
+      <c r="A120" s="70"/>
+      <c r="B120" s="73"/>
       <c r="C120" s="41">
         <v>13</v>
       </c>
       <c r="D120" s="41" t="s">
-        <v>193</v>
+        <v>192</v>
       </c>
       <c r="E120" s="41">
         <v>20514</v>
       </c>
       <c r="F120" s="41" t="s">
-        <v>117</v>
+        <v>116</v>
       </c>
       <c r="G120" s="42"/>
     </row>
     <row r="121" spans="1:7">
-      <c r="A121" s="69"/>
-      <c r="B121" s="72"/>
+      <c r="A121" s="70"/>
+      <c r="B121" s="73"/>
       <c r="C121" s="41">
         <v>14</v>
       </c>
       <c r="D121" s="41" t="s">
-        <v>194</v>
+        <v>193</v>
       </c>
       <c r="E121" s="41">
         <v>20514</v>
       </c>
       <c r="F121" s="41" t="s">
-        <v>117</v>
+        <v>116</v>
       </c>
       <c r="G121" s="42"/>
     </row>
     <row r="122" spans="1:7">
-      <c r="A122" s="69"/>
-      <c r="B122" s="72"/>
+      <c r="A122" s="70"/>
+      <c r="B122" s="73"/>
       <c r="C122" s="41">
         <v>15</v>
       </c>
       <c r="D122" s="41" t="s">
-        <v>195</v>
+        <v>194</v>
       </c>
       <c r="E122" s="41">
         <v>20514</v>
       </c>
       <c r="F122" s="41" t="s">
-        <v>117</v>
+        <v>116</v>
       </c>
       <c r="G122" s="42"/>
     </row>
     <row r="123" spans="1:7">
-      <c r="A123" s="69"/>
-      <c r="B123" s="72"/>
+      <c r="A123" s="70"/>
+      <c r="B123" s="73"/>
       <c r="C123" s="41">
         <v>16</v>
       </c>
       <c r="D123" s="41" t="s">
-        <v>196</v>
+        <v>195</v>
       </c>
       <c r="E123" s="41">
         <v>20514</v>
       </c>
       <c r="F123" s="41" t="s">
-        <v>117</v>
+        <v>116</v>
       </c>
       <c r="G123" s="42"/>
     </row>
     <row r="124" spans="1:7">
-      <c r="A124" s="69"/>
-      <c r="B124" s="72"/>
+      <c r="A124" s="70"/>
+      <c r="B124" s="73"/>
       <c r="C124" s="41">
         <v>17</v>
       </c>
       <c r="D124" s="41" t="s">
-        <v>197</v>
+        <v>196</v>
       </c>
       <c r="E124" s="41">
         <v>20514</v>
       </c>
       <c r="F124" s="41" t="s">
-        <v>117</v>
+        <v>116</v>
       </c>
       <c r="G124" s="42"/>
     </row>
     <row r="125" spans="1:7">
-      <c r="A125" s="69"/>
-      <c r="B125" s="72"/>
+      <c r="A125" s="70"/>
+      <c r="B125" s="73"/>
       <c r="C125" s="41">
         <v>18</v>
       </c>
       <c r="D125" s="41" t="s">
-        <v>198</v>
+        <v>197</v>
       </c>
       <c r="E125" s="41">
         <v>20514</v>
       </c>
       <c r="F125" s="41" t="s">
-        <v>117</v>
+        <v>116</v>
       </c>
       <c r="G125" s="42"/>
     </row>
     <row r="126" spans="1:7">
-      <c r="A126" s="69"/>
-      <c r="B126" s="72"/>
+      <c r="A126" s="70"/>
+      <c r="B126" s="73"/>
       <c r="C126" s="41">
         <v>19</v>
       </c>
       <c r="D126" s="41" t="s">
-        <v>199</v>
+        <v>198</v>
       </c>
       <c r="E126" s="41">
         <v>20514</v>
       </c>
       <c r="F126" s="41" t="s">
-        <v>117</v>
+        <v>116</v>
       </c>
       <c r="G126" s="42"/>
     </row>
     <row r="127" spans="1:7">
-      <c r="A127" s="69"/>
-      <c r="B127" s="72"/>
+      <c r="A127" s="70"/>
+      <c r="B127" s="73"/>
       <c r="C127" s="41">
         <v>20</v>
       </c>
       <c r="D127" s="41" t="s">
-        <v>200</v>
+        <v>199</v>
       </c>
       <c r="E127" s="41">
         <v>20514</v>
       </c>
       <c r="F127" s="41" t="s">
-        <v>117</v>
+        <v>116</v>
       </c>
       <c r="G127" s="42"/>
     </row>
     <row r="128" spans="1:7">
-      <c r="A128" s="69"/>
-      <c r="B128" s="72"/>
+      <c r="A128" s="70"/>
+      <c r="B128" s="73"/>
       <c r="C128" s="41">
         <v>21</v>
       </c>
       <c r="D128" s="41" t="s">
-        <v>201</v>
+        <v>200</v>
       </c>
       <c r="E128" s="41">
         <v>20514</v>
       </c>
       <c r="F128" s="41" t="s">
-        <v>117</v>
+        <v>116</v>
       </c>
       <c r="G128" s="42"/>
     </row>
     <row r="129" spans="1:7">
-      <c r="A129" s="69"/>
-      <c r="B129" s="72"/>
+      <c r="A129" s="70"/>
+      <c r="B129" s="73"/>
       <c r="C129" s="41">
         <v>22</v>
       </c>
       <c r="D129" s="41" t="s">
-        <v>202</v>
+        <v>201</v>
       </c>
       <c r="E129" s="41">
         <v>20514</v>
       </c>
       <c r="F129" s="41" t="s">
-        <v>117</v>
+        <v>116</v>
       </c>
       <c r="G129" s="42"/>
     </row>
     <row r="130" spans="1:7">
-      <c r="A130" s="69"/>
-      <c r="B130" s="72"/>
+      <c r="A130" s="70"/>
+      <c r="B130" s="73"/>
       <c r="C130" s="41">
         <v>23</v>
       </c>
       <c r="D130" s="41" t="s">
-        <v>203</v>
+        <v>202</v>
       </c>
       <c r="E130" s="41">
         <v>20514</v>
       </c>
       <c r="F130" s="41" t="s">
-        <v>117</v>
+        <v>116</v>
       </c>
       <c r="G130" s="42"/>
     </row>
     <row r="131" spans="1:7" ht="17.5" thickBot="1">
-      <c r="A131" s="70"/>
-      <c r="B131" s="73"/>
+      <c r="A131" s="71"/>
+      <c r="B131" s="74"/>
       <c r="C131" s="44">
         <v>24</v>
       </c>
       <c r="D131" s="44" t="s">
-        <v>204</v>
+        <v>203</v>
       </c>
       <c r="E131" s="44">
         <v>20514</v>
       </c>
       <c r="F131" s="44" t="s">
-        <v>117</v>
+        <v>116</v>
       </c>
       <c r="G131" s="45"/>
     </row>
     <row r="132" spans="1:7">
-      <c r="A132" s="68">
+      <c r="A132" s="69">
         <v>7</v>
       </c>
-      <c r="B132" s="80" t="s">
-        <v>227</v>
+      <c r="B132" s="66" t="s">
+        <v>226</v>
       </c>
       <c r="C132" s="39">
         <v>0</v>
       </c>
       <c r="D132" s="39" t="s">
-        <v>106</v>
+        <v>105</v>
       </c>
       <c r="E132" s="39">
         <v>325</v>
       </c>
       <c r="F132" s="39" t="s">
-        <v>107</v>
+        <v>106</v>
       </c>
       <c r="G132" s="40" t="s">
-        <v>226</v>
+        <v>225</v>
       </c>
     </row>
     <row r="133" spans="1:7">
-      <c r="A133" s="69"/>
-      <c r="B133" s="81"/>
+      <c r="A133" s="70"/>
+      <c r="B133" s="67"/>
       <c r="C133" s="41">
         <v>1</v>
       </c>
       <c r="D133" s="41" t="s">
-        <v>108</v>
+        <v>107</v>
       </c>
       <c r="E133" s="41">
         <v>325</v>
       </c>
       <c r="F133" s="41" t="s">
-        <v>107</v>
+        <v>106</v>
       </c>
       <c r="G133" s="42"/>
     </row>
     <row r="134" spans="1:7">
-      <c r="A134" s="69"/>
-      <c r="B134" s="81"/>
+      <c r="A134" s="70"/>
+      <c r="B134" s="67"/>
       <c r="C134" s="41">
         <v>2</v>
       </c>
       <c r="D134" s="41" t="s">
-        <v>109</v>
+        <v>108</v>
       </c>
       <c r="E134" s="41">
         <v>325</v>
       </c>
       <c r="F134" s="41" t="s">
-        <v>110</v>
+        <v>109</v>
       </c>
       <c r="G134" s="42"/>
     </row>
     <row r="135" spans="1:7">
-      <c r="A135" s="69"/>
-      <c r="B135" s="81"/>
+      <c r="A135" s="70"/>
+      <c r="B135" s="67"/>
       <c r="C135" s="41">
         <v>3</v>
       </c>
       <c r="D135" s="41" t="s">
-        <v>239</v>
+        <v>238</v>
       </c>
       <c r="E135" s="41">
         <v>325</v>
       </c>
       <c r="F135" s="41" t="s">
-        <v>107</v>
+        <v>106</v>
       </c>
       <c r="G135" s="42" t="s">
-        <v>264</v>
+        <v>263</v>
       </c>
     </row>
     <row r="136" spans="1:7">
-      <c r="A136" s="69"/>
-      <c r="B136" s="81"/>
+      <c r="A136" s="70"/>
+      <c r="B136" s="67"/>
       <c r="C136" s="41">
         <v>4</v>
       </c>
       <c r="D136" s="41" t="s">
-        <v>240</v>
+        <v>239</v>
       </c>
       <c r="E136" s="41">
         <v>325</v>
       </c>
       <c r="F136" s="41" t="s">
-        <v>107</v>
+        <v>106</v>
       </c>
       <c r="G136" s="42"/>
     </row>
     <row r="137" spans="1:7">
-      <c r="A137" s="69"/>
-      <c r="B137" s="81"/>
+      <c r="A137" s="70"/>
+      <c r="B137" s="67"/>
       <c r="C137" s="41">
         <v>5</v>
       </c>
       <c r="D137" s="41" t="s">
-        <v>241</v>
+        <v>240</v>
       </c>
       <c r="E137" s="41">
         <v>325</v>
       </c>
       <c r="F137" s="41" t="s">
-        <v>107</v>
+        <v>106</v>
       </c>
       <c r="G137" s="42"/>
     </row>
     <row r="138" spans="1:7">
-      <c r="A138" s="69"/>
-      <c r="B138" s="81"/>
+      <c r="A138" s="70"/>
+      <c r="B138" s="67"/>
       <c r="C138" s="41">
         <v>6</v>
       </c>
       <c r="D138" s="41" t="s">
-        <v>242</v>
+        <v>241</v>
       </c>
       <c r="E138" s="41">
         <v>325</v>
       </c>
       <c r="F138" s="41" t="s">
-        <v>107</v>
+        <v>106</v>
       </c>
       <c r="G138" s="42"/>
     </row>
     <row r="139" spans="1:7">
-      <c r="A139" s="69"/>
-      <c r="B139" s="81"/>
+      <c r="A139" s="70"/>
+      <c r="B139" s="67"/>
       <c r="C139" s="41">
         <v>7</v>
       </c>
       <c r="D139" s="41" t="s">
-        <v>243</v>
+        <v>242</v>
       </c>
       <c r="E139" s="41">
         <v>325</v>
       </c>
       <c r="F139" s="41" t="s">
-        <v>107</v>
+        <v>106</v>
       </c>
       <c r="G139" s="42"/>
     </row>
     <row r="140" spans="1:7">
-      <c r="A140" s="69"/>
-      <c r="B140" s="81"/>
+      <c r="A140" s="70"/>
+      <c r="B140" s="67"/>
       <c r="C140" s="41">
         <v>8</v>
       </c>
       <c r="D140" s="41" t="s">
-        <v>244</v>
+        <v>243</v>
       </c>
       <c r="E140" s="41">
         <v>325</v>
       </c>
       <c r="F140" s="41" t="s">
-        <v>107</v>
+        <v>106</v>
       </c>
       <c r="G140" s="42"/>
     </row>
     <row r="141" spans="1:7">
-      <c r="A141" s="69"/>
-      <c r="B141" s="81"/>
+      <c r="A141" s="70"/>
+      <c r="B141" s="67"/>
       <c r="C141" s="41">
         <v>9</v>
       </c>
       <c r="D141" s="41" t="s">
-        <v>245</v>
+        <v>244</v>
       </c>
       <c r="E141" s="41">
         <v>325</v>
       </c>
       <c r="F141" s="41" t="s">
-        <v>107</v>
+        <v>106</v>
       </c>
       <c r="G141" s="42"/>
     </row>
     <row r="142" spans="1:7">
-      <c r="A142" s="69"/>
-      <c r="B142" s="81"/>
+      <c r="A142" s="70"/>
+      <c r="B142" s="67"/>
       <c r="C142" s="41">
         <v>10</v>
       </c>
       <c r="D142" s="41" t="s">
-        <v>246</v>
+        <v>245</v>
       </c>
       <c r="E142" s="41">
         <v>325</v>
       </c>
       <c r="F142" s="41" t="s">
-        <v>107</v>
+        <v>106</v>
       </c>
       <c r="G142" s="42"/>
     </row>
     <row r="143" spans="1:7">
-      <c r="A143" s="69"/>
-      <c r="B143" s="81"/>
+      <c r="A143" s="70"/>
+      <c r="B143" s="67"/>
       <c r="C143" s="41">
         <v>11</v>
       </c>
       <c r="D143" s="41" t="s">
-        <v>247</v>
+        <v>246</v>
       </c>
       <c r="E143" s="41">
         <v>325</v>
       </c>
       <c r="F143" s="41" t="s">
-        <v>107</v>
+        <v>106</v>
       </c>
       <c r="G143" s="42"/>
     </row>
     <row r="144" spans="1:7">
-      <c r="A144" s="69"/>
-      <c r="B144" s="81"/>
+      <c r="A144" s="70"/>
+      <c r="B144" s="67"/>
       <c r="C144" s="41">
         <v>12</v>
       </c>
       <c r="D144" s="41" t="s">
-        <v>248</v>
+        <v>247</v>
       </c>
       <c r="E144" s="41">
         <v>325</v>
       </c>
       <c r="F144" s="41" t="s">
-        <v>107</v>
+        <v>106</v>
       </c>
       <c r="G144" s="42"/>
     </row>
     <row r="145" spans="1:7">
-      <c r="A145" s="69"/>
-      <c r="B145" s="81"/>
+      <c r="A145" s="70"/>
+      <c r="B145" s="67"/>
       <c r="C145" s="41">
         <v>13</v>
       </c>
       <c r="D145" s="41" t="s">
-        <v>249</v>
+        <v>248</v>
       </c>
       <c r="E145" s="41">
         <v>325</v>
       </c>
       <c r="F145" s="41" t="s">
-        <v>107</v>
+        <v>106</v>
       </c>
       <c r="G145" s="42"/>
     </row>
     <row r="146" spans="1:7">
-      <c r="A146" s="69"/>
-      <c r="B146" s="81"/>
+      <c r="A146" s="70"/>
+      <c r="B146" s="67"/>
       <c r="C146" s="41">
         <v>14</v>
       </c>
       <c r="D146" s="41" t="s">
-        <v>250</v>
+        <v>249</v>
       </c>
       <c r="E146" s="41">
         <v>325</v>
       </c>
       <c r="F146" s="41" t="s">
-        <v>107</v>
+        <v>106</v>
       </c>
       <c r="G146" s="42"/>
     </row>
     <row r="147" spans="1:7">
-      <c r="A147" s="69"/>
-      <c r="B147" s="81"/>
+      <c r="A147" s="70"/>
+      <c r="B147" s="67"/>
       <c r="C147" s="41">
         <v>15</v>
       </c>
       <c r="D147" s="41" t="s">
-        <v>251</v>
+        <v>250</v>
       </c>
       <c r="E147" s="41">
         <v>325</v>
       </c>
       <c r="F147" s="41" t="s">
-        <v>107</v>
+        <v>106</v>
       </c>
       <c r="G147" s="42"/>
     </row>
     <row r="148" spans="1:7">
-      <c r="A148" s="69"/>
-      <c r="B148" s="81"/>
+      <c r="A148" s="70"/>
+      <c r="B148" s="67"/>
       <c r="C148" s="41">
         <v>16</v>
       </c>
       <c r="D148" s="41" t="s">
-        <v>252</v>
+        <v>251</v>
       </c>
       <c r="E148" s="41">
         <v>325</v>
       </c>
       <c r="F148" s="41" t="s">
-        <v>107</v>
+        <v>106</v>
       </c>
       <c r="G148" s="42"/>
     </row>
     <row r="149" spans="1:7">
-      <c r="A149" s="69"/>
-      <c r="B149" s="81"/>
+      <c r="A149" s="70"/>
+      <c r="B149" s="67"/>
       <c r="C149" s="41">
         <v>17</v>
       </c>
       <c r="D149" s="41" t="s">
-        <v>253</v>
+        <v>252</v>
       </c>
       <c r="E149" s="41">
         <v>325</v>
       </c>
       <c r="F149" s="41" t="s">
-        <v>107</v>
+        <v>106</v>
       </c>
       <c r="G149" s="42"/>
     </row>
     <row r="150" spans="1:7">
-      <c r="A150" s="69"/>
-      <c r="B150" s="81"/>
+      <c r="A150" s="70"/>
+      <c r="B150" s="67"/>
       <c r="C150" s="41">
         <v>18</v>
       </c>
       <c r="D150" s="41" t="s">
-        <v>254</v>
+        <v>253</v>
       </c>
       <c r="E150" s="41">
         <v>325</v>
       </c>
       <c r="F150" s="41" t="s">
-        <v>107</v>
+        <v>106</v>
       </c>
       <c r="G150" s="42"/>
     </row>
     <row r="151" spans="1:7">
-      <c r="A151" s="69"/>
-      <c r="B151" s="81"/>
+      <c r="A151" s="70"/>
+      <c r="B151" s="67"/>
       <c r="C151" s="41">
         <v>19</v>
       </c>
       <c r="D151" s="41" t="s">
-        <v>255</v>
+        <v>254</v>
       </c>
       <c r="E151" s="41">
         <v>325</v>
       </c>
       <c r="F151" s="41" t="s">
-        <v>107</v>
+        <v>106</v>
       </c>
       <c r="G151" s="42"/>
     </row>
     <row r="152" spans="1:7">
-      <c r="A152" s="69"/>
-      <c r="B152" s="81"/>
+      <c r="A152" s="70"/>
+      <c r="B152" s="67"/>
       <c r="C152" s="41">
         <v>20</v>
       </c>
       <c r="D152" s="41" t="s">
-        <v>256</v>
+        <v>255</v>
       </c>
       <c r="E152" s="41">
         <v>325</v>
       </c>
       <c r="F152" s="41" t="s">
-        <v>107</v>
+        <v>106</v>
       </c>
       <c r="G152" s="42"/>
     </row>
     <row r="153" spans="1:7">
-      <c r="A153" s="69"/>
-      <c r="B153" s="81"/>
+      <c r="A153" s="70"/>
+      <c r="B153" s="67"/>
       <c r="C153" s="41">
         <v>21</v>
       </c>
       <c r="D153" s="41" t="s">
-        <v>257</v>
+        <v>256</v>
       </c>
       <c r="E153" s="41">
         <v>325</v>
       </c>
       <c r="F153" s="41" t="s">
-        <v>107</v>
+        <v>106</v>
       </c>
       <c r="G153" s="42"/>
     </row>
     <row r="154" spans="1:7">
-      <c r="A154" s="69"/>
-      <c r="B154" s="81"/>
+      <c r="A154" s="70"/>
+      <c r="B154" s="67"/>
       <c r="C154" s="41">
         <v>22</v>
       </c>
       <c r="D154" s="41" t="s">
-        <v>258</v>
+        <v>257</v>
       </c>
       <c r="E154" s="41">
         <v>325</v>
       </c>
       <c r="F154" s="41" t="s">
-        <v>107</v>
+        <v>106</v>
       </c>
       <c r="G154" s="42"/>
     </row>
     <row r="155" spans="1:7">
-      <c r="A155" s="69"/>
-      <c r="B155" s="81"/>
+      <c r="A155" s="70"/>
+      <c r="B155" s="67"/>
       <c r="C155" s="41">
         <v>23</v>
       </c>
       <c r="D155" s="41" t="s">
-        <v>259</v>
+        <v>258</v>
       </c>
       <c r="E155" s="41">
         <v>325</v>
       </c>
       <c r="F155" s="41" t="s">
-        <v>107</v>
+        <v>106</v>
       </c>
       <c r="G155" s="42"/>
     </row>
     <row r="156" spans="1:7" ht="17.5" thickBot="1">
-      <c r="A156" s="70"/>
-      <c r="B156" s="82"/>
+      <c r="A156" s="71"/>
+      <c r="B156" s="68"/>
       <c r="C156" s="44">
         <v>24</v>
       </c>
       <c r="D156" s="44" t="s">
-        <v>260</v>
+        <v>259</v>
       </c>
       <c r="E156" s="44">
         <v>325</v>
       </c>
       <c r="F156" s="44" t="s">
-        <v>107</v>
+        <v>106</v>
       </c>
       <c r="G156" s="45"/>
     </row>
     <row r="157" spans="1:7">
-      <c r="A157" s="68">
+      <c r="A157" s="69">
         <v>8</v>
       </c>
-      <c r="B157" s="80" t="s">
-        <v>232</v>
+      <c r="B157" s="66" t="s">
+        <v>231</v>
       </c>
       <c r="C157" s="39">
         <v>0</v>
       </c>
       <c r="D157" s="39" t="s">
-        <v>106</v>
+        <v>105</v>
       </c>
       <c r="E157" s="39">
         <v>325</v>
       </c>
       <c r="F157" s="39" t="s">
-        <v>107</v>
+        <v>106</v>
       </c>
       <c r="G157" s="40" t="s">
-        <v>226</v>
+        <v>225</v>
       </c>
     </row>
     <row r="158" spans="1:7">
-      <c r="A158" s="69"/>
-      <c r="B158" s="81"/>
+      <c r="A158" s="70"/>
+      <c r="B158" s="67"/>
       <c r="C158" s="41">
         <v>1</v>
       </c>
       <c r="D158" s="41" t="s">
-        <v>108</v>
+        <v>107</v>
       </c>
       <c r="E158" s="41">
         <v>325</v>
       </c>
       <c r="F158" s="41" t="s">
-        <v>107</v>
+        <v>106</v>
       </c>
       <c r="G158" s="42"/>
     </row>
     <row r="159" spans="1:7">
-      <c r="A159" s="69"/>
-      <c r="B159" s="81"/>
+      <c r="A159" s="70"/>
+      <c r="B159" s="67"/>
       <c r="C159" s="41">
         <v>2</v>
       </c>
       <c r="D159" s="41" t="s">
-        <v>109</v>
+        <v>108</v>
       </c>
       <c r="E159" s="41">
         <v>325</v>
       </c>
       <c r="F159" s="41" t="s">
-        <v>110</v>
+        <v>109</v>
       </c>
       <c r="G159" s="42"/>
     </row>
     <row r="160" spans="1:7" ht="68">
-      <c r="A160" s="69"/>
-      <c r="B160" s="81"/>
+      <c r="A160" s="70"/>
+      <c r="B160" s="67"/>
       <c r="C160" s="41">
         <v>3</v>
       </c>
       <c r="D160" s="41" t="s">
-        <v>233</v>
+        <v>232</v>
       </c>
       <c r="E160" s="41">
         <v>325</v>
       </c>
       <c r="F160" s="41" t="s">
-        <v>110</v>
+        <v>109</v>
       </c>
       <c r="G160" s="43" t="s">
-        <v>265</v>
+        <v>264</v>
       </c>
     </row>
     <row r="161" spans="1:7">
-      <c r="A161" s="69"/>
-      <c r="B161" s="81"/>
+      <c r="A161" s="70"/>
+      <c r="B161" s="67"/>
       <c r="C161" s="41">
         <v>4</v>
       </c>
       <c r="D161" s="41" t="s">
-        <v>234</v>
+        <v>233</v>
       </c>
       <c r="E161" s="41">
         <v>325</v>
       </c>
       <c r="F161" s="41" t="s">
-        <v>110</v>
+        <v>109</v>
       </c>
       <c r="G161" s="42"/>
     </row>
     <row r="162" spans="1:7">
-      <c r="A162" s="69"/>
-      <c r="B162" s="81"/>
+      <c r="A162" s="70"/>
+      <c r="B162" s="67"/>
       <c r="C162" s="41">
         <v>5</v>
       </c>
       <c r="D162" s="41" t="s">
-        <v>235</v>
+        <v>234</v>
       </c>
       <c r="E162" s="41">
         <v>325</v>
       </c>
       <c r="F162" s="41" t="s">
-        <v>107</v>
+        <v>106</v>
       </c>
       <c r="G162" s="42"/>
     </row>
     <row r="163" spans="1:7">
-      <c r="A163" s="69"/>
-      <c r="B163" s="81"/>
+      <c r="A163" s="70"/>
+      <c r="B163" s="67"/>
       <c r="C163" s="41">
         <v>6</v>
       </c>
       <c r="D163" s="41" t="s">
-        <v>236</v>
+        <v>235</v>
       </c>
       <c r="E163" s="41">
         <v>325</v>
       </c>
       <c r="F163" s="41" t="s">
-        <v>107</v>
+        <v>106</v>
       </c>
       <c r="G163" s="42"/>
     </row>
     <row r="164" spans="1:7">
-      <c r="A164" s="69"/>
-      <c r="B164" s="81"/>
+      <c r="A164" s="70"/>
+      <c r="B164" s="67"/>
       <c r="C164" s="41">
         <v>7</v>
       </c>
       <c r="D164" s="41" t="s">
-        <v>237</v>
+        <v>236</v>
       </c>
       <c r="E164" s="41">
         <v>325</v>
       </c>
       <c r="F164" s="41" t="s">
-        <v>107</v>
+        <v>106</v>
       </c>
       <c r="G164" s="42"/>
     </row>
     <row r="165" spans="1:7" ht="17.5" thickBot="1">
-      <c r="A165" s="70"/>
-      <c r="B165" s="82"/>
+      <c r="A165" s="71"/>
+      <c r="B165" s="68"/>
       <c r="C165" s="44">
         <v>8</v>
       </c>
       <c r="D165" s="44" t="s">
-        <v>238</v>
+        <v>237</v>
       </c>
       <c r="E165" s="44">
         <v>325</v>
       </c>
       <c r="F165" s="44" t="s">
-        <v>107</v>
+        <v>106</v>
       </c>
       <c r="G165" s="45"/>
     </row>
@@ -6218,11 +6219,6 @@
     <filterColumn colId="3" showButton="0"/>
   </autoFilter>
   <mergeCells count="17">
-    <mergeCell ref="B157:B165"/>
-    <mergeCell ref="A157:A165"/>
-    <mergeCell ref="B132:B156"/>
-    <mergeCell ref="A132:A156"/>
-    <mergeCell ref="B107:B131"/>
     <mergeCell ref="A1:G1"/>
     <mergeCell ref="A3:A14"/>
     <mergeCell ref="A107:A131"/>
@@ -6235,6 +6231,11 @@
     <mergeCell ref="B3:B14"/>
     <mergeCell ref="A82:A92"/>
     <mergeCell ref="B82:B92"/>
+    <mergeCell ref="B157:B165"/>
+    <mergeCell ref="A157:A165"/>
+    <mergeCell ref="B132:B156"/>
+    <mergeCell ref="A132:A156"/>
+    <mergeCell ref="B107:B131"/>
   </mergeCells>
   <phoneticPr fontId="1" type="noConversion"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
@@ -6255,7 +6256,7 @@
   <sheetData>
     <row r="1" spans="1:5">
       <c r="A1" s="83" t="s">
-        <v>269</v>
+        <v>268</v>
       </c>
       <c r="B1" s="83"/>
       <c r="C1" s="83"/>
@@ -6264,19 +6265,19 @@
     </row>
     <row r="2" spans="1:5">
       <c r="A2" s="58" t="s">
-        <v>208</v>
+        <v>207</v>
       </c>
       <c r="B2" s="58" t="s">
         <v>0</v>
       </c>
       <c r="C2" s="58" t="s">
-        <v>123</v>
+        <v>122</v>
       </c>
       <c r="D2" s="58" t="s">
+        <v>269</v>
+      </c>
+      <c r="E2" s="58" t="s">
         <v>270</v>
-      </c>
-      <c r="E2" s="58" t="s">
-        <v>271</v>
       </c>
     </row>
     <row r="3" spans="1:5" ht="112">
@@ -6284,16 +6285,16 @@
         <v>1</v>
       </c>
       <c r="B3" s="20" t="s">
-        <v>276</v>
+        <v>275</v>
       </c>
       <c r="C3" s="57" t="s">
+        <v>272</v>
+      </c>
+      <c r="D3" s="57" t="s">
         <v>273</v>
       </c>
-      <c r="D3" s="57" t="s">
+      <c r="E3" s="19" t="s">
         <v>274</v>
-      </c>
-      <c r="E3" s="19" t="s">
-        <v>275</v>
       </c>
     </row>
     <row r="4" spans="1:5" ht="48">
@@ -6301,16 +6302,16 @@
         <v>2</v>
       </c>
       <c r="B4" s="20" t="s">
-        <v>281</v>
+        <v>280</v>
       </c>
       <c r="C4" s="57" t="s">
+        <v>277</v>
+      </c>
+      <c r="D4" s="57" t="s">
         <v>278</v>
       </c>
-      <c r="D4" s="57" t="s">
+      <c r="E4" s="19" t="s">
         <v>279</v>
-      </c>
-      <c r="E4" s="19" t="s">
-        <v>280</v>
       </c>
     </row>
     <row r="5" spans="1:5">
@@ -6318,16 +6319,16 @@
         <v>3</v>
       </c>
       <c r="B5" s="20" t="s">
-        <v>209</v>
+        <v>208</v>
       </c>
       <c r="C5" s="59" t="s">
-        <v>114</v>
+        <v>113</v>
       </c>
       <c r="D5" s="20" t="s">
-        <v>282</v>
+        <v>281</v>
       </c>
       <c r="E5" s="19" t="s">
-        <v>285</v>
+        <v>284</v>
       </c>
     </row>
     <row r="6" spans="1:5">
@@ -6335,16 +6336,16 @@
         <v>4</v>
       </c>
       <c r="B6" s="20" t="s">
-        <v>209</v>
+        <v>208</v>
       </c>
       <c r="C6" s="59" t="s">
-        <v>113</v>
+        <v>112</v>
       </c>
       <c r="D6" s="20" t="s">
+        <v>282</v>
+      </c>
+      <c r="E6" s="19" t="s">
         <v>283</v>
-      </c>
-      <c r="E6" s="19" t="s">
-        <v>284</v>
       </c>
     </row>
     <row r="7" spans="1:5" ht="32">
@@ -6352,10 +6353,10 @@
         <v>5</v>
       </c>
       <c r="B7" s="19" t="s">
+        <v>286</v>
+      </c>
+      <c r="C7" s="57" t="s">
         <v>287</v>
-      </c>
-      <c r="C7" s="57" t="s">
-        <v>288</v>
       </c>
       <c r="D7" s="57"/>
       <c r="E7" s="57"/>
@@ -6381,10 +6382,10 @@
   <sheetData>
     <row r="1" spans="1:2">
       <c r="A1" s="8" t="s">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="B1" s="9" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
     </row>
     <row r="2" spans="1:2">
@@ -6392,7 +6393,7 @@
         <v>0</v>
       </c>
       <c r="B2" s="4" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
     </row>
     <row r="3" spans="1:2">
@@ -6401,7 +6402,7 @@
     </row>
     <row r="4" spans="1:2">
       <c r="A4" s="7" t="s">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="B4" s="4"/>
     </row>
@@ -6431,19 +6432,19 @@
     </row>
     <row r="9" spans="1:2" ht="34">
       <c r="A9" s="7" t="s">
-        <v>5</v>
+        <v>288</v>
       </c>
       <c r="B9" s="4"/>
     </row>
     <row r="10" spans="1:2">
       <c r="A10" s="7" t="s">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="B10" s="4"/>
     </row>
     <row r="11" spans="1:2">
       <c r="A11" s="7" t="s">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="B11" s="4"/>
     </row>
@@ -6453,7 +6454,7 @@
     </row>
     <row r="13" spans="1:2">
       <c r="A13" s="6" t="s">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="B13" s="5">
         <v>46259.645833333336</v>
@@ -6461,7 +6462,7 @@
     </row>
     <row r="14" spans="1:2">
       <c r="A14" s="6" t="s">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="B14" s="5">
         <v>46259.5</v>
@@ -6483,77 +6484,77 @@
   <sheetData>
     <row r="1" spans="1:1" ht="21">
       <c r="A1" s="27" t="s">
-        <v>61</v>
+        <v>60</v>
       </c>
     </row>
     <row r="2" spans="1:1">
       <c r="A2" s="2" t="s">
-        <v>62</v>
+        <v>61</v>
       </c>
     </row>
     <row r="3" spans="1:1">
       <c r="A3" s="3" t="s">
-        <v>63</v>
+        <v>62</v>
       </c>
     </row>
     <row r="4" spans="1:1">
       <c r="A4" s="3" t="s">
-        <v>64</v>
+        <v>63</v>
       </c>
     </row>
     <row r="5" spans="1:1">
       <c r="A5" s="3" t="s">
-        <v>65</v>
+        <v>64</v>
       </c>
     </row>
     <row r="6" spans="1:1">
       <c r="A6" s="3" t="s">
-        <v>66</v>
+        <v>65</v>
       </c>
     </row>
     <row r="8" spans="1:1" ht="21">
       <c r="A8" s="27" t="s">
-        <v>67</v>
+        <v>66</v>
       </c>
     </row>
     <row r="9" spans="1:1">
       <c r="A9" s="3" t="s">
-        <v>68</v>
+        <v>67</v>
       </c>
     </row>
     <row r="10" spans="1:1">
       <c r="A10" s="3" t="s">
-        <v>69</v>
+        <v>68</v>
       </c>
     </row>
     <row r="11" spans="1:1">
       <c r="A11" s="3" t="s">
-        <v>70</v>
+        <v>69</v>
       </c>
     </row>
     <row r="12" spans="1:1">
       <c r="A12" s="3" t="s">
-        <v>71</v>
+        <v>70</v>
       </c>
     </row>
     <row r="14" spans="1:1" ht="21">
       <c r="A14" s="27" t="s">
-        <v>72</v>
+        <v>71</v>
       </c>
     </row>
     <row r="15" spans="1:1">
       <c r="A15" s="2" t="s">
-        <v>75</v>
+        <v>74</v>
       </c>
     </row>
     <row r="16" spans="1:1">
       <c r="A16" s="2" t="s">
-        <v>73</v>
+        <v>72</v>
       </c>
     </row>
     <row r="17" spans="1:1">
       <c r="A17" s="2" t="s">
-        <v>74</v>
+        <v>73</v>
       </c>
     </row>
   </sheetData>

</xml_diff>